<commit_message>
Revalidate lot1baseend spec against updated protocol PDF
Updated all 38 rows with correct protocol section references matching
the updated lot protocol.pdf. Key changes:
- Section references updated from generic "Section 5.1/6/7" to specific
  rule numbers (Rules 1-8 in Section 5.1.1)
- Permissible substitution language updated to match simplified protocol
  wording ("biologic reference product with any of its biosimilars")
- Steroid handling notes updated with explicit protocol quote "All rules
  described below are based on oncology therapies only (e.g., not
  corticosteroids)" - flagged potential misalignment with code
- SCT/tandem/allo references updated to correct Section 5.1 locations
- CAR-T 30-day consolidation reference corrected to Section 5.1.1
- Mesna exclusion reference corrected to Section 5.1
- All Date Modified fields updated to CV 2026-04-02
- Regenerated Excel file with color-coded formatting

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="10. LOT1_BASE_END" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LOT1 Base End Validated" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'10. LOT1_BASE_END'!$A$1:$L$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LOT1 Base End Validated'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,35 +28,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="009C6500"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00006100"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -89,8 +69,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E2F3"/>
-        <bgColor rgb="00D9E2F3"/>
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+        <bgColor rgb="00D6EAF8"/>
       </patternFill>
     </fill>
   </fills>
@@ -112,24 +98,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -500,18 +489,18 @@
   <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -599,7 +588,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1/6: LOT1 base period ends at the earliest of: discontinuation of all induction medications (gap &gt;= 90 days from OBS_END_DT), addition of a new non-induction medication, a LOT-ending SCT event, or end of observation (censoring at death/disenrollment/study end). The priority order is SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED. The conditioning period's MAP algorithm (Section 5B) determines medication coverage dates.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications (gap &gt;= 90 days from OBS_END_DT), addition of a new non-induction medication, a LOT-ending SCT event, or end of observation (censoring at death/disenrollment/study end). The priority order is SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED. The MAP algorithm (Section 5.1.1, Rule 2) defines run-out dates using 28-day assumed supply for medical claims. Priority order: SCT (Rule 3) &gt; MED_ADD (Rule 2) &gt; DISCONTINUATION (Rule 2) &gt; CENSORED (Rules 5-7).</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -622,7 +611,11 @@
           <t>Spec: N - uses simple min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP which is not yet defined; also garbled label text ('The end date for the 1date'). Protocol: Y - defines LOT1 end as earliest qualifying event with clear priority. Code: Y - implements priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCON &gt; CENSORED) which correctly reflects protocol priority; maintenance not yet integrated but logged as pending (line 4037).</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Original spec uses min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP, but the code uses a priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) rather than a simple minimum. The spec's label is garbled ('The end date for the 1date' should read 'The end date for the base period'). The inclusion of LOT1_BASE_MAINT_END_DT_TEMP in the min() is not applicable as maintenance is not enabled and is intentionally out of scope (confirmed by code comment at lot_program.R line 4037-4038).</t>
@@ -675,7 +668,11 @@
           <t>Spec: N - defines LOT1_END_DT_ORIG as a distinct variable for multi-step processing. Protocol: Y - protocol defines end date determination without specifying intermediate storage. Code: N - code does not create a separate LOT1_END_DT_ORIG variable; it computes the final end date directly in one step. The spec's multi-step approach (TEMP -&gt; ORIG -&gt; extend) differs from the code's single-pass approach.</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_END_DT_ORIG as '= LOT1_END_DT_TEMP' (a copy). The code does not implement this intermediate variable. Instead, the code computes LOT1_BASE_END_DT directly using a priority-based CASE statement at lot_program.R lines 4018-4028. The multi-step approach in the spec (calculate TEMP, save ORIG, then extend) is an implementation design choice that the code handles differently.</t>
@@ -705,7 +702,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1/6/7: LOT1 ends for one of these reasons: (1) Discontinuation - all induction medications' MAP coverage ends with a sufficient gap (&gt;= 90 days per cfg$lot_discon_gap_days) before observation end; (2) New medication addition - a medication not in the induction regimen is started; (3) Censoring - patient reaches end of observation without another event; (4) Death - captured via T_DOD; (5-7) SCT events - autologous, allogeneic, or CAR-T transplant ends the LOT. Priority: SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED (per protocol, transplant definitively ends a treatment line).</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (1) Discontinuation - all induction medications' MAP coverage ends with a sufficient gap (&gt;= 90 days per cfg$lot_discon_gap_days) before observation end; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events - autologous SCT &gt;180 days after previous, allogeneic always ends LOT, CAR-T starts new LOT. Protocol explicitly numbers LOT end events as Rules 1-8. Priority in code: SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -728,7 +725,11 @@
           <t>Spec: N - uses numeric codes 1-7 with date-matching logic and includes DEATH (4) as a separate end reason distinct from CENSOR. Protocol: Y - defines end reasons consistent with code priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED). Code: Y - uses string end reasons ('SCT_AUTO', 'SCT_ALLO', 'SCT_CART', 'MED_ADD', 'DISCONTINUATION', 'CENSORED') with priority-based CASE; death is subsumed into CENSORED via OBS_END_DT.</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Multiple discrepancies: (1) Spec uses numeric codes (1-7) while code uses descriptive strings ('DISCONTINUATION', 'MED_ADD', 'CENSORED', 'SCT_AUTO', 'SCT_ALLO', 'SCT_CART'). (2) Spec has DEATH as a separate end reason (code 4); code subsumes death into CENSORED since DEATH_DT is incorporated into OBS_END_DT/ENDDATE. (3) Spec determines end reason by matching LOT1_END_DT_TEMP against each candidate date; code uses explicit priority-based CASE (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED). (4) Spec's if/else chain checks LOT1_END_DT_TEMP against LOT1_DISCON_DT first, giving DISCONTINUATION highest priority among non-SCT reasons; code gives MED_ADD higher priority than DISCONTINUATION (when MED_ADD &lt;= DISCON). (5) Spec includes LOT1_BASE_MAINT_END_DT_TEMP in the initial min() which could set end reason to 2 (NEW MED) - maintenance is not yet implemented.</t>
@@ -758,7 +759,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7 (SCT): The protocol specifies that if a patient discontinues induction therapy and then receives an HSCT within the conditioning period window, the LOT1 should be extended to include the HSCT. The 60-day window represents the conditioning period before transplant. The code handles this differently by giving SCT events top priority in the end reason determination, so if an SCT occurs, it directly ends the LOT regardless of whether discontinuation was detected first.</t>
+          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Protocol states 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.' (Section 5.1.1). Single and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.' The code handles this by giving SCT events top priority in the end reason determination rather than using a separate extension flag.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -781,7 +782,11 @@
           <t>Spec: N - defines LOT1_EXTEND_FLG as explicit 60-day extension from discontinuation. Protocol: N - protocol describes extending LOT1 for HSCT during conditioning but the code implements this differently. Code: Y - handles HSCT-during-conditioning via SCT priority in end reason CASE statement rather than a separate extension flag. The clinical intent is preserved but the implementation architecture differs significantly.</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_EXTEND_FLG as a multi-step process: (1) check if LOT1 ended due to discontinuation, (2) check if HSCT occurred within 60 days, (3) extend LOT1 end date to include HSCT. The code does NOT implement this variable. Instead, the code gives SCT events highest priority in the LOT1_BASE_END_REASON CASE statement (lot_program.R lines 4001-4011), so if an SCT event occurs before discontinuation, it directly sets the end reason to SCT_AUTO/SCT_ALLO/SCT_CART. The 60-day extension concept from the spec is architecturally different from the code's priority-based approach. The code also logs that maintenance integration is pending (line 4037-4038).</t>
@@ -811,7 +816,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7: Related to the HSCT conditioning period concept. The protocol describes the interval between treatment discontinuation and transplant as the conditioning period. This variable quantifies that interval. Not directly specified as a named protocol variable but implied by the HSCT extension logic.</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): Related to the HSCT conditioning period concept. The protocol describes the interval between treatment discontinuation and transplant as the conditioning period. This variable quantifies that interval. Not directly specified as a named protocol variable but implied by the HSCT extension logic.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -834,7 +839,11 @@
           <t>Spec: N - defines variable as LOT1_END_DT_TEMP - LOT1_END_DT_ORIG. Protocol: N - does not explicitly name this metric. Code: Y - does not implement this variable (the code's architecture does not require it since SCT priority replaces the extension concept).</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_EXTEND_LENGTH = LOT1_END_DT_TEMP - LOT1_END_DT_ORIG. This variable is not implemented in the R code because the code does not use the multi-step extension approach. The code's priority-based CASE statement makes this variable unnecessary in the current implementation.</t>
@@ -864,7 +873,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7: After HSCT evaluation, if the LOT1 is extended to include an HSCT, the end reason should reflect whether the patient received maintenance after HSCT or if the LOT ended at the HSCT. The protocol does not explicitly define a 'SWITCH' concept for end reasons; this appears to be a spec-level implementation detail.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules): After HSCT evaluation, if the LOT1 is extended to include an HSCT, the end reason should reflect whether the patient received maintenance after HSCT or if the LOT ended at the HSCT. The protocol does not explicitly define a 'SWITCH' concept for end reasons; this appears to be a spec-level implementation detail.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -887,7 +896,11 @@
           <t>Spec: N - defines a multi-step update process for end reason. Protocol: N - does not define a 'switch' concept explicitly. Code: Y - computes final end reason in single CASE statement without intermediate switch step.</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_END_REASON_SWITCH as an updated version of LOT1_END_REASON_TEMP after HSCT extension logic. The code does not implement this as a separate variable. The code's single-pass LOT1_BASE_END_REASON (lot_program.R lines 4001-4017) serves as the final end reason. The spec's multi-step approach (TEMP -&gt; extend -&gt; SWITCH) is collapsed into one computation in the code.</t>
@@ -940,7 +953,11 @@
           <t>Spec: N - defines SWITCH_FLG based on LOT1_SAME_CLASS_1ST_DT which is not found in the code. Protocol: N - references same-class switching conceptually but does not define a specific flag variable. Code: Y - does not implement SWITCH_FLG; handles same-class via permissible_subs (lines 3346-3354) which treats certain within-class switches as part of the same LOT.</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Spec defines SWITCH_FLG = 1 if LOT1_SAME_CLASS_1ST_DT &lt;= LOT1_END_DT_TEMP. Neither LOT1_SAME_CLASS_1ST_DT nor SWITCH_FLG are implemented in the R code. The code handles same-class medication changes through the permissible substitutions mechanism (lot_program.R lines 3346-3354) rather than a separate flag. The spec's SWITCH_FLG concept is not present in the current codebase.</t>
@@ -970,7 +987,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7 (SCT): Autologous HSCT identification uses a 14-day claim windowing algorithm, requiring at least 60 days between distinct AUTO events. A single AUTO is one that is not part of a valid tandem pair. The protocol specifies that AUTO SCT claims within 14 days are grouped together, and events must be at least 60 days apart to be considered separate transplants.</t>
+          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Autologous SCT identification uses a 14-day claim windowing algorithm (operationalized as &gt;1 procedure code for an SCT per Section 5.1), requiring at least 60 days between distinct AUTO events. A single AUTO is one that is not part of a valid tandem pair. The protocol specifies that AUTO SCT claims within 14 days are grouped together, and events must be at least 60 days apart to be considered separate transplants.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -993,7 +1010,11 @@
           <t>Spec: N - includes additional logic to reset flag to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (HSCT occurred after LOT1 ended). Protocol: Y - defines single AUTO HSCT criteria. Code: Y - computes flag based on AUTO dates and tandem validation but does not reset to 0 based on LOT1_END_DT_TEMP; instead, the SCT priority logic in Step S16 handles this implicitly.</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Spec includes logic to set LOT1_HSCT_AUTO_SING_FLG to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (i.e., the HSCT occurred after the LOT ended). The code at lot_program.R lines 3911-3917 does not include this temporal filter - the flag is set purely based on AUTO date existence and tandem validation. However, in the code's Step S16 end reason logic (lines 4001-4011), SCT events are only used if LOT1_TX_ENDDATE &lt;= other end dates, effectively achieving the same clinical filtering.</t>
@@ -1023,7 +1044,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7 (SCT): Tandem autologous HSCT is defined as two autologous transplants within 180 days (cfg$sct_tandem_days) with no intervening allogeneic transplant. The first AUTO sets AUTO_DT_1, the second sets AUTO_DT_2. For tandem patients, a 3rd AUTO would end the LOT; for single AUTO patients, a 2nd AUTO ends the LOT.</t>
+          <t>Protocol Section 5.1 (Planned Tandem SCT): Protocol: 'Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart.' An autologous-to-allogeneic sequence is NOT considered planned. Tandem SCTs are 'considered planned and a continuation of the line of therapy' (Section 5.1.1). The first AUTO sets AUTO_DT_1, the second sets AUTO_DT_2. For tandem patients, a 3rd AUTO would end the LOT; for single AUTO patients, a 2nd AUTO ends the LOT.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1046,7 +1067,11 @@
           <t>Spec: N - includes reset logic if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. Protocol: Y - defines tandem as 2 AUTO within 180 days with no ALLO between. Code: Y - implements tandem flag matching protocol definition; temporal filtering handled implicitly by Step S16 priority logic.</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Spec includes logic to reset LOT1_HSCT_AUTO_TAND_FLG to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. The code (lot_program.R lines 3904-3909) does not include this reset. Similar to SING_FLG, the temporal relationship is handled by Step S16's SCT priority logic rather than modifying the flag itself.</t>
@@ -1076,7 +1101,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7: The latest AUTO date is relevant for determining the LOT-ending SCT event. For tandem patients, the 2nd AUTO is the latest valid AUTO (the 3rd AUTO, if it exists, would end the LOT). For single AUTO patients, the 1st AUTO is the latest (the 2nd would end the LOT).</t>
+          <t>Protocol Section 5.1 (Planned Tandem SCT): The latest AUTO date is relevant for determining the LOT-ending SCT event. For tandem patients, the 2nd AUTO is the latest valid AUTO (the 3rd AUTO, if it exists, would end the LOT). For single AUTO patients, the 1st AUTO is the latest (the 2nd would end the LOT).</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1099,7 +1124,11 @@
           <t>Spec: N - defines explicit LOT1_TX_AUTO_MAX_DT variable. Protocol: Y - defines which AUTO date is the latest valid one. Code: Y - has equivalent data (AUTO_DT_1, AUTO_DT_2) but does not create a named LOT1_TX_AUTO_MAX_DT variable.</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_TX_AUTO_MAX_DT as a named variable. The code does not create this specific variable but has the underlying data (AUTO_DT_1, AUTO_DT_2 at lot_program.R lines 3901-3902). The max valid AUTO date can be derived from the existing variables.</t>
@@ -1129,7 +1158,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7: Indicates whether the patient received any valid autologous transplant during the study period, regardless of whether it was single or tandem.</t>
+          <t>Protocol Section 5.1 (SCT): Indicates whether the patient received any valid autologous transplant during the study period, regardless of whether it was single or tandem.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1152,7 +1181,11 @@
           <t>Spec: N - defines explicit combined flag. Protocol: Y - concept is clear. Code: Y - does not create combined flag but has constituent flags (TAND and SING) from which it can be derived.</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_TX_AUTO_FLG as a combined flag. The code does not create this specific variable but has LOT1_SCT_AUTO_TAND_FLG and LOT1_SCT_AUTO_SING_FLG (lot_program.R lines 3904-3917) from which the combined flag is trivially derivable.</t>
@@ -1182,7 +1215,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 7: When LOT1 is extended to include an HSCT, the end date moves to the HSCT date (for single) or the second HSCT date (for tandem). If the patient receives maintenance after the HSCT, the LOT1 end date will be further extended (maintenance not yet implemented).</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): When LOT1 is extended to include an HSCT, the end date moves to the HSCT date (for single) or the second HSCT date (for tandem). If the patient receives maintenance after the HSCT, the LOT1 end date will be further extended (maintenance not yet implemented).</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1205,7 +1238,11 @@
           <t>Spec: N - updates TEMP variable iteratively to HSCT date. Protocol: N - describes extending to include HSCT. Code: Y - uses LOT1_TX_ENDDATE (day before LOT-ending SCT) as the end date when SCT has priority. Key difference: spec extends LOT1 TO the HSCT date; code sets end to day BEFORE the LOT-ending SCT (which is the next AUTO after the included one).</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Spec updates LOT1_END_DT_TEMP to the included HSCT date (AUTO_DT_1 for single, AUTO_DT_2 for tandem). The code's LOT1_TX_ENDDATE is date_sub(ENDING_AUTO_DT, 1) where ENDING_AUTO_DT is the NEXT AUTO beyond what's included (AUTO_DT_2 for single, AUTO_DT_3 for tandem). This means the code's end date is the day before the LOT-ending SCT, not the date of the included SCT. The architectural approach differs significantly between spec and code.</t>
@@ -1235,7 +1272,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1/6: Induction medications are all MM therapies initiated within the induction window from LOT1 start date. The medication list defines the base regimen for the LOT. Permissible substitutions (within-class switches that do not constitute a new LOT) are included as part of the base regimen.</t>
+          <t>Protocol Section 5.1.1 (LOT regimen): Induction medications are all MM therapies initiated within the induction window from LOT1 start date. The medication list defines the base regimen for the LOT. Permissible substitutions (within-class switches that do not constitute a new LOT) are included as part of the base regimen.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1258,7 +1295,11 @@
           <t>Spec: Y - defines LOT1_BASE_MEDS as induction medications from LOT1_BASE dataset. Protocol: Y - defines induction regimen as medications in the induction window. Code: Y - implements via concat_ws/sort_array/collect_set of MED_ABBR from lot1_induction_meds.</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -1288,7 +1329,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Protocol: Maintenance therapy follows induction/consolidation therapy. The maintenance period starts when a patient transitions from multi-agent induction to single-agent (mono) or dual-agent (dual) maintenance therapy. The protocol specifies mono-maintenance (single non-steroid medication with MONOMAINTENANCE=1 flag) and dual-maintenance (two medications where the combination is in the DUALMAINTENANCEWITH field of CL_MMA_ROLLUP).</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance therapy follows induction/consolidation therapy. The maintenance period starts when a patient transitions from multi-agent induction to single-agent (mono) or dual-agent (dual) maintenance therapy. The protocol specifies mono-maintenance (single non-steroid medication with MONOMAINTENANCE=1 flag) and dual-maintenance (two medications where the combination is in the DUALMAINTENANCEWITH field of CL_MMA_ROLLUP).</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1301,7 +1342,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED. Line 4037-4038: 'NOTE: Maintenance (mono/dual) specs not yet provided; LOT1_BASE_END_REASON does not yet include MAINTENANCE_START. Will need integration when available.' Maintenance is intentionally out of scope in the current implementation. Maintenance analysis exists separately in lot_analysis.R lines 1224-1350 for reporting but is not integrated into the LOT1 end date/reason computation.</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1311,7 +1352,11 @@
           <t>Spec: N - defines LOT1_BASEMAINT_START with specific logic but maintenance is not enabled. Protocol: - (maintenance concept defined in protocol but not currently in scope for implementation). Code: N - maintenance intentionally not enabled; explicitly logged at line 4037-4038. This is a deliberate scope decision, not an implementation gap.</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_START with detailed conditions (120-day gap check, comparison with other end events). Maintenance is NOT ENABLED in the current implementation. The code explicitly logs that maintenance specs are not yet provided (lot_program.R lines 4037-4038). This is a deliberate scope decision - maintenance variables in the spec are aspirational and will require future implementation when maintenance is brought into scope.</t>
@@ -1341,7 +1386,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Protocol: The maintenance medication type identifies which drug is used for maintenance (e.g., LENA for lenalidomide, BORT for bortezomib). For mono-maintenance, this is a single medication; for dual-maintenance, this would describe the combination.</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): The maintenance medication type identifies which drug is used for maintenance (e.g., LENA for lenalidomide, BORT for bortezomib). For mono-maintenance, this is a single medication; for dual-maintenance, this would describe the combination.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1354,7 +1399,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED (see line 4037-4038). Maintenance type tracking exists in lot_analysis.R for analysis purposes but is not connected to LOT1_BASE_END. Intentionally out of scope.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1364,7 +1409,11 @@
           <t>Spec: N - defines variable from LOT1_BASE_MAINT dataset but maintenance is not enabled. Protocol: - (defines maintenance medication concept but not in scope). Code: N - maintenance intentionally not enabled.</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_TYP from the LOT1_BASE_MAINT input dataset. MAINTENANCE IS NOT ENABLED in the current implementation. This is an aspirational spec variable that will require future implementation when maintenance is brought into scope.</t>
@@ -1394,7 +1443,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Protocol: The maintenance period ends when the patient discontinues maintenance therapy, adds a new medication (signaling a new LOT), receives an SCT, dies, or reaches end of observation. The end of maintenance also considers the same priority hierarchy as the base period end.</t>
+          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): The maintenance period ends when the patient discontinues maintenance therapy, adds a new medication (signaling a new LOT), receives an SCT, dies, or reaches end of observation. The end of maintenance also considers the same priority hierarchy as the base period end.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1407,7 +1456,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED (see line 4037-4038). The spec describes complex maintenance end date logic involving LOT1_MAINT_ADD_FLG and comparison with multiple end dates, none of which are currently computed. Intentionally out of scope.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1417,7 +1466,11 @@
           <t>Spec: N - defines complex maintenance end date logic but maintenance is not enabled. Protocol: - (describes maintenance end conceptually but not in scope). Code: N - maintenance intentionally not enabled.</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_END with detailed conditional logic. MAINTENANCE IS NOT ENABLED in the current implementation. This is an aspirational spec variable pending future scope decision.</t>
@@ -1447,7 +1500,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Protocol: Maintenance medication flags identify the specific drugs used during maintenance. These are a subset of the full medication list (BORT=bortezomib, DARA=daratumumab, IXAZ=ixazomib, LENA=lenalidomide, CARF=carfilzomib). The CL_MMA_ROLLUP codelist (Tab 40) defines which medications are eligible for maintenance via the MONOMAINTENANCE flag and DUALMAINTENANCEWITH field.</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance medication flags identify the specific drugs used during maintenance. These are a subset of the full medication list (BORT=bortezomib, DARA=daratumumab, IXAZ=ixazomib, LENA=lenalidomide, CARF=carfilzomib). The CL_MMA_ROLLUP codelist (Tab 40) defines which medications are eligible for maintenance via the MONOMAINTENANCE flag and DUALMAINTENANCEWITH field.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1460,7 +1513,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED. Induction medication flags (LOT1_MED_BORT, LOT1_MED_DARA, etc.) exist at Step S10 lines 3389 via med_flag_exprs (lines 2886-2889). Maintenance-specific flags (LOT1_BASEMAINT_MED_BORT, etc.) are not computed. Intentionally out of scope.</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1470,7 +1523,11 @@
           <t>Spec: N - defines maintenance medication flags but maintenance is not enabled. Protocol: - (defines maintenance medications conceptually but not in scope). Code: N - maintenance intentionally not enabled. Induction med flags exist separately.</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_MED_[MED] for BORT, DARA, IXAZ, LENA, CARF. MAINTENANCE IS NOT ENABLED in the current implementation. Induction medication flags (LOT1_MED_BORT, etc.) are implemented at lot_program.R Step S10 lines 3389 but these are separate from the maintenance flags. Aspirational spec variable pending future scope decision.</t>
@@ -1500,7 +1557,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Protocol: Maintenance period end reasons follow a similar logic to the base period end reasons. The maintenance period can end due to discontinuation of maintenance therapy, addition of a new medication (indicating progression to next LOT), censoring, death, or an SCT event.</t>
+          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): Maintenance period end reasons follow a similar logic to the base period end reasons. The maintenance period can end due to discontinuation of maintenance therapy, addition of a new medication (indicating progression to next LOT), censoring, death, or an SCT event.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1513,7 +1570,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED (see line 4037-4038). The spec describes maintenance end reason logic that depends on LOT1_MAINT_ADD_FLG and LOT1_BASE_MAINT_END_DT_TEMP, neither of which are computed. Intentionally out of scope. Note: end reason values in spec are numeric (1-6) while the code uses string values for the base end reason.</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1523,7 +1580,11 @@
           <t>Spec: N - defines maintenance end reason with numeric codes but maintenance is not enabled. Protocol: - (describes maintenance end conceptually but not in scope). Code: N - maintenance intentionally not enabled.</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_END_REASON with numeric codes (1-6). MAINTENANCE IS NOT ENABLED in the current implementation. Additionally, the spec uses 6 values (1-6) while the base end reason has 7 (1-7, including CART) - the maintenance end reason omits CART (7), which may be intentional or an oversight. Aspirational spec variable pending future scope decision.</t>
@@ -1531,1067 +1592,1147 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_END_DT</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Final LOT1 base period end date</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>The final computed end date for the LOT1 base period after all adjustments (SCT evaluation, HSCT extension, maintenance integration). This is the definitive end date used for downstream analysis. In the code, this is directly computed via a priority-based CASE statement: (1) LOT1_TX_ENDDATE if SCT has priority, (2) LOT1_BASE_1ST_ADD_MED_DT if medication addition, (3) LOT1_BASE_DISCON_DT if discontinuation, (4) OBS_END_DT if censored.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1 (LOT end date): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. This final variable should be the non-temporary version after all adjustments. The original spec only defines TEMP versions but never creates the final LOT1_BASE_END_DT.</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (LOT end date, Rules 1-8): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. This final variable should be the non-temporary version after all adjustments. The original spec only defines TEMP versions but never creates the final LOT1_BASE_END_DT.</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_END_DT derived from priority evaluation of dates from T_MEDICAL/T_RX (MAP_END_DT for discontinuation, MAP_START_DT for new med), T_MEDICAL procedure codes (SCT events), T_DOD (YMDOD for death), T_MEMBER_CONT_ENROLLMENT (ELIGEND for disenrollment), and study_end config parameter.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S16 lines 4018-4028: LOT1_BASE_END_DT = CASE WHEN SCT priority THEN sct.LOT1_TX_ENDDATE; WHEN MED_ADD priority THEN lb.LOT1_BASE_1ST_ADD_MED_DT; WHEN DISCON THEN lb.LOT1_BASE_DISCON_DT; ELSE lb.OBS_END_DT END. This is the final (non-temporary) end date used in the lot1_base_end view.</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (defines end date concept but spec only has TEMP versions). Code: Y - implements LOT1_BASE_END_DT as the final computed end date. This variable is missing from the original spec which only has LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never creates the final non-temporary version.</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr"/>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never defines the final LOT1_BASE_END_DT. The code creates this as the definitive end date at lot_program.R Step S16 lines 4018-4028. The spec should include this final variable to show the output of the LOT1_BASE_END section.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_END_REASON</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Final LOT1 base period end reason</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>The final computed end reason for the LOT1 base period. Values: 'DISCONTINUATION' (all induction meds ran out with sufficient gap), 'MED_ADD' (new non-induction medication added), 'CENSORED' (end of observation - death/disenrollment/study end), 'SCT_AUTO' (LOT ended by autologous transplant), 'SCT_ALLO' (LOT ended by allogeneic transplant), 'SCT_CART' (LOT ended by CAR-T therapy). Priority: SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED.</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: LOT ends when (1) a transplant occurs (highest priority - allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. The original spec only defines TEMP and SWITCH versions with numeric codes but never creates the final string-valued LOT1_BASE_END_REASON.</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (highest priority - allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. The original spec only defines TEMP and SWITCH versions with numeric codes but never creates the final string-valued LOT1_BASE_END_REASON.</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>End reason derived from evaluation of dates across T_MEDICAL/T_RX (medication events), T_MEDICAL (SCT procedure codes), T_DOD (death), and T_MEMBER_CONT_ENROLLMENT (disenrollment). Priority logic applied analytically.</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S16 lines 4001-4017: LOT1_BASE_END_REASON = CASE WHEN SCT AND earliest THEN 'SCT_AUTO'/'SCT_ALLO'/'SCT_CART'; WHEN MED_ADD AND earliest THEN 'MED_ADD'; WHEN DISCON THEN 'DISCONTINUATION'; ELSE 'CENSORED' END. QC query at lines 4032-4035 produces distribution of end reasons.</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present as final variable; only TEMP and SWITCH versions). Protocol: - (defines end reasons conceptually). Code: Y - implements LOT1_BASE_END_REASON as the final string-valued end reason.</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_REASON_TEMP and LOT1_END_REASON_SWITCH with numeric codes (1-7) but never creates the final LOT1_BASE_END_REASON. The code creates this with string values at lot_program.R Step S16 lines 4001-4017.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>LOT1_1ST_SCT_DT</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Date of first SCT event of any type during LOT1</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>The earliest SCT event (autologous, allogeneic, or CAR-T) occurring during the LOT1 period. Computed as LEAST(LOT1_TX_AUTO_DT_1, FIRST_ALLO_DT, FIRST_CART_DT). This date is relevant for determining when SCT-related treatment changes begin and for calculating intervals between induction end and transplant.</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1/7: 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.' LOT1_1ST_SCT_DT enables validation of this 60-day window rule.</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.' LOT1_1ST_SCT_DT enables validation of this 60-day window rule.</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>First SCT date derived from T_MEDICAL procedure codes matching CL_SCT_CODELIST entries (Tab 44). AUTO type identified by SCT_TYPE='AUTO'; ALLO by SCT_TYPE='ALLO'; CAR-T by SCT_TYPE='CART'. Dates from FST_DT in T_MEDICAL after 14-day claim windowing and 60-day gap validation.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S15 lines 3963-3972: LOT1_1ST_SCT_DT = CASE WHEN any SCT date exists THEN least(coalesce(AUTO_DT_1, '9999-12-31'), coalesce(FIRST_ALLO_DT, '9999-12-31'), coalesce(FIRST_CART_DT, '9999-12-31')) ELSE NULL END. Carried into lot1_base_end view at Step S16 line 3998.</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (concept exists via 60-day SCT window rule). Code: Y - implemented at Step S15 lines 3963-3972 and carried through to lot1_base_end.</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code computes LOT1_1ST_SCT_DT at lot_program.R Step S15 (lines 3963-3972) as the earliest SCT of any type. This is useful for validating the protocol's 60-day window rule (SCT must occur within 60 days of induction/maintenance end to be continuation of LOT). The spec should include this variable.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>FIRST_ALLO_DT</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Date of first allogeneic HSCT during LOT1</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>The date of the first allogeneic (ALLO) HSCT occurring during the LOT1 period. Per protocol, any allogeneic SCT always ends the current LOT because an allogeneic SCT typically follows failed autologous SCTs and represents a fundamentally different treatment approach.</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' This is a hard rule - ALLO always ends the LOT regardless of timing relative to other events.</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' (Section 5.1). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs' (Section 5.1.1, Rule 3). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' This is a hard rule - ALLO always ends the LOT regardless of timing relative to other events.</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>ALLO SCT identified from T_MEDICAL procedure codes matching CL_SCT_CODELIST entries where SCT_TYPE='ALLO'. Date from FST_DT in T_MEDICAL. Sequential ordering applied to identify first ALLO event.</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S14 lines 3796-3825: tx_allo_cart_dates extracts ALLO dates from sct_events. Step S15 line 3929: FIRST_ALLO_DT = fa.ALLO_DT from first_allo CTE. Carried into lot1_base_end at Step S16 line 3999. Used in LOT1_TX_ENDDATE calculation (lines 3939-3949) and LOT1_TX_ENDDATE_REASON (lines 3951-3962).</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present as standalone variable; referenced indirectly via SCT_ALLO end reason). Protocol: - (defines ALLO as always ending LOT). Code: Y - implemented at Step S15 line 3929 and used in end date/reason calculations.</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
-      <c r="K23" s="6" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_ALLO_DT at lot_program.R Step S15 (line 3929) and uses it in the LOT1_TX_ENDDATE and LOT1_TX_ENDDATE_REASON calculations. The protocol explicitly states that any ALLO SCT ends the current LOT (Section 5.1.1). The spec references SCT_ALLO as end reason code 6 but does not define FIRST_ALLO_DT as a standalone variable.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>FIRST_CART_DT</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Date of first CAR-T therapy during LOT1</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>The date of the first CAR-T cellular therapy occurring during the LOT1 period. Per protocol, CAR-T therapy starts a new LOT, so the current LOT ends the day before the CAR-T date. Supportive agents (including corticosteroids) given within 30 days of CAR-T are consolidated as part of the CAR-T LOT.</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.2: 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' CAR-T always starts a new LOT, ending the current one. The 30-day supportive agent consolidation rule means medications within 30 days of CAR-T are attributed to the CAR-T LOT, not the preceding LOT.</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (CAR-T): 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' CAR-T always starts a new LOT, ending the current one. The 30-day supportive agent consolidation rule means medications within 30 days of CAR-T are attributed to the CAR-T LOT, not the preceding LOT.</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>CAR-T identified from T_MEDICAL procedure codes matching CL_SCT_CODELIST entries where SCT_TYPE='CART'. Date from FST_DT in T_MEDICAL.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S14 lines 3796-3825: tx_allo_cart_dates extracts CART dates from sct_events. Step S15 line 3930: FIRST_CART_DT = fc.CART_DT from first_cart CTE. Carried into lot1_base_end at Step S16 line 4000. Used in LOT1_TX_ENDDATE (lines 3939-3949) and LOT1_TX_ENDDATE_REASON (lines 3951-3962, mapped to reason=3='SCT_CART').</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present as standalone variable; referenced indirectly via CART end reason code 7). Protocol: - (defines CAR-T as starting new LOT with 30-day consolidation rule). Code: Y - implemented at Step S15 line 3930.</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr"/>
-      <c r="K24" s="6" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_CART_DT at lot_program.R Step S15 (line 3930). The protocol defines CAR-T as always starting a new LOT (Section 5.1.2) with a 30-day supportive agent consolidation rule. The spec has CART as end reason code 7 but does not define FIRST_CART_DT as a standalone variable.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>LOT_DISCON_GAP_DAYS</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Discontinuation gap threshold (days)</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>The minimum number of days between the last medication run-out date and the observation end date required for a discontinuation to be recognized. Default value: 90 days. If the gap between the last MAP_END_DT for induction medications and OBS_END_DT is less than this threshold, the patient is NOT considered discontinued (they are censored instead). This prevents classifying patients whose medications simply ran out near the end of follow-up as discontinued.</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The run-out date is the MAP_END_DT (last day of medication availability). The gap threshold ensures there is sufficient time after medication ends to confirm the patient truly discontinued rather than being censored. The 90-day default is consistent with a treatment cycle of approximately 3 months. This parameter is configurable for sensitivity analysis per Protocol Section 5.3.</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The run-out date is the MAP_END_DT (last day of medication availability). The gap threshold ensures there is sufficient time after medication ends to confirm the patient truly discontinued rather than being censored. The 90-day default is consistent with a treatment cycle of approximately 3 months. Configurable for sensitivity analysis per Protocol Section 5.3 which states 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Gap calculated as datediff(OBS_END_DT, RAW_DISCON_DT) where OBS_END_DT is derived from T_MEMBER_CONT_ENROLLMENT (ELIGEND), T_DOD (YMDOD), and study_end config. RAW_DISCON_DT is max(MAP_END_DT) from T_MEDICAL/T_RX for induction medications.</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>lot_program.R line 73: lot_discon_gap_days = as.integer(Sys.getenv('LOT_DISCON_GAP_DAYS', unset = '90')). Applied at Step S10 line 3376: LOT1_BASE_DISCON_DT = RAW_DISCON_DT only WHEN datediff(OBS_END_DT, RAW_DISCON_DT) &gt;= cfg$lot_discon_gap_days. Otherwise NULL (patient is censored, not discontinued). Configurable via LOT_DISCON_GAP_DAYS env var.</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not defined as a parameter; implicitly used but not documented). Protocol: - (defines discontinuation concept but does not specify exact gap threshold). Code: Y - implements as configurable parameter defaulting to 90 days at line 73, applied at line 3376.</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
-      <c r="K25" s="6" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
         <is>
           <t>Parameter missing from original spec. The code uses lot_discon_gap_days=90 (lot_program.R line 73) to determine whether a patient is truly discontinued vs censored. This critical threshold affects whether LOT1_BASE_DISCON_DT is set or left NULL. The spec should document this parameter as it directly affects the LOT1_END_REASON classification.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>MEDICAL_DAY_SUPPLY</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Assumed days supply for medical claims</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>When days supply is missing from medical claims (infused/injected medications), a default of 28 days is assumed. This affects MAP_END_DT calculation which directly impacts LOT1_BASE_DISCON_DT and therefore LOT1_BASE_END_DT. For pharmacy claims with missing or anomalous days supply values, 28 days is also assumed.</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'The days supply on medical claims is always missing and therefore a 28 days supply is assumed. When pharmacy claims are missing days supply, or when days supply values are anomalous, 28 days will be assumed.' This is a fundamental parameter for the MAP algorithm that feeds into the LOT1 end date calculation. The 28-day assumption represents approximately one treatment cycle.</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 2 - run-out date): 'The days' supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days' supply, or when days' supply values are anomalous, a 28-day supply is assumed.' (Section 5.1.1, under Rule 2). This is a fundamental parameter for the MAP algorithm that feeds into the LOT1 end date calculation. The 28-day assumption represents approximately one treatment cycle.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>Applied to T_MEDICAL claims where DAYS_SUPPLY is NULL. For T_RX pharmacy claims, DAYS_SUPPLY is typically populated but when missing/anomalous, 28 days is substituted. The assumed supply extends MAP_END_DT = FST_DT (or FILL_DT) + days_supply - 1.</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>lot_program.R line 74: medical_day_supply = as.integer(Sys.getenv('MEDICAL_DAY_SUPPLY', unset = '28')). Used in MAP construction (Step S05/S06 area) to set MAP_END_DT for medical claims. Configurable via MEDICAL_DAY_SUPPLY env var. This feeds into LOT1_BASE_DISCON_DT via max(MAP_END_DT).</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not documented in LOT1_BASE_END tab). Protocol: - (defined in Section 5.1.1 under MAP algorithm). Code: Y - implemented as configurable parameter defaulting to 28 days at line 74.</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
-      <c r="K26" s="6" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses medical_day_supply=28 (lot_program.R line 74) for MAP_END_DT calculation on medical claims. While this is defined in the MAP section (5B), it directly affects LOT1_BASE_DISCON_DT and should be cross-referenced here. Protocol Section 5.1.1 explicitly states the 28-day assumption.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_LENGTH</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>LOT1 base period duration in days</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>The number of days in the LOT1 base period, computed as datediff(LOT1_BASE_END_DT, LOT1_START_DT) + 1. Uses the priority-based end date: if MED_ADD occurs before DISCON, length is to MED_ADD date; if DISCON is first, length is to DISCON date; otherwise length is to OBS_END_DT (censored).</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: LOT duration is the span from LOT start (first non-steroid MAP) to LOT end. The +1 ensures inclusive day counting (both start and end dates are counted). Duration is relevant for assessing treatment patterns and time-to-event analyses.</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (LOT start/end): LOT duration is the span from LOT start (first non-steroid MAP) to LOT end. The +1 ensures inclusive day counting (both start and end dates are counted). Duration is relevant for assessing treatment patterns and time-to-event analyses.</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Duration computed from dates already derived from T_MEDICAL/T_RX (LOT1_START_DT from first MAP_START_DT) and LOT1_BASE_END_DT (priority-based end date).</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S10 lines 3447-3455: LOT1_BASE_LENGTH = CASE WHEN MED_ADD &lt;= DISCON THEN datediff(LOT1_BASE_1ST_ADD_MED_DT, LOT1_START_DT) + 1; WHEN DISCON THEN datediff(LOT1_BASE_DISCON_DT, LOT1_START_DT) + 1; ELSE datediff(OBS_END_DT, LOT1_START_DT) + 1 END. QC at line 3466: avg(LOT1_BASE_LENGTH) computed in validation query.</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not defined in LOT1_BASE_END tab). Protocol: - (duration concept implied). Code: Y - computed at Step S10 lines 3447-3455 with priority MED_ADD &gt; DISCON &gt; CENSORED.</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
-      <c r="K27" s="6" t="inlineStr">
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab. The code computes LOT1_BASE_LENGTH at lot_program.R Step S10 (lines 3447-3455) using a priority-based CASE matching the same hierarchy as LOT1_BASE_END_DT. Note: this is computed in the LOT1_BASE step (S10) rather than LOT1_BASE_END (S16), but it represents the base period duration which should be documented here.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>LOT1_SCT_TO_MAINT_180D_RULE</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>SCT not followed by maintenance within 180 days - LOT end rule</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Protocol rule: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT. This rule determines whether LOT1 extends beyond the SCT to include a maintenance period or ends at the SCT itself. This is distinct from the 60-day conditioning period window (LOT1_EXTEND_FLG) which determines whether an SCT is included in LOT1 at all.</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' This rule interacts with the maintenance logic: if maintenance starts within 180 days of SCT, LOT1 is extended to include the maintenance period. If no maintenance within 180 days, LOT1 ends at the SCT date. The 180-day window is consistent with the tandem SCT definition (cfg$sct_tandem_days=180).</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 4 - SCTs not followed by maintenance): Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Also Section 5.1 (Maintenance regimen, situation 2): 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT).' This rule interacts with the maintenance logic: if maintenance starts within 180 days of SCT, LOT1 is extended to include the maintenance period. If no maintenance within 180 days, LOT1 ends at the SCT date. The 180-day window is consistent with the tandem SCT definition (cfg$sct_tandem_days=180).</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>Would require checking T_MEDICAL/T_RX claims for maintenance medications (MONOMAINTENANCE=1 or valid DUALMAINTENANCEWITH in CL_MMA_ROLLUP) within 180 days after the SCT date (LOT1_1ST_SCT_DT or LOT1_TX_AUTO_MAX_DT).</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>lot_program.R: NOT APPLICABLE - MAINTENANCE IS NOT ENABLED. This rule depends on maintenance integration which is intentionally out of scope (line 4037-4038). The code currently ends LOT1 at LOT1_TX_ENDDATE (day before LOT-ending SCT) when SCT has priority. This 180-day rule will only become relevant if/when maintenance is brought into scope.</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>--N</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not defined). Protocol: - (defined in Section 5.1.1). Code: N - not applicable because maintenance is not enabled. This protocol rule will only be relevant when maintenance is brought into scope.</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr"/>
-      <c r="K28" s="6" t="inlineStr">
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.1 states that if SCT is not followed by maintenance within 180 days, the LOT ends at the SCT date. NOT APPLICABLE in current implementation because maintenance is not enabled. This rule should be implemented if/when maintenance is brought into scope.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>PERMISSIBLE_SUBS_EFFECT</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Permissible substitution rules affecting LOT1 end</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Certain medication switches do NOT advance the LOT (i.e., do not set LOT1_BASE_1ST_ADD_MED_DT). These permissible substitutions include: (1) rituximab &lt;-&gt; rituximab/hyaluronidase, (2) daratumumab &lt;-&gt; daratumumab/hyaluronidase, (3) reference product &lt;-&gt; biosimilar (e.g., trastuzumab &lt;-&gt; trastuzumab-anns), (4) bortezomib induction -&gt; ixazomib maintenance. The code implements this via the permissible_subs table which is joined into base_meds, effectively treating substitutions as part of the original regimen.</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1 (Substitution of a new MM treatment): Explicit rules for permissible substitutions that do not advance the LOT. This directly affects LOT1_BASE_1ST_ADD_MED_DT: if the 'new' medication is a permissible substitute, it should not be counted as an addition. The permissible_subs table codifies these rules.</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Certain medication switches do NOT advance the LOT (i.e., do not set LOT1_BASE_1ST_ADD_MED_DT). Per the updated protocol (Rule 1): 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT.' Specific substitutions in code: (1) rituximab &lt;-&gt; rituximab/hyaluronidase, (2) daratumumab &lt;-&gt; daratumumab/hyaluronidase, (3) reference product &lt;-&gt; biosimilar, (4) bortezomib induction -&gt; ixazomib maintenance. The code implements this via the permissible_subs table which is joined into base_meds, effectively treating substitutions as part of the original regimen.</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 1 - Permissible substitutions): Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.' This directly affects LOT1_BASE_1ST_ADD_MED_DT: if the 'new' medication is a permissible substitute, it should not be counted as an addition. The permissible_subs table codifies these rules.</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Substitutions tracked via CL_MMA_ROLLUP (Tab 40) which maps medication abbreviations. The permissible_subs reference table pairs original_med with substitute_med. When a new medication claim appears in T_MEDICAL/T_RX, it is checked against permissible_subs before being classified as a new medication addition.</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S02 lines 2796-2803: permissible_subs view created from embedded or external table. Step S10 lines 3346-3354: base_meds CTE includes UNION with permissible_subs (im.MED_ABBR joined to ps.original_med -&gt; ps.substitute_med added to base_meds). This means first_add_candidates (lines 3413-3425) will NOT flag permissible substitutes as new medications because they are already in base_meds. Embedded permissible_subs defined at line 273.</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>Spec: - (permissible substitutions not documented in LOT1_BASE_END tab). Protocol: - (defined in Section 5.1.1). Code: Y - implemented via permissible_subs table joined into base_meds CTE at Step S10 lines 3346-3354.</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr"/>
-      <c r="K29" s="6" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>Concept missing from original spec's LOT1_BASE_END tab. The code implements permissible substitutions by expanding base_meds to include substitutes (lot_program.R Step S10 lines 3346-3354). This is critical for correct LOT1_BASE_1ST_ADD_MED_DT calculation: without it, a permissible substitute (e.g., daratumumab/hyaluronidase replacing daratumumab) would incorrectly trigger a MED_ADD end reason. Protocol Section 5.1.1 explicitly defines which substitutions are permissible.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>STEROID_HANDLING</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Steroid inclusion/exclusion in LOT1 base end logic</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Steroids (corticosteroids) are included in the LOT1 induction medication list (LOT1_BASE_MEDS) but per protocol are NOT counted when determining LOT1 start date (LOT1_START_DT uses first non-steroid MAP). The code includes steroids in the base_meds CTE used for LOT1_BASE_DISCON_DT calculation, meaning steroid MAPs can extend the discontinuation date. This is a deliberate design decision documented in the code with a note that stakeholders may prefer to exclude steroids from the discontinuation computation.</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Steroids are MM therapies and are included in the regimen, but the LOT start is anchored to the first non-steroid therapy. The protocol does not explicitly state whether steroids should extend the discontinuation date, creating ambiguity that the code acknowledges.</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Steroids (corticosteroids) are included in the LOT1 induction medication list (LOT1_BASE_MEDS) but per the updated protocol 'all rules described below are based on oncology therapies only (e.g., not corticosteroids)' (Section 5.1). LOT1_START_DT uses first non-steroid MAP. The code includes steroids in the base_meds CTE used for LOT1_BASE_DISCON_DT calculation, meaning steroid MAPs can extend the discontinuation date. This may conflict with the protocol's intent to exclude steroids from LOT rules. This is a deliberate design decision documented in the code with a note that stakeholders may prefer to exclude steroids from the discontinuation computation.</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Section 5.1 explicitly states: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Also: 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of active MM treatment.' The protocol excludes steroids from LOT rules, but the code includes steroids in the discontinuation calculation - this is a deliberate design decision documented with a code comment for stakeholder review.</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Steroid medications identified via MED_CLASS='STEROID' in CL_MMA_ROLLUP (Tab 40). Steroid claims from T_MEDICAL (PROC_CD/NDC) and T_RX (NDC). Steroid MAPs included in MAP construction and extend MAP_END_DT contributing to LOT1_BASE_DISCON_DT.</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S08 line 3321: LOT1_START_DT = min(MAP_START_DT) WHERE MAP_MED_CLASS &lt;&gt; 'STEROID' (steroids excluded from start date). Step S10 lines 3355-3359: Code comment - 'DECISION: Steroid MAPs are included in base_meds... If stakeholders prefer to exclude steroids from the discontinuation computation, filter base_meds above to exclude steroid MED_CLASS.' Currently steroids ARE included in discon calculation.</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>Spec: - (not documented). Protocol: - (ambiguous on steroid role in discontinuation). Code: Y - steroids included in discontinuation with explicit code comment noting this is a design decision (lines 3355-3359) that stakeholders may want to change.</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr"/>
-      <c r="K30" s="6" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>Spec: - (not documented). Protocol: - (Section 5.1 states 'All rules described below are based on oncology therapies only (e.g., not corticosteroids)' - suggests steroids should be excluded from LOT rules including discontinuation). Code: Y - steroids included in discontinuation with explicit code comment noting this is a design decision (lines 3355-3359) that stakeholders may want to change. POTENTIAL MISALIGNMENT: code includes steroids in discontinuation but protocol excludes them from LOT rules.</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>Design decision missing from original spec. The code includes steroids in the LOT1_BASE_DISCON_DT calculation (lot_program.R Step S10 lines 3355-3359) but documents this as a deliberate choice with a note for stakeholder review. The spec should document whether steroids should extend the discontinuation date, as this directly affects LOT1_BASE_END_DT for patients whose last active medication is a steroid.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>LOT1_TX_ENDDATE_REASON</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>SCT end reason type (AUTO/ALLO/CART)</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Numeric code identifying which SCT type caused the LOT-ending event. Values: 1=AUTO (autologous HSCT), 2=ALLO (allogeneic HSCT), 3=CART (CAR-T cellular therapy). Determined by comparing the earliest LOT-ending date among ENDING_AUTO_DT, FIRST_ALLO_DT, and FIRST_CART_DT. This value is mapped to string end reasons (SCT_AUTO, SCT_ALLO, SCT_CART) in LOT1_BASE_END_REASON.</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1/7: SCT type determines how LOT1 ends. Autologous SCT: single AUTO is allowed within LOT; excess AUTO (2nd for single, 3rd for tandem) ends LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT. The reason type is essential for correctly classifying the end reason.</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 3 - Unplanned SCTs) and Section 5.1 (SCT types): SCT type determines how LOT1 ends. Autologous SCT: single AUTO is allowed within LOT; excess AUTO (2nd for single, 3rd for tandem) ends LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT. The reason type is essential for correctly classifying the end reason.</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>SCT type determined from T_MEDICAL procedure codes matched against CL_SCT_CODELIST (Tab 44) which classifies procedures as AUTO, ALLO, or CART. Priority is earliest LOT-ending date wins.</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S15 lines 3951-3962: LOT1_TX_ENDDATE_REASON = CASE WHEN ENDING_AUTO_DT &lt;= FIRST_ALLO_DT AND ENDING_AUTO_DT &lt;= FIRST_CART_DT THEN 1; WHEN FIRST_ALLO_DT &lt;= FIRST_CART_DT THEN 2; ELSE 3 END. Used in Step S16 lines 4006-4010 to map: 1='SCT_AUTO', 2='SCT_ALLO', 3='SCT_CART'.</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present as standalone variable; only indirectly via end reason codes 5-7). Protocol: - (defines SCT types and their LOT-ending behavior). Code: Y - implemented at Step S15 lines 3951-3962 and consumed by Step S16 lines 4006-4010.</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr"/>
-      <c r="K31" s="6" t="inlineStr">
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec as standalone row. The code computes LOT1_TX_ENDDATE_REASON (lot_program.R lines 3951-3962) to bridge SCT type to end reason. The spec references SCT types indirectly via end reason codes 5=SCT_AUTO, 6=SCT_ALLO, 7=CART but does not define the intermediate reason variable.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>LOT1_TX_AUTO_DT_1 / LOT1_TX_AUTO_DT_2</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>Dates of first and second valid autologous HSCT</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>LOT1_TX_AUTO_DT_1: date of the first valid autologous HSCT after 14-day claim windowing and 60-day gap validation. LOT1_TX_AUTO_DT_2: date of the second valid autologous HSCT (if exists). These dates are the foundation for tandem detection (DT_2 within 180 days of DT_1 with no ALLO between), single AUTO identification, and determining which AUTO event ends the LOT (2nd for single, 3rd for tandem).</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1/7: AUTO SCT dates are identified using a 14-day claim windowing algorithm (claims within 14 days grouped together, selecting the last date in the window). Events must be at least 60 days apart (cfg$sct_auto_gap_days=60). Tandem pair defined as DT_1 and DT_2 within 180 days with no ALLO between them. The spec references these dates extensively in the HSCT extension logic but does not define them as standalone rows.</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1 (Planned Tandem SCT) and Section 5.1.1 (Events that will not end LOT): AUTO SCT dates are identified using a 14-day claim windowing algorithm (claims within 14 days grouped together, selecting the last date in the window). Events must be at least 60 days apart (cfg$sct_auto_gap_days=60). Tandem pair defined as DT_1 and DT_2 within 180 days with no ALLO between them. The spec references these dates extensively in the HSCT extension logic but does not define them as standalone rows.</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>AUTO HSCT dates derived from T_MEDICAL procedure codes (PROC_CD, BILL_PROC_CD) matched against CL_SCT_CODELIST where SCT_TYPE='AUTO'. FST_DT from T_MEDICAL is the raw claim date. 14-day windowing groups claims; 60-day gap validation separates distinct events.</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S13 lines 3620-3793: 14-day windowing algorithm with cfg$sct_auto_window_days=13, cfg$sct_auto_gap_days=60, cfg$sct_tandem_days=180. Step S15 lines 3901-3902: LOT1_TX_AUTO_DT_1 = ap.AUTO_DT_1, LOT1_TX_AUTO_DT_2 = ap.AUTO_DT_2 from auto_pivot CTE. Carried into lot1_base_end at Step S16 lines 3992-3993.</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>Spec: - (referenced in HSCT extension logic but not as standalone rows). Protocol: - (defines AUTO SCT date identification). Code: Y - implemented at Step S13/S15 and output in lot1_base_end view.</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr"/>
-      <c r="K32" s="6" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>Variables missing from original spec as standalone rows. The spec's HSCT extension logic (LOT1_EXTEND_FLG, updated LOT1_END_DT_TEMP) references LOT1_TX_AUTO_DT_1 and _DT_2 extensively but never defines them as their own variables. The code computes them at lot_program.R Step S15 lines 3901-3902 via the 14-day windowing algorithm at Step S13.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_DISCON_DT</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>LOT1 base period discontinuation date</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>The date when all induction medications (including permissible substitutions) are considered discontinued. Computed as max(MAP_END_DT) for all base medication MAPs, but only set when the gap between this date and OBS_END_DT is &gt;= lot_discon_gap_days (default 90 days). If the gap is insufficient, set to NULL (patient is censored, not discontinued). This is one of the candidate dates for LOT1_BASE_END_DT.</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'Discontinuation is defined as the run-out date of all MM treatments in the LOT. Run-out date is the last date that a medication for a specific prescription is considered to be available.' The gap threshold ensures true discontinuation vs censoring near end of follow-up.</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT. Run-out date is the last date that a medication for a specific prescription is considered to be available.' The gap threshold ensures true discontinuation vs censoring near end of follow-up.</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>max(MAP_END_DT) derived from T_MEDICAL (FST_DT + medical_day_supply - 1) and T_RX (FILL_DT + DAYS_SUP - 1) for induction medications matched via CL_MMA_CODELIST. Gap validated against OBS_END_DT from T_MEMBER_CONT_ENROLLMENT/T_DOD.</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S10 lines 3360-3382: discon_raw CTE computes RAW_DISCON_DT = max(MAP_END_DT) for base meds. discon CTE applies gap check: LOT1_BASE_DISCON_DT = RAW_DISCON_DT only WHEN datediff(OBS_END_DT, RAW_DISCON_DT) &gt;= cfg$lot_discon_gap_days (default 90). Otherwise NULL.</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>Spec: - (referenced in min() formula and end reason logic but not defined as standalone row in LOT1_BASE_END tab). Protocol: - (defines discontinuation concept). Code: Y - computed at Step S10 lines 3360-3382.</t>
         </is>
       </c>
-      <c r="J33" s="6" t="inlineStr"/>
-      <c r="K33" s="6" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab as a standalone row. The spec references LOT1_BASE_DISCON_DT in the min() formula for LOT1_END_DT_TEMP and in the end reason logic, but never defines it. It is a key input variable computed at lot_program.R Step S10 lines 3360-3382.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_1ST_ADD_MED_DT / LOT1_BASE_1ST_ADD_MED</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Date and name of first non-induction medication added</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>LOT1_BASE_1ST_ADD_MED_DT: the day before the first MAP_START_DT of a medication NOT in the induction regimen (and not a permissible substitution). This represents when LOT1 ends due to medication addition (MED_ADD end reason). LOT1_BASE_1ST_ADD_MED: the abbreviation of that first added medication (alphabetically first if same-day ties). These are candidate dates/reasons for LOT1_BASE_END_DT/REASON.</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: Addition of a new MM therapy not in the original regimen (and not a permissible substitution) signals the end of the current LOT and start of a new one. The LOT end date is set to the day BEFORE the new medication starts (date_sub(ADD_START_DT, 1)). Per protocol, permissible substitutions (rituximab/hyaluronidase swap, biosimilars, bortezomib-&gt;ixazomib for maintenance) do NOT trigger a new LOT.</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation with new agent): Rule 2: 'With initiation of a new MM agent that was not present in the induction regimen (i.e., the regimen is interrupted by a new agent).' 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Rule 1 (permissible substitutions) does NOT trigger a new LOT. The LOT end date is set to the day BEFORE the new medication starts (date_sub(ADD_START_DT, 1)). Per protocol, permissible substitutions (rituximab/hyaluronidase swap, biosimilars, bortezomib-&gt;ixazomib for maintenance) do NOT trigger a new LOT.</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>First non-induction medication identified from T_MEDICAL (PROC_CD, BILL_PROC_CD, NDC) and T_RX (NDC) matched against CL_MMA_CODELIST (Tab 41) where the medication is NOT in base_meds (induction + permissible subs). MAP_START_DT from MAP algorithm.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>lot_program.R Step S10 lines 3413-3441: first_add_candidates CTE selects non-induction MAPs where bm.MED_ABBR IS NULL (not in base_meds). first_add_dt gets min(MAP_START_DT). first_add_pick computes LOT1_BASE_1ST_ADD_MED_DT = date_sub(ADD_START_DT, 1) and LOT1_BASE_1ST_ADD_MED = min(MAP_MED_TYPE) for determinism (line 3435-3436 comment: 'Spec says random for same-day ties; we use min() for determinism').</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
+      <c r="I34" s="7" t="inlineStr">
         <is>
           <t>Spec: - (referenced in min() and end reason logic but not standalone rows in LOT1_BASE_END tab). Protocol: - (defines new medication addition as LOT-ending event). Code: Y - computed at Step S10 lines 3413-3441. Code note: spec says 'random' for same-day ties but code uses min() (deliberate deviation at line 3435).</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr"/>
-      <c r="K34" s="6" t="inlineStr">
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
         <is>
           <t>Variables missing from original spec's LOT1_BASE_END tab as standalone rows. The spec references LOT1_BASE_1ST_ADD_MED_DT in the min() formula and end reason logic but never defines it. Code deviation: spec says 'random' selection for same-day medication ties; code uses min() for determinism (lot_program.R line 3435). Also: LOT1_BASE_1ST_ADD_MED_DT = date_sub(ADD_START_DT, 1), meaning the end date is the day BEFORE the new med starts.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>INDUCTION_WINDOW_DAYS</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>Induction regimen identification window (days)</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>The number of days from LOT1_START_DT within which all medications are considered part of the induction regimen. Default: 60 days. Any medication with MAP_START_DT within [LOT1_START_DT, LOT1_START_DT + 59] is included in LOT1_BASE_MEDS. Medications starting after this window that are not in the base regimen (or permissible substitutions) trigger LOT1_BASE_1ST_ADD_MED_DT and potentially a MED_ADD end reason.</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'A LOT regimen includes all MM therapies received within 60 (30) days (Madduri, 2021) on and following the start of LOT1 (LOT2-5).' The 60-day window is the primary parameter; 30-day is noted as an alternative from literature. This parameter directly determines what is in the base regimen and therefore what constitutes a 'new' medication triggering MED_ADD. Configurable for sensitivity analysis per Protocol Section 5.3.</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (LOT regimen): 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' For LOT2-5: 'the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' The 60-day window is the primary parameter; 30-day is noted as an alternative from literature. This parameter directly determines what is in the base regimen and therefore what constitutes a 'new' medication triggering MED_ADD. Configurable for sensitivity analysis per Protocol Section 5.3.</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Applied to MAP_START_DT from T_MEDICAL/T_RX claims. Medications with MAP_START_DT within the window are classified as induction via CL_MMA_CODELIST/CL_MMA_ROLLUP matching.</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>lot_program.R line 71: induction_window_days = as.integer(Sys.getenv('INDUCTION_WINDOW_DAYS', unset = '60')). Step S09 line 3338: WHERE ms.MAP_START_DT &lt;= date_add(l1.LOT1_START_DT, {cfg$induction_window_days - 1}). Configurable via INDUCTION_WINDOW_DAYS env var.</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr">
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not documented as a parameter in LOT1_BASE_END tab). Protocol: - (defines 60-day window). Code: Y - implemented as configurable parameter at line 71, used at line 3338.</t>
         </is>
       </c>
-      <c r="J35" s="6" t="inlineStr"/>
-      <c r="K35" s="6" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses induction_window_days=60 (lot_program.R line 71) to determine which medications are in the induction regimen. This is critical: it directly controls what triggers MED_ADD end reason. Protocol Section 5.1.1 specifies 60 days (with 30-day alternative from Madduri 2021).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>ALLO_ALWAYS_ENDS_LOT</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>Allogeneic SCT always ends current LOT (protocol rule)</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Protocol rule: Any allogeneic HSCT immediately ends the current line of therapy. The LOT end date is set to the day before the ALLO SCT date. An auto-to-allo sequence is NOT considered a planned tandem and indicates treatment failure. This is a hard rule with no exceptions - ALLO SCT has the same LOT-ending priority as any other SCT in the code's CASE statement.</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Also: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Additionally, the presence of an ALLO between two AUTO SCTs invalidates the tandem classification (coalesce(n_allo_between, 0) = 0 required for tandem).</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): Section 5.1: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Section 5.1.1 (Rule 3): 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Also: 'Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.' Also: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Additionally, the presence of an ALLO between two AUTO SCTs invalidates the tandem classification (coalesce(n_allo_between, 0) = 0 required for tandem).</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>ALLO SCT identified from T_MEDICAL procedure codes matched against CL_SCT_CODELIST where SCT_TYPE='ALLO'. Date from FST_DT in T_MEDICAL.</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>lot_program.R: ALLO always ends LOT implemented via: (1) FIRST_ALLO_DT captured at Step S14 lines 3796-3825 and Step S15 line 3929. (2) LOT1_TX_ENDDATE includes ALLO at lines 3939-3949: least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT) - 1. (3) ALLO between AUTOs invalidates tandem at line 3907: coalesce(ab.n_allo_between, 0) = 0. (4) Step S16 line 4008: LOT1_TX_ENDDATE_REASON=2 maps to 'SCT_ALLO'.</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>Spec: - (implicit via SCT_ALLO end reason code 6 but not stated as an explicit rule). Protocol: - (explicit rule in Section 5.1.1). Code: Y - implemented via ALLO priority in LOT1_TX_ENDDATE and tandem invalidation.</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr"/>
-      <c r="K36" s="6" t="inlineStr">
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
         <is>
           <t>Protocol rule not explicitly stated in original spec. The spec has SCT_ALLO as end reason code 6 but does not document the rule that ALLO always ends the LOT unconditionally, or that auto-to-allo is not considered planned. The code implements this at lot_program.R via FIRST_ALLO_DT inclusion in LOT1_TX_ENDDATE (lines 3939-3949) and tandem invalidation (line 3907).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>CART_30D_CONSOLIDATION</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>CAR-T 30-day supportive agent consolidation rule</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Protocol rule: Therapies (including supportive agents such as corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT, not the preceding LOT. This means medications administered near a CAR-T event should be attributed to the CAR-T LOT rather than LOT1. This rule is NOT currently implemented in the code.</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.2: 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' This 30-day window affects medication attribution near the LOT1/CAR-T boundary. Without this rule, medications given in the 30 days before CAR-T could incorrectly extend LOT1's discontinuation date or trigger a MED_ADD end reason.</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 (CAR-T): 'CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' (Section 5.1.1) This 30-day window affects medication attribution near the LOT1/CAR-T boundary. Without this rule, medications given in the 30 days before CAR-T could incorrectly extend LOT1's discontinuation date or trigger a MED_ADD end reason.</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Would require checking T_MEDICAL/T_RX claims within 30 days of FIRST_CART_DT and reclassifying them from LOT1 to the CAR-T LOT. Affects MAP_END_DT for induction meds and MAP_START_DT for potential new meds.</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>lot_program.R: NOT IMPLEMENTED. The code treats CAR-T as a simple LOT-ending event (Step S14 lines 3796-3825: CART dates extracted; Step S15 line 3930: FIRST_CART_DT captured). LOT1 ends the day before CART (LOT1_TX_ENDDATE = date_sub(FIRST_CART_DT, 1) at lines 3939-3949). No 30-day consolidation window is applied to reclassify medications near the CAR-T boundary.</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>--N</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (defined in Section 5.1.2). Code: N - not implemented; CAR-T simply ends LOT1 without 30-day medication reclassification.</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr"/>
-      <c r="K37" s="6" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.2 specifies that therapies within 30 days of CAR-T are consolidated as part of the CAR-T LOT. The code does not implement this 30-day consolidation window. Impact: medications given in the 30 days before CAR-T could incorrectly influence LOT1's DISCON_DT or trigger MED_ADD. This should be implemented for correct medication attribution near CAR-T events.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>MESNA_EXCLUSION</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>Mesna excluded from LOT definition</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>Protocol rule: Mesna is excluded from LOT definitions. Mesna is a supportive agent used to protect the bladder against toxic side-effects of certain anticancer drugs (e.g., cyclophosphamide conditioning). Mesna claims should NOT be counted as MM therapy and should NOT trigger MED_ADD end reason or contribute to MAP coverage calculations.</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>Protocol Section 5.1.1: 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion beyond the general steroid handling. Mesna should be excluded from CL_MMA_CODELIST or filtered out during medication identification.</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1 (MM therapies): 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion beyond the general steroid handling. Mesna should be excluded from CL_MMA_CODELIST or filtered out during medication identification.</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Mesna identified via NDC codes in T_RX or HCPCS codes in T_MEDICAL. Should be excluded from CL_MMA_CODELIST (Tab 41) or filtered during MMA claim extraction in Step S05 (mma_med).</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>lot_program.R: Mesna is not explicitly referenced in the code. It is likely excluded by not being present in the CL_MMA_CODELIST/CL_MMA_ROLLUP codelists (Tab 40/41). If mesna codes ARE in the codelist, they would incorrectly be treated as MM therapy. Verification would require checking the codelist contents.</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>--?</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (explicit exclusion in Section 5.1.1). Code: ? - likely excluded by omission from codelist but not explicitly filtered. Cannot confirm without checking codelist contents.</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr"/>
-      <c r="K38" s="6" t="inlineStr">
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
         <is>
           <t>Protocol exclusion rule not in original spec. Protocol Section 5.1.1 explicitly excludes mesna from LOTs. The code likely handles this by not including mesna in CL_MMA_CODELIST/CL_MMA_ROLLUP, but this should be verified. If mesna codes were inadvertently included in the codelist, they would incorrectly affect LOT1 end date calculations.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>NAMING_DISCREPANCY_SCT_VS_HSCT</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Variable naming: spec uses HSCT prefix vs code uses SCT prefix</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>The original spec names autologous transplant flags as LOT1_HSCT_AUTO_SING_FLG and LOT1_HSCT_AUTO_TAND_FLG (using 'HSCT' prefix). The code names them LOT1_SCT_AUTO_SING_FLG and LOT1_SCT_AUTO_TAND_FLG (using 'SCT' prefix). Both refer to the same variables. This naming inconsistency should be reconciled.</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>Protocol uses 'SCT' (Stem Cell Transplant) terminology consistently. The spec uses 'HSCT' (Hematopoietic Stem Cell Transplant). Both are acceptable medical abbreviations for the same concept. The code aligns with the protocol's 'SCT' convention.</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>N/A - naming convention only.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>lot_program.R: Uses SCT prefix consistently: LOT1_SCT_AUTO_SING_FLG (line 3917), LOT1_SCT_AUTO_TAND_FLG (line 3909). CL_SCT_CODELIST table name also uses SCT. Configuration parameters use sct_ prefix (sct_auto_window_days, sct_auto_gap_days, sct_tandem_days at lines 87-89).</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>N-Y</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>Spec: N - uses HSCT prefix (LOT1_HSCT_AUTO_*). Protocol: - (uses SCT terminology). Code: Y - uses SCT prefix (LOT1_SCT_AUTO_*) matching protocol convention.</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr"/>
-      <c r="K39" s="6" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>Naming discrepancy: spec uses LOT1_HSCT_AUTO_SING_FLG / LOT1_HSCT_AUTO_TAND_FLG while code uses LOT1_SCT_AUTO_SING_FLG / LOT1_SCT_AUTO_TAND_FLG. Recommend aligning spec to use SCT prefix to match both code and protocol convention.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L39"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revise Definition column to contain only protocol-sourced text
Removed code implementation details and interpretive additions from
the Definition (Validated from Protocol) column across all 38 rows.
Each definition now contains only direct quotes and references from
the LOT protocol PDF (Sections 5.1 and 5.1.1). Regenerated Excel.

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -10,7 +10,7 @@
     <sheet name="LOT1 Base End Validated" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LOT1 Base End Validated'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LOT1 Base End Validated'!$A$1:$L$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,15 +28,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,20 +59,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -98,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,9 +112,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,14 +482,14 @@
   <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -583,7 +576,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The earliest nonmissing date among: LOT1_BASE_DISCON_DT (last MAP_END_DT for induction meds with sufficient gap to observation end), ENDDATE (earliest of study end or death), LOT1_BASE_1ST_ADD_MED_DT (day before first non-induction medication), and LOT1_TX_ENDDATE (day before LOT-ending SCT event). The code determines the end date using a priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) rather than a simple min() of all dates. The protocol requires that LOT1 ends at the earliest qualifying event. Note: LOT1_BASE_MAINT_END_DT_TEMP is listed in the original spec's min() but maintenance is not enabled and is intentionally out of scope in the current implementation.</t>
+          <t>The LOT will continue until the earliest of any of the following events (Protocol Section 5.1.1, Rules 1-8): (1) substitution of a biologic reference product with any of its biosimilars does not advance the LOT; (2) discontinuation of all agents in the regimen - the LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available; (3) unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, the LOT will end the day before the latter SCT; any allogeneic SCTs are considered a new LOT; (4) SCTs not followed by maintenance within 180 days - the last day of the LOT is the date of the SCT; (5) death; (6) health plan disenrollment; (7) end of the study period; (8) end of maintenance regimen.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -640,7 +633,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>A copy of the originally calculated LOT1 base period end date, preserved before any HSCT extension logic modifies LOT1_END_DT_TEMP. This allows tracking how much the LOT1 end date was extended if an HSCT occurred within the extension window.</t>
+          <t>The protocol defines LOT1 end date determination (Section 5.1.1) but does not explicitly specify preserving the original date as a separate variable before HSCT extension. This variable is an implementation artifact from the original program spec; it has no direct protocol equivalent.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -658,7 +651,7 @@
           <t>lot_program.R: No direct equivalent variable. The code computes LOT1_BASE_END_DT in a single CASE statement (lines 4018-4028) without a multi-step temporary approach. The HSCT extension logic described in the spec (extending LOT1 by 60 days to capture an HSCT) is handled differently in the code: SCT events are evaluated in the priority-based end reason logic at Step S16 (lines 4001-4017) where SCT takes highest priority, so if an SCT occurs before other end events, it directly sets the end date.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>NYN</t>
         </is>
@@ -697,7 +690,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>The reason why LOT1 base period ended. Determined by matching LOT1_END_DT_TEMP against candidate end dates. Values: 1=DISCONTINUATION (LOT1_END_DT_TEMP matches LOT1_DISCON_DT), 2=NEW MED ADD (matches LOT1_BASE_1ST_ADD_MED_DT), 3=CENSOR (matches ENDDATE), 4=DEATH (matches DEATH_DT), 5=SCT_AUTO (matches LOT1_TX_ENDDATE with TX_ENDDATE_REASON=1), 6=SCT_ALLO (matches LOT1_TX_ENDDATE with TX_ENDDATE_REASON=2), 7=CART (matches LOT1_TX_ENDDATE with TX_ENDDATE_REASON=3). The code uses string-valued end reasons and a priority-based approach rather than numeric codes with date-matching.</t>
+          <t>Per Protocol Section 5.1.1, the LOT ends for one of these reasons: (Rule 2) Discontinuation of all agents in the regimen, with or without switch to a new agent; (Rule 2) If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent; (Rule 3) Unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, or any allogeneic SCT; (Rule 4) SCTs not followed by maintenance within 180 days; (Rule 5) Death; (Rule 6) Health plan disenrollment; (Rule 7) End of the study period; (Rule 8) End of maintenance regimen.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -754,7 +747,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Flag (0/1) indicating the patient had an autologous HSCT occurring within 60 days of LOT1 ending due to discontinuation. Conditions per spec: LOT1_END_REASON_TEMP = 1 (DISCONTINUATION) AND (LOT1_HSCT_AUTO_TAND_FLG or LOT1_HSCT_AUTO_SING_FLG) AND LOT1_END_DT_TEMP &lt;= LOT1_TX_AUTO_DT_1 &lt;= LOT1_END_DT_TEMP + 60 AND (missing(LOT1_TX_ENDDATE) or LOT1_TX_AUTO_DT_1 &lt;= ENDDATE). If all conditions met, the LOT1 end date is extended to include the HSCT. The code does NOT implement this variable; instead SCT events are evaluated directly in the end reason priority logic.</t>
+          <t>Per Protocol Section 5.1.1: 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum's KOL and informed by Charalampous et al.'s findings that the median time from end of induction to transplant was 33 days (interquartile range=27-42).' Single autologous SCTs and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.'</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -772,7 +765,7 @@
           <t>lot_program.R: LOT1_EXTEND_FLG is NOT directly implemented. The code's approach at Step S16 (lines 4001-4017) gives SCT highest priority: if LOT1_TX_ENDDATE (SCT end minus 1 day) occurs at or before DISCON_DT and ADD_MED_DT, then end reason = SCT_AUTO/SCT_ALLO/SCT_CART. The SCT dates are computed at Step S15 (lines 3897-3983) with 14-day windowing (cfg$sct_auto_window_days=13), 60-day gap (cfg$sct_auto_gap_days=60), and 180-day tandem (cfg$sct_tandem_days=180). The conditioning period concept is implicitly handled by the SCT date processing at lines 3620-3793.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>NNY</t>
         </is>
@@ -811,7 +804,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>The number of days between the conditioning period's discontinuation date and an HSCT that occurred at least within the extension window. Per spec: if LOT1_EXTEND_FLG then = LOT1_END_DT_TEMP - LOT1_END_DT_ORIG. This measures how much the LOT1 end date was pushed out to accommodate the HSCT. The code does not implement this variable.</t>
+          <t>The protocol does not define a named variable for the number of days between discontinuation and HSCT. The concept is implied by the 60-day SCT extension rule (Section 5.1.1): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.'</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -829,7 +822,7 @@
           <t>lot_program.R: NOT IMPLEMENTED. The code does not compute LOT1_EXTEND_LENGTH because it does not use the multi-step TEMP/ORIG extension approach. The code computes LOT1_BASE_END_DT directly (lines 4018-4028). If the equivalent metric is needed, it could be derived as datediff(LOT1_TX_AUTO_DT_1 or _DT_2, LOT1_BASE_DISCON_DT) from the lot1_base_end view.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>NNY</t>
         </is>
@@ -868,7 +861,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>The base period end reason updated after HSCT extension and same-class switching considerations. Per spec: same values as LOT1_END_REASON_TEMP (1=DISCONTINUATION through 7=CART). If LOT1_EXTEND_FLG then the end reason may change to reflect HSCT-based ending. Otherwise leave unchanged from LOT1_END_REASON_TEMP. The code handles this in a single step via the priority CASE statement.</t>
+          <t>The protocol does not define a 'SWITCH' concept for end reasons. The protocol's LOT end rules (Section 5.1.1, Rules 1-8) define the final end reason directly without an intermediate update step. This variable is a spec-level implementation detail with no direct protocol equivalent.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -886,7 +879,7 @@
           <t>lot_program.R: NOT IMPLEMENTED as a separate variable. The code's LOT1_BASE_END_REASON (Step S16 lines 4001-4017) is the final end reason computed in a single pass. There is no intermediate 'SWITCH' step. The end reason directly accounts for SCT priority. The maintenance-related updates described in the spec (where end reason changes based on maintenance after HSCT) are not yet implemented (line 4037-4038).</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>NNY</t>
         </is>
@@ -925,7 +918,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Flag (0/1) indicating the patient had a same-class medication during LOT1 BASE period. Per spec: if LOT1_SAME_CLASS_1ST_DT &lt;= LOT1_END_DT_TEMP then = 1, else = 0. This identifies patients who switched to a different medication within the same drug class during their induction therapy.</t>
+          <t>The protocol does not define a same-class switch flag. Per Protocol Section 5.1.1 Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.'</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -943,7 +936,7 @@
           <t>lot_program.R: SWITCH_FLG is NOT IMPLEMENTED. The code does track LOT1_CLASS_* flags (e.g., LOT1_CLASS_PROTINHIB, LOT1_CLASS_IMMUNOMOD) via med_summary at Step S10 (lines 3389-3390) to identify which drug classes are in the induction regimen. Permissible substitutions are handled at lines 3346-3354 (base_meds CTE includes permissible_subs). However, there is no explicit SWITCH_FLG or LOT1_SAME_CLASS_1ST_DT variable computed. LOT1_SAME_CLASS_1ST_DT is not defined in the code.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>NNY</t>
         </is>
@@ -982,7 +975,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Flag (0/1) indicating the patient had a single valid autologous HSCT (not part of a valid tandem). Set to 1 when AUTO_DT_1 exists but the patient does NOT have a valid tandem (either no AUTO_DT_2, or AUTO_DT_2 is more than 180 days from AUTO_DT_1, or there is an ALLO between them). Per spec: updated based on whether LOT1 base ends before HSCT date (if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 then set to 0).</t>
+          <t>Per Protocol Section 5.1: 'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT. SCT is operationalized as &gt;1 procedure code for an SCT.' A single autologous SCT is one that is not part of a valid tandem pair. Per Section 5.1.1: 'Single autologous SCTs and tandem SCTs are not unplanned SCTs and are considered a continuation of the line of therapy.'</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1039,7 +1032,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Flag (0/1) indicating the patient had a valid tandem autologous HSCT. Set to 1 when two AUTO transplants occur within 180 days of each other with no allogeneic (ALLO) transplant between them. Per spec: updated based on whether LOT1 base ends before HSCT date (if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 then set to 0).</t>
+          <t>Per Protocol Section 5.1: 'Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart; otherwise, they will be considered unplanned (Rajkumar, 2015). An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Per Section 5.1.1: 'Tandem SCTs are two SCTs &gt;60 to &lt;180 days apart. These are considered planned and a continuation of the line of therapy.'</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1096,7 +1089,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The latest date of a patient's valid autologous HSCT. Per spec: if LOT1_HSCT_AUTO_TAND_FLG then = LOT1_TX_AUTO_DT_2; else if LOT1_HSCT_AUTO_SING_FLG then = LOT1_TX_AUTO_DT_1. This represents the most recent valid AUTO transplant date for the patient.</t>
+          <t>The protocol does not define this as a named variable. Per Protocol Section 5.1: tandem SCTs are two autologous SCTs &gt;60 to &lt;180 days apart. The latest valid AUTO date is the second SCT for tandem patients or the first SCT for single-AUTO patients. Per Section 5.1.1: 'Single autologous SCTs and tandem stem-cell transplants (SCT) &lt;180 days apart' are considered a continuation of the LOT.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1153,7 +1146,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Flag (0/1) indicating the patient had any valid autologous HSCT. Per spec: if (LOT1_HSCT_AUTO_TAND_FLG or LOT1_HSCT_AUTO_SING_FLG) then = 1, else = 0. This is a convenience flag combining single and tandem.</t>
+          <t>Per Protocol Section 5.1: 'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT.' This binary variable indicates whether the patient received any valid autologous transplant, regardless of single or tandem.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1210,7 +1203,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>If LOT1_EXTEND_FLG = 1 and LOT1_HSCT_AUTO_SING_FLG, update LOT1_END_DT_TEMP to LOT1_TX_AUTO_DT_1. If LOT1_HSCT_AUTO_TAND_FLG, update to LOT1_TX_AUTO_DT_2. Per spec: this extends the LOT1 end date to the date of the HSCT (or second HSCT for tandem). The code handles this via SCT priority in the end reason CASE statement.</t>
+          <t>Per Protocol Section 5.1.1: 'Single autologous SCT or tandem stem-cell transplants (SCT) &lt;180 days apart: SCTs are usually preceded by induction therapy and followed by consolidation and maintenance therapy.' These are 'considered planned and a continuation of the line of therapy.' 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.'</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1228,7 +1221,7 @@
           <t>lot_program.R: The code does not update LOT1_END_DT_TEMP iteratively. Instead, LOT1_BASE_END_DT (Step S16 lines 4018-4028) is set to LOT1_TX_ENDDATE when SCT has priority. LOT1_TX_ENDDATE = date_sub(least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT), 1) at lines 3939-3949. For single AUTO, ENDING_AUTO_DT = AUTO_DT_2 (the LOT-ending event, line 3926). For tandem, ENDING_AUTO_DT = AUTO_DT_3 (line 3924). Note: the code's LOT1_TX_ENDDATE is the day BEFORE the LOT-ending SCT, not the date of the included SCT.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>NNY</t>
         </is>
@@ -1267,7 +1260,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Space-separated sorted list of induction medication abbreviations. Originally from the LOT1_BASE dataset. Includes all medications (including permissible substitutions) with MAP_START_DT within the induction window (default 60 days) from LOT1_START_DT. Steroid MAPs are included in the medication list. Example values: 'BORT LENA', 'DARA LENA', 'BORT DARA LENA'.</t>
+          <t>Per Protocol Section 5.1.1: 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date. For LOT1, the first therapy received is considered the induction therapy.' Per Section 5.1.1 Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT.' All rules are 'based on oncology therapies only (e.g., not corticosteroids).'</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1285,7 +1278,7 @@
           <t>lot_program.R Step S09 lines 3327-3341: lot1_induction_meds selects DISTINCT PATID, MED_ABBR, MED_CLASS where MAP_START_DT between LOT1_START_DT and LOT1_START_DT + induction_window_days - 1. Step S10 line 3388: LOT1_BASE_MEDS = concat_ws(' ', sort_array(collect_set(im.MED_ABBR))). Permissible substitutions added at lines 3346-3354.</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>YYY</t>
         </is>
@@ -1324,7 +1317,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>The start date of a maintenance period following LOT1 base therapy. Per spec: set to LOT1_BASE_MAINT_START_DT from the LOT1_BASE_MAINT input dataset if certain conditions are met (minimum gap from base end date to maintenance start &gt;= 120 days, and maintenance start occurs before other end events). Otherwise set to missing.</t>
+          <t>Per Protocol Section 5.1: 'A maintenance regimen is a period of 120 days or longer during which only a valid maintenance therapy is available. Maintenance is not required to be prescribed continuously for the duration of the 120 day period. Furthermore, the maintenance therapy must have been a part of the LOT's initial regimen.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1342,7 +1335,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED. Line 4037-4038: 'NOTE: Maintenance (mono/dual) specs not yet provided; LOT1_BASE_END_REASON does not yet include MAINTENANCE_START. Will need integration when available.' Maintenance is intentionally out of scope in the current implementation. Maintenance analysis exists separately in lot_analysis.R lines 1224-1350 for reporting but is not integrated into the LOT1 end date/reason computation.</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1381,7 +1374,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>The abbreviation of the maintenance medication type. Per spec: if LOT1_MAINT_START_DT is not missing, set to LOT1_MAINT_TYPE from the LOT1_BASE_MAINT input dataset. Otherwise set to missing.</t>
+          <t>Per Protocol Section 5.1: valid maintenance therapies per NCCN Guidelines include lenalidomide monotherapy, bortezomib monotherapy, daratumumab monotherapy, ixazomib monotherapy, thalidomide monotherapy, bortezomib/lenalidomide dual, carfilzomib/lenalidomide dual, and daratumumab/lenalidomide dual. MAINTENANCE IS NOT ENABLED in the current implementation.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1399,7 +1392,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED (see line 4037-4038). Maintenance type tracking exists in lot_analysis.R for analysis purposes but is not connected to LOT1_BASE_END. Intentionally out of scope.</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1438,7 +1431,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>The temporary end date of a maintenance period. Per spec: Complex logic based on LOT1_MAINT_ADD_FLG and comparison with min(LOT1_BASE_DISCON_DT, ENDDATE, LOT1_BASE_1ST_ADD_MED_DT, LOT1_TX_ENDDATE). If LOT1_MAINT_ADD_FLG=1 and LOT1_BASE_MAINT_END_DT_TEMP &lt; min of the end dates, then set to LOT1_BASE_MAINT_END_DT_TEMP from the input dataset. Otherwise set to the value of LOT1_END_DT_TEMP calculated above.</t>
+          <t>Per Protocol Section 5.1: 'Once a maintenance regimen has begun, it continues until discontinuation, presence of an SCT, right censoring (i.e. end of follow-up), or the addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1456,7 +1449,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED (see line 4037-4038). The spec describes complex maintenance end date logic involving LOT1_MAINT_ADD_FLG and comparison with multiple end dates, none of which are currently computed. Intentionally out of scope.</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1495,7 +1488,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Flag (0/1) for each maintenance medication. Per spec: For [MED] in (BORT, DARA, IXAZ, LENA, CARF): if LOT1_MAINT_START_DT is not missing, set to LOT1_MAINT_MED_[MED] from the LOT1_BASE_MAINT input dataset. Otherwise set to missing. These flags identify which specific medications are used in the maintenance regimen.</t>
+          <t>Per Protocol Section 5.1: valid maintenance therapies per NCCN Guidelines (Kumar, 2020) include mono-maintenance (lenalidomide, bortezomib, daratumumab, ixazomib, thalidomide) and dual-maintenance (bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide). 'Any of the maintenance medications listed above will be considered maintenance medications for all patients, regardless of transplant status.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1513,7 +1506,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED. Induction medication flags (LOT1_MED_BORT, LOT1_MED_DARA, etc.) exist at Step S10 lines 3389 via med_flag_exprs (lines 2886-2889). Maintenance-specific flags (LOT1_BASEMAINT_MED_BORT, etc.) are not computed. Intentionally out of scope.</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1552,7 +1545,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>The reason why the maintenance period ended. Per spec: values 1=DISCONTINUATION, 2=NEW MED ADD, 3=CENSOR, 4=DEATH, 5=HSCT AUTO, 6=HSCT ALLO. Logic: if LOT1_MAINT_START_DT is not missing: if LOT1_BASEMAINT_END_DT_TEMP = LOT1_BASE_MAINT_END_DT_TEMP and LOT1_MAINT_ADD_FLG=1 then set to 2; where LOT1_BASEMAINT_END_DT_TEMP is defined on the input dataset (LOT1_BASE_MAINT). Otherwise set to the value of LOT1_END_REASON_TEMP calculated above.</t>
+          <t>Per Protocol Section 5.1.1 Rule 8: 'The LOT will end after a maintenance regimen ends due to: unplanned SCTs, death, health plan disenrollment, and end of study period.' Per Section 5.1: 'The addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1570,7 +1563,7 @@
           <t>lot_program.R: MAINTENANCE IS NOT ENABLED (see line 4037-4038). The spec describes maintenance end reason logic that depends on LOT1_MAINT_ADD_FLG and LOT1_BASE_MAINT_END_DT_TEMP, neither of which are computed. Intentionally out of scope. Note: end reason values in spec are numeric (1-6) while the code uses string values for the base end reason.</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>N-N</t>
         </is>
@@ -1592,1147 +1585,1147 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>LOT1_BASE_END_DT</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Final LOT1 base period end date</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>The final computed end date for the LOT1 base period after all adjustments (SCT evaluation, HSCT extension, maintenance integration). This is the definitive end date used for downstream analysis. In the code, this is directly computed via a priority-based CASE statement: (1) LOT1_TX_ENDDATE if SCT has priority, (2) LOT1_BASE_1ST_ADD_MED_DT if medication addition, (3) LOT1_BASE_DISCON_DT if discontinuation, (4) OBS_END_DT if censored.</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1: 'The LOT will continue until the earliest of any of the following' (Rules 1-8). The LOT end date is the final computed date after evaluating all end conditions. Per Rule 2: 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.' 'If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent.'</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (LOT end date, Rules 1-8): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. This final variable should be the non-temporary version after all adjustments. The original spec only defines TEMP versions but never creates the final LOT1_BASE_END_DT.</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>LOT1_BASE_END_DT derived from priority evaluation of dates from T_MEDICAL/T_RX (MAP_END_DT for discontinuation, MAP_START_DT for new med), T_MEDICAL procedure codes (SCT events), T_DOD (YMDOD for death), T_MEMBER_CONT_ENROLLMENT (ELIGEND for disenrollment), and study_end config parameter.</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S16 lines 4018-4028: LOT1_BASE_END_DT = CASE WHEN SCT priority THEN sct.LOT1_TX_ENDDATE; WHEN MED_ADD priority THEN lb.LOT1_BASE_1ST_ADD_MED_DT; WHEN DISCON THEN lb.LOT1_BASE_DISCON_DT; ELSE lb.OBS_END_DT END. This is the final (non-temporary) end date used in the lot1_base_end view.</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (defines end date concept but spec only has TEMP versions). Code: Y - implements LOT1_BASE_END_DT as the final computed end date. This variable is missing from the original spec which only has LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never creates the final non-temporary version.</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never defines the final LOT1_BASE_END_DT. The code creates this as the definitive end date at lot_program.R Step S16 lines 4018-4028. The spec should include this final variable to show the output of the LOT1_BASE_END section.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>LOT1_BASE_END_REASON</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Final LOT1 base period end reason</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>The final computed end reason for the LOT1 base period. Values: 'DISCONTINUATION' (all induction meds ran out with sufficient gap), 'MED_ADD' (new non-induction medication added), 'CENSORED' (end of observation - death/disenrollment/study end), 'SCT_AUTO' (LOT ended by autologous transplant), 'SCT_ALLO' (LOT ended by allogeneic transplant), 'SCT_CART' (LOT ended by CAR-T therapy). Priority: SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED.</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1: LOT ends for one of the following reasons (Rules 1-8): (1) permissible substitution (does not end LOT); (2) discontinuation of all agents; (3) unplanned SCTs; (4) SCTs not followed by maintenance within 180 days; (5) death; (6) health plan disenrollment; (7) end of study period; (8) end of maintenance regimen.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (highest priority - allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. The original spec only defines TEMP and SWITCH versions with numeric codes but never creates the final string-valued LOT1_BASE_END_REASON.</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>End reason derived from evaluation of dates across T_MEDICAL/T_RX (medication events), T_MEDICAL (SCT procedure codes), T_DOD (death), and T_MEMBER_CONT_ENROLLMENT (disenrollment). Priority logic applied analytically.</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S16 lines 4001-4017: LOT1_BASE_END_REASON = CASE WHEN SCT AND earliest THEN 'SCT_AUTO'/'SCT_ALLO'/'SCT_CART'; WHEN MED_ADD AND earliest THEN 'MED_ADD'; WHEN DISCON THEN 'DISCONTINUATION'; ELSE 'CENSORED' END. QC query at lines 4032-4035 produces distribution of end reasons.</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present as final variable; only TEMP and SWITCH versions). Protocol: - (defines end reasons conceptually). Code: Y - implements LOT1_BASE_END_REASON as the final string-valued end reason.</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_REASON_TEMP and LOT1_END_REASON_SWITCH with numeric codes (1-7) but never creates the final LOT1_BASE_END_REASON. The code creates this with string values at lot_program.R Step S16 lines 4001-4017.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>LOT1_1ST_SCT_DT</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Date of first SCT event of any type during LOT1</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>The earliest SCT event (autologous, allogeneic, or CAR-T) occurring during the LOT1 period. Computed as LEAST(LOT1_TX_AUTO_DT_1, FIRST_ALLO_DT, FIRST_CART_DT). This date is relevant for determining when SCT-related treatment changes begin and for calculating intervals between induction end and transplant.</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1: 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum's KOL and informed by Charalampous et al.'s findings that the median time from end of induction to transplant was 33 days (interquartile range=27-42) (Charalampous, 2023).'</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Events that will not end LOT): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.' LOT1_1ST_SCT_DT enables validation of this 60-day window rule.</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>First SCT date derived from T_MEDICAL procedure codes matching CL_SCT_CODELIST entries (Tab 44). AUTO type identified by SCT_TYPE='AUTO'; ALLO by SCT_TYPE='ALLO'; CAR-T by SCT_TYPE='CART'. Dates from FST_DT in T_MEDICAL after 14-day claim windowing and 60-day gap validation.</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S15 lines 3963-3972: LOT1_1ST_SCT_DT = CASE WHEN any SCT date exists THEN least(coalesce(AUTO_DT_1, '9999-12-31'), coalesce(FIRST_ALLO_DT, '9999-12-31'), coalesce(FIRST_CART_DT, '9999-12-31')) ELSE NULL END. Carried into lot1_base_end view at Step S16 line 3998.</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (concept exists via 60-day SCT window rule). Code: Y - implemented at Step S15 lines 3963-3972 and carried through to lot1_base_end.</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K22" s="7" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code computes LOT1_1ST_SCT_DT at lot_program.R Step S15 (lines 3963-3972) as the earliest SCT of any type. This is useful for validating the protocol's 60-day window rule (SCT must occur within 60 days of induction/maintenance end to be continuation of LOT). The spec should include this variable.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>FIRST_ALLO_DT</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Date of first allogeneic HSCT during LOT1</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>The date of the first allogeneic (ALLO) HSCT occurring during the LOT1 period. Per protocol, any allogeneic SCT always ends the current LOT because an allogeneic SCT typically follows failed autologous SCTs and represents a fundamentally different treatment approach.</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1: 'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Per Section 5.1.1 Rule 3: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Per Section 5.1.1 (LOT Classification): 'Allogeneic SCT: Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.'</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' (Section 5.1). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs' (Section 5.1.1, Rule 3). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' This is a hard rule - ALLO always ends the LOT regardless of timing relative to other events.</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>ALLO SCT identified from T_MEDICAL procedure codes matching CL_SCT_CODELIST entries where SCT_TYPE='ALLO'. Date from FST_DT in T_MEDICAL. Sequential ordering applied to identify first ALLO event.</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S14 lines 3796-3825: tx_allo_cart_dates extracts ALLO dates from sct_events. Step S15 line 3929: FIRST_ALLO_DT = fa.ALLO_DT from first_allo CTE. Carried into lot1_base_end at Step S16 line 3999. Used in LOT1_TX_ENDDATE calculation (lines 3939-3949) and LOT1_TX_ENDDATE_REASON (lines 3951-3962).</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present as standalone variable; referenced indirectly via SCT_ALLO end reason). Protocol: - (defines ALLO as always ending LOT). Code: Y - implemented at Step S15 line 3929 and used in end date/reason calculations.</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_ALLO_DT at lot_program.R Step S15 (line 3929) and uses it in the LOT1_TX_ENDDATE and LOT1_TX_ENDDATE_REASON calculations. The protocol explicitly states that any ALLO SCT ends the current LOT (Section 5.1.1). The spec references SCT_ALLO as end reason code 6 but does not define FIRST_ALLO_DT as a standalone variable.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>FIRST_CART_DT</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Date of first CAR-T therapy during LOT1</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>The date of the first CAR-T cellular therapy occurring during the LOT1 period. Per protocol, CAR-T therapy starts a new LOT, so the current LOT ends the day before the CAR-T date. Supportive agents (including corticosteroids) given within 30 days of CAR-T are consolidated as part of the CAR-T LOT.</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 (LOT Classification): 'CAR-T: CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (CAR-T): 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' CAR-T always starts a new LOT, ending the current one. The 30-day supportive agent consolidation rule means medications within 30 days of CAR-T are attributed to the CAR-T LOT, not the preceding LOT.</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>CAR-T identified from T_MEDICAL procedure codes matching CL_SCT_CODELIST entries where SCT_TYPE='CART'. Date from FST_DT in T_MEDICAL.</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S14 lines 3796-3825: tx_allo_cart_dates extracts CART dates from sct_events. Step S15 line 3930: FIRST_CART_DT = fc.CART_DT from first_cart CTE. Carried into lot1_base_end at Step S16 line 4000. Used in LOT1_TX_ENDDATE (lines 3939-3949) and LOT1_TX_ENDDATE_REASON (lines 3951-3962, mapped to reason=3='SCT_CART').</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present as standalone variable; referenced indirectly via CART end reason code 7). Protocol: - (defines CAR-T as starting new LOT with 30-day consolidation rule). Code: Y - implemented at Step S15 line 3930.</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K24" s="7" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_CART_DT at lot_program.R Step S15 (line 3930). The protocol defines CAR-T as always starting a new LOT (Section 5.1.2) with a 30-day supportive agent consolidation rule. The spec has CART as end reason code 7 but does not define FIRST_CART_DT as a standalone variable.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>LOT_DISCON_GAP_DAYS</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Discontinuation gap threshold (days)</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>The minimum number of days between the last medication run-out date and the observation end date required for a discontinuation to be recognized. Default value: 90 days. If the gap between the last MAP_END_DT for induction medications and OBS_END_DT is less than this threshold, the patient is NOT considered discontinued (they are censored instead). This prevents classifying patients whose medications simply ran out near the end of follow-up as discontinued.</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 Rule 2: 'Discontinuation of the regimen occurs when all MM agents in the LOT are stopped.' 'If the regimen is discontinued and no new agent starts before a qualifying gap, the LOT end date is the run-out date immediately before that gap.' The protocol references a 'qualifying gap' but does not specify the exact number of days. Per Section 5.3: 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The run-out date is the MAP_END_DT (last day of medication availability). The gap threshold ensures there is sufficient time after medication ends to confirm the patient truly discontinued rather than being censored. The 90-day default is consistent with a treatment cycle of approximately 3 months. Configurable for sensitivity analysis per Protocol Section 5.3 which states 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Gap calculated as datediff(OBS_END_DT, RAW_DISCON_DT) where OBS_END_DT is derived from T_MEMBER_CONT_ENROLLMENT (ELIGEND), T_DOD (YMDOD), and study_end config. RAW_DISCON_DT is max(MAP_END_DT) from T_MEDICAL/T_RX for induction medications.</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>lot_program.R line 73: lot_discon_gap_days = as.integer(Sys.getenv('LOT_DISCON_GAP_DAYS', unset = '90')). Applied at Step S10 line 3376: LOT1_BASE_DISCON_DT = RAW_DISCON_DT only WHEN datediff(OBS_END_DT, RAW_DISCON_DT) &gt;= cfg$lot_discon_gap_days. Otherwise NULL (patient is censored, not discontinued). Configurable via LOT_DISCON_GAP_DAYS env var.</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not defined as a parameter; implicitly used but not documented). Protocol: - (defines discontinuation concept but does not specify exact gap threshold). Code: Y - implements as configurable parameter defaulting to 90 days at line 73, applied at line 3376.</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K25" s="7" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Parameter missing from original spec. The code uses lot_discon_gap_days=90 (lot_program.R line 73) to determine whether a patient is truly discontinued vs censored. This critical threshold affects whether LOT1_BASE_DISCON_DT is set or left NULL. The spec should document this parameter as it directly affects the LOT1_END_REASON classification.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>MEDICAL_DAY_SUPPLY</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Assumed days supply for medical claims</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>When days supply is missing from medical claims (infused/injected medications), a default of 28 days is assumed. This affects MAP_END_DT calculation which directly impacts LOT1_BASE_DISCON_DT and therefore LOT1_BASE_END_DT. For pharmacy claims with missing or anomalous days supply values, 28 days is also assumed.</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 Rule 2: 'The days supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days supply, or when days supply values are anomalous, a 28-day supply is assumed.'</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 2 - run-out date): 'The days' supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days' supply, or when days' supply values are anomalous, a 28-day supply is assumed.' (Section 5.1.1, under Rule 2). This is a fundamental parameter for the MAP algorithm that feeds into the LOT1 end date calculation. The 28-day assumption represents approximately one treatment cycle.</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Applied to T_MEDICAL claims where DAYS_SUPPLY is NULL. For T_RX pharmacy claims, DAYS_SUPPLY is typically populated but when missing/anomalous, 28 days is substituted. The assumed supply extends MAP_END_DT = FST_DT (or FILL_DT) + days_supply - 1.</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>lot_program.R line 74: medical_day_supply = as.integer(Sys.getenv('MEDICAL_DAY_SUPPLY', unset = '28')). Used in MAP construction (Step S05/S06 area) to set MAP_END_DT for medical claims. Configurable via MEDICAL_DAY_SUPPLY env var. This feeds into LOT1_BASE_DISCON_DT via max(MAP_END_DT).</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not documented in LOT1_BASE_END tab). Protocol: - (defined in Section 5.1.1 under MAP algorithm). Code: Y - implemented as configurable parameter defaulting to 28 days at line 74.</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K26" s="7" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses medical_day_supply=28 (lot_program.R line 74) for MAP_END_DT calculation on medical claims. While this is defined in the MAP section (5B), it directly affects LOT1_BASE_DISCON_DT and should be cross-referenced here. Protocol Section 5.1.1 explicitly states the 28-day assumption.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>LOT1_BASE_LENGTH</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>LOT1 base period duration in days</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>The number of days in the LOT1 base period, computed as datediff(LOT1_BASE_END_DT, LOT1_START_DT) + 1. Uses the priority-based end date: if MED_ADD occurs before DISCON, length is to MED_ADD date; if DISCON is first, length is to DISCON date; otherwise length is to OBS_END_DT (censored).</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>The protocol does not define LOT1_BASE_LENGTH as a named variable. Duration is implied by Protocol Section 5.1.1 which defines LOT start date ('LOT1 begins on the date of the first fill for an MM therapy following a patient's index date') and LOT end date (earliest of Rules 1-8).</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (LOT start/end): LOT duration is the span from LOT start (first non-steroid MAP) to LOT end. The +1 ensures inclusive day counting (both start and end dates are counted). Duration is relevant for assessing treatment patterns and time-to-event analyses.</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Duration computed from dates already derived from T_MEDICAL/T_RX (LOT1_START_DT from first MAP_START_DT) and LOT1_BASE_END_DT (priority-based end date).</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S10 lines 3447-3455: LOT1_BASE_LENGTH = CASE WHEN MED_ADD &lt;= DISCON THEN datediff(LOT1_BASE_1ST_ADD_MED_DT, LOT1_START_DT) + 1; WHEN DISCON THEN datediff(LOT1_BASE_DISCON_DT, LOT1_START_DT) + 1; ELSE datediff(OBS_END_DT, LOT1_START_DT) + 1 END. QC at line 3466: avg(LOT1_BASE_LENGTH) computed in validation query.</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not defined in LOT1_BASE_END tab). Protocol: - (duration concept implied). Code: Y - computed at Step S10 lines 3447-3455 with priority MED_ADD &gt; DISCON &gt; CENSORED.</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab. The code computes LOT1_BASE_LENGTH at lot_program.R Step S10 (lines 3447-3455) using a priority-based CASE matching the same hierarchy as LOT1_BASE_END_DT. Note: this is computed in the LOT1_BASE step (S10) rather than LOT1_BASE_END (S16), but it represents the base period duration which should be documented here.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>LOT1_SCT_TO_MAINT_180D_RULE</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>SCT not followed by maintenance within 180 days - LOT end rule</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>Protocol rule: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT. This rule determines whether LOT1 extends beyond the SCT to include a maintenance period or ends at the SCT itself. This is distinct from the 60-day conditioning period window (LOT1_EXTEND_FLG) which determines whether an SCT is included in LOT1 at all.</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Per Section 5.1: 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT). The expectation after an SCT is for a maintenance period and thus instead of the usual 120 days, we check for a valid 30-day (minimum) maintenance period.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 4 - SCTs not followed by maintenance): Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Also Section 5.1 (Maintenance regimen, situation 2): 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT).' This rule interacts with the maintenance logic: if maintenance starts within 180 days of SCT, LOT1 is extended to include the maintenance period. If no maintenance within 180 days, LOT1 ends at the SCT date. The 180-day window is consistent with the tandem SCT definition (cfg$sct_tandem_days=180).</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Would require checking T_MEDICAL/T_RX claims for maintenance medications (MONOMAINTENANCE=1 or valid DUALMAINTENANCEWITH in CL_MMA_ROLLUP) within 180 days after the SCT date (LOT1_1ST_SCT_DT or LOT1_TX_AUTO_MAX_DT).</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>lot_program.R: NOT APPLICABLE - MAINTENANCE IS NOT ENABLED. This rule depends on maintenance integration which is intentionally out of scope (line 4037-4038). The code currently ends LOT1 at LOT1_TX_ENDDATE (day before LOT-ending SCT) when SCT has priority. This 180-day rule will only become relevant if/when maintenance is brought into scope.</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>--N</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not defined). Protocol: - (defined in Section 5.1.1). Code: N - not applicable because maintenance is not enabled. This protocol rule will only be relevant when maintenance is brought into scope.</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K28" s="7" t="inlineStr">
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.1 states that if SCT is not followed by maintenance within 180 days, the LOT ends at the SCT date. NOT APPLICABLE in current implementation because maintenance is not enabled. This rule should be implemented if/when maintenance is brought into scope.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>PERMISSIBLE_SUBS_EFFECT</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Permissible substitution rules affecting LOT1 end</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Certain medication switches do NOT advance the LOT (i.e., do not set LOT1_BASE_1ST_ADD_MED_DT). Per the updated protocol (Rule 1): 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT.' Specific substitutions in code: (1) rituximab &lt;-&gt; rituximab/hyaluronidase, (2) daratumumab &lt;-&gt; daratumumab/hyaluronidase, (3) reference product &lt;-&gt; biosimilar, (4) bortezomib induction -&gt; ixazomib maintenance. The code implements this via the permissible_subs table which is joined into base_meds, effectively treating substitutions as part of the original regimen.</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.'</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 1 - Permissible substitutions): Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.' This directly affects LOT1_BASE_1ST_ADD_MED_DT: if the 'new' medication is a permissible substitute, it should not be counted as an addition. The permissible_subs table codifies these rules.</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Substitutions tracked via CL_MMA_ROLLUP (Tab 40) which maps medication abbreviations. The permissible_subs reference table pairs original_med with substitute_med. When a new medication claim appears in T_MEDICAL/T_RX, it is checked against permissible_subs before being classified as a new medication addition.</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S02 lines 2796-2803: permissible_subs view created from embedded or external table. Step S10 lines 3346-3354: base_meds CTE includes UNION with permissible_subs (im.MED_ABBR joined to ps.original_med -&gt; ps.substitute_med added to base_meds). This means first_add_candidates (lines 3413-3425) will NOT flag permissible substitutes as new medications because they are already in base_meds. Embedded permissible_subs defined at line 273.</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Spec: - (permissible substitutions not documented in LOT1_BASE_END tab). Protocol: - (defined in Section 5.1.1). Code: Y - implemented via permissible_subs table joined into base_meds CTE at Step S10 lines 3346-3354.</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="inlineStr">
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>Concept missing from original spec's LOT1_BASE_END tab. The code implements permissible substitutions by expanding base_meds to include substitutes (lot_program.R Step S10 lines 3346-3354). This is critical for correct LOT1_BASE_1ST_ADD_MED_DT calculation: without it, a permissible substitute (e.g., daratumumab/hyaluronidase replacing daratumumab) would incorrectly trigger a MED_ADD end reason. Protocol Section 5.1.1 explicitly defines which substitutions are permissible.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>STEROID_HANDLING</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Steroid inclusion/exclusion in LOT1 base end logic</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Steroids (corticosteroids) are included in the LOT1 induction medication list (LOT1_BASE_MEDS) but per the updated protocol 'all rules described below are based on oncology therapies only (e.g., not corticosteroids)' (Section 5.1). LOT1_START_DT uses first non-steroid MAP. The code includes steroids in the base_meds CTE used for LOT1_BASE_DISCON_DT calculation, meaning steroid MAPs can extend the discontinuation date. This may conflict with the protocol's intent to exclude steroids from LOT rules. This is a deliberate design decision documented in the code with a note that stakeholders may prefer to exclude steroids from the discontinuation computation.</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Per Section 4.2 (Inclusion Criterion 5): 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of receiving an approved MM oncology therapy.' Per Section 5.1.1 (CAR-T): 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Section 5.1 explicitly states: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Also: 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of active MM treatment.' The protocol excludes steroids from LOT rules, but the code includes steroids in the discontinuation calculation - this is a deliberate design decision documented with a code comment for stakeholder review.</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Steroid medications identified via MED_CLASS='STEROID' in CL_MMA_ROLLUP (Tab 40). Steroid claims from T_MEDICAL (PROC_CD/NDC) and T_RX (NDC). Steroid MAPs included in MAP construction and extend MAP_END_DT contributing to LOT1_BASE_DISCON_DT.</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S08 line 3321: LOT1_START_DT = min(MAP_START_DT) WHERE MAP_MED_CLASS &lt;&gt; 'STEROID' (steroids excluded from start date). Step S10 lines 3355-3359: Code comment - 'DECISION: Steroid MAPs are included in base_meds... If stakeholders prefer to exclude steroids from the discontinuation computation, filter base_meds above to exclude steroid MED_CLASS.' Currently steroids ARE included in discon calculation.</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not documented). Protocol: - (Section 5.1 states 'All rules described below are based on oncology therapies only (e.g., not corticosteroids)' - suggests steroids should be excluded from LOT rules including discontinuation). Code: Y - steroids included in discontinuation with explicit code comment noting this is a design decision (lines 3355-3359) that stakeholders may want to change. POTENTIAL MISALIGNMENT: code includes steroids in discontinuation but protocol excludes them from LOT rules.</t>
         </is>
       </c>
-      <c r="J30" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K30" s="7" t="inlineStr">
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>Design decision missing from original spec. The code includes steroids in the LOT1_BASE_DISCON_DT calculation (lot_program.R Step S10 lines 3355-3359) but documents this as a deliberate choice with a note for stakeholder review. The spec should document whether steroids should extend the discontinuation date, as this directly affects LOT1_BASE_END_DT for patients whose last active medication is a steroid.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>LOT1_TX_ENDDATE_REASON</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>SCT end reason type (AUTO/ALLO/CART)</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Numeric code identifying which SCT type caused the LOT-ending event. Values: 1=AUTO (autologous HSCT), 2=ALLO (allogeneic HSCT), 3=CART (CAR-T cellular therapy). Determined by comparing the earliest LOT-ending date among ENDING_AUTO_DT, FIRST_ALLO_DT, and FIRST_CART_DT. This value is mapped to string end reasons (SCT_AUTO, SCT_ALLO, SCT_CART) in LOT1_BASE_END_REASON.</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1: SCT type determines how LOT1 ends. Autologous SCT: 'Presence of an unplanned SCT will end the current LOT the day before the unplanned SCT.' Allogeneic SCT: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Per Section 5.1.1 (LOT Classification): 'CAR-T cellular therapy infusions are classified as their own LOT.'</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 3 - Unplanned SCTs) and Section 5.1 (SCT types): SCT type determines how LOT1 ends. Autologous SCT: single AUTO is allowed within LOT; excess AUTO (2nd for single, 3rd for tandem) ends LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT. The reason type is essential for correctly classifying the end reason.</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>SCT type determined from T_MEDICAL procedure codes matched against CL_SCT_CODELIST (Tab 44) which classifies procedures as AUTO, ALLO, or CART. Priority is earliest LOT-ending date wins.</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S15 lines 3951-3962: LOT1_TX_ENDDATE_REASON = CASE WHEN ENDING_AUTO_DT &lt;= FIRST_ALLO_DT AND ENDING_AUTO_DT &lt;= FIRST_CART_DT THEN 1; WHEN FIRST_ALLO_DT &lt;= FIRST_CART_DT THEN 2; ELSE 3 END. Used in Step S16 lines 4006-4010 to map: 1='SCT_AUTO', 2='SCT_ALLO', 3='SCT_CART'.</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present as standalone variable; only indirectly via end reason codes 5-7). Protocol: - (defines SCT types and their LOT-ending behavior). Code: Y - implemented at Step S15 lines 3951-3962 and consumed by Step S16 lines 4006-4010.</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr">
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec as standalone row. The code computes LOT1_TX_ENDDATE_REASON (lot_program.R lines 3951-3962) to bridge SCT type to end reason. The spec references SCT types indirectly via end reason codes 5=SCT_AUTO, 6=SCT_ALLO, 7=CART but does not define the intermediate reason variable.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>LOT1_TX_AUTO_DT_1 / LOT1_TX_AUTO_DT_2</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Dates of first and second valid autologous HSCT</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>LOT1_TX_AUTO_DT_1: date of the first valid autologous HSCT after 14-day claim windowing and 60-day gap validation. LOT1_TX_AUTO_DT_2: date of the second valid autologous HSCT (if exists). These dates are the foundation for tandem detection (DT_2 within 180 days of DT_1 with no ALLO between), single AUTO identification, and determining which AUTO event ends the LOT (2nd for single, 3rd for tandem).</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1: 'Planned Tandem SCT: Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart.' 'SCT is operationalized as &gt;1 procedure code for an SCT.' Per Section 5.1.1: 'Tandem SCTs are two SCTs &gt;60 to &lt;180 days apart. These are considered planned and a continuation of the line of therapy. Codes for SCTs are in the programming specification document.'</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1 (Planned Tandem SCT) and Section 5.1.1 (Events that will not end LOT): AUTO SCT dates are identified using a 14-day claim windowing algorithm (claims within 14 days grouped together, selecting the last date in the window). Events must be at least 60 days apart (cfg$sct_auto_gap_days=60). Tandem pair defined as DT_1 and DT_2 within 180 days with no ALLO between them. The spec references these dates extensively in the HSCT extension logic but does not define them as standalone rows.</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>AUTO HSCT dates derived from T_MEDICAL procedure codes (PROC_CD, BILL_PROC_CD) matched against CL_SCT_CODELIST where SCT_TYPE='AUTO'. FST_DT from T_MEDICAL is the raw claim date. 14-day windowing groups claims; 60-day gap validation separates distinct events.</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S13 lines 3620-3793: 14-day windowing algorithm with cfg$sct_auto_window_days=13, cfg$sct_auto_gap_days=60, cfg$sct_tandem_days=180. Step S15 lines 3901-3902: LOT1_TX_AUTO_DT_1 = ap.AUTO_DT_1, LOT1_TX_AUTO_DT_2 = ap.AUTO_DT_2 from auto_pivot CTE. Carried into lot1_base_end at Step S16 lines 3992-3993.</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Spec: - (referenced in HSCT extension logic but not as standalone rows). Protocol: - (defines AUTO SCT date identification). Code: Y - implemented at Step S13/S15 and output in lot1_base_end view.</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K32" s="7" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>Variables missing from original spec as standalone rows. The spec's HSCT extension logic (LOT1_EXTEND_FLG, updated LOT1_END_DT_TEMP) references LOT1_TX_AUTO_DT_1 and _DT_2 extensively but never defines them as their own variables. The code computes them at lot_program.R Step S15 lines 3901-3902 via the 14-day windowing algorithm at Step S13.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>LOT1_BASE_DISCON_DT</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>LOT1 base period discontinuation date</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>The date when all induction medications (including permissible substitutions) are considered discontinued. Computed as max(MAP_END_DT) for all base medication MAPs, but only set when the gap between this date and OBS_END_DT is &gt;= lot_discon_gap_days (default 90 days). If the gap is insufficient, set to NULL (patient is censored, not discontinued). This is one of the candidate dates for LOT1_BASE_END_DT.</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 Rule 2: 'Discontinuation of the regimen occurs when all MM agents in the LOT are stopped, either: without initiation of a new MM agent (all agents have reached their run-out dates and no further MM administrations/dispenses are observed), or with initiation of a new MM agent that was not present in the induction regimen.' 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.'</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT. Run-out date is the last date that a medication for a specific prescription is considered to be available.' The gap threshold ensures true discontinuation vs censoring near end of follow-up.</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>max(MAP_END_DT) derived from T_MEDICAL (FST_DT + medical_day_supply - 1) and T_RX (FILL_DT + DAYS_SUP - 1) for induction medications matched via CL_MMA_CODELIST. Gap validated against OBS_END_DT from T_MEMBER_CONT_ENROLLMENT/T_DOD.</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S10 lines 3360-3382: discon_raw CTE computes RAW_DISCON_DT = max(MAP_END_DT) for base meds. discon CTE applies gap check: LOT1_BASE_DISCON_DT = RAW_DISCON_DT only WHEN datediff(OBS_END_DT, RAW_DISCON_DT) &gt;= cfg$lot_discon_gap_days (default 90). Otherwise NULL.</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Spec: - (referenced in min() formula and end reason logic but not defined as standalone row in LOT1_BASE_END tab). Protocol: - (defines discontinuation concept). Code: Y - computed at Step S10 lines 3360-3382.</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K33" s="7" t="inlineStr">
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab as a standalone row. The spec references LOT1_BASE_DISCON_DT in the min() formula for LOT1_END_DT_TEMP and in the end reason logic, but never defines it. It is a key input variable computed at lot_program.R Step S10 lines 3360-3382.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>LOT1_BASE_1ST_ADD_MED_DT / LOT1_BASE_1ST_ADD_MED</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Date and name of first non-induction medication added</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>LOT1_BASE_1ST_ADD_MED_DT: the day before the first MAP_START_DT of a medication NOT in the induction regimen (and not a permissible substitution). This represents when LOT1 ends due to medication addition (MED_ADD end reason). LOT1_BASE_1ST_ADD_MED: the abbreviation of that first added medication (alphabetically first if same-day ties). These are candidate dates/reasons for LOT1_BASE_END_DT/REASON.</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 Rule 2: 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Per Rule 1: permissible substitutions (biologic reference product with biosimilars) 'do not advance the LOT.'</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation with new agent): Rule 2: 'With initiation of a new MM agent that was not present in the induction regimen (i.e., the regimen is interrupted by a new agent).' 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Rule 1 (permissible substitutions) does NOT trigger a new LOT. The LOT end date is set to the day BEFORE the new medication starts (date_sub(ADD_START_DT, 1)). Per protocol, permissible substitutions (rituximab/hyaluronidase swap, biosimilars, bortezomib-&gt;ixazomib for maintenance) do NOT trigger a new LOT.</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>First non-induction medication identified from T_MEDICAL (PROC_CD, BILL_PROC_CD, NDC) and T_RX (NDC) matched against CL_MMA_CODELIST (Tab 41) where the medication is NOT in base_meds (induction + permissible subs). MAP_START_DT from MAP algorithm.</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>lot_program.R Step S10 lines 3413-3441: first_add_candidates CTE selects non-induction MAPs where bm.MED_ABBR IS NULL (not in base_meds). first_add_dt gets min(MAP_START_DT). first_add_pick computes LOT1_BASE_1ST_ADD_MED_DT = date_sub(ADD_START_DT, 1) and LOT1_BASE_1ST_ADD_MED = min(MAP_MED_TYPE) for determinism (line 3435-3436 comment: 'Spec says random for same-day ties; we use min() for determinism').</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>Spec: - (referenced in min() and end reason logic but not standalone rows in LOT1_BASE_END tab). Protocol: - (defines new medication addition as LOT-ending event). Code: Y - computed at Step S10 lines 3413-3441. Code note: spec says 'random' for same-day ties but code uses min() (deliberate deviation at line 3435).</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K34" s="7" t="inlineStr">
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
         <is>
           <t>Variables missing from original spec's LOT1_BASE_END tab as standalone rows. The spec references LOT1_BASE_1ST_ADD_MED_DT in the min() formula and end reason logic but never defines it. Code deviation: spec says 'random' selection for same-day medication ties; code uses min() for determinism (lot_program.R line 3435). Also: LOT1_BASE_1ST_ADD_MED_DT = date_sub(ADD_START_DT, 1), meaning the end date is the day BEFORE the new med starts.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>INDUCTION_WINDOW_DAYS</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Induction regimen identification window (days)</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>The number of days from LOT1_START_DT within which all medications are considered part of the induction regimen. Default: 60 days. Any medication with MAP_START_DT within [LOT1_START_DT, LOT1_START_DT + 59] is included in LOT1_BASE_MEDS. Medications starting after this window that are not in the base regimen (or permissible substitutions) trigger LOT1_BASE_1ST_ADD_MED_DT and potentially a MED_ADD end reason.</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1: 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' 'For LOT2-LOT5, the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.'</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (LOT regimen): 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' For LOT2-5: 'the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' The 60-day window is the primary parameter; 30-day is noted as an alternative from literature. This parameter directly determines what is in the base regimen and therefore what constitutes a 'new' medication triggering MED_ADD. Configurable for sensitivity analysis per Protocol Section 5.3.</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Applied to MAP_START_DT from T_MEDICAL/T_RX claims. Medications with MAP_START_DT within the window are classified as induction via CL_MMA_CODELIST/CL_MMA_ROLLUP matching.</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>lot_program.R line 71: induction_window_days = as.integer(Sys.getenv('INDUCTION_WINDOW_DAYS', unset = '60')). Step S09 line 3338: WHERE ms.MAP_START_DT &lt;= date_add(l1.LOT1_START_DT, {cfg$induction_window_days - 1}). Configurable via INDUCTION_WINDOW_DAYS env var.</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not documented as a parameter in LOT1_BASE_END tab). Protocol: - (defines 60-day window). Code: Y - implemented as configurable parameter at line 71, used at line 3338.</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K35" s="7" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses induction_window_days=60 (lot_program.R line 71) to determine which medications are in the induction regimen. This is critical: it directly controls what triggers MED_ADD end reason. Protocol Section 5.1.1 specifies 60 days (with 30-day alternative from Madduri 2021).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>ALLO_ALWAYS_ENDS_LOT</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Allogeneic SCT always ends current LOT (protocol rule)</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>Protocol rule: Any allogeneic HSCT immediately ends the current line of therapy. The LOT end date is set to the day before the ALLO SCT date. An auto-to-allo sequence is NOT considered a planned tandem and indicates treatment failure. This is a hard rule with no exceptions - ALLO SCT has the same LOT-ending priority as any other SCT in the code's CASE statement.</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1: 'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Per Section 5.1: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Per Section 5.1.1 Rule 3: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Per Section 5.1.1 (LOT Classification): 'Allogeneic SCT: Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.'</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): Section 5.1: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Section 5.1.1 (Rule 3): 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Also: 'Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.' Also: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Additionally, the presence of an ALLO between two AUTO SCTs invalidates the tandem classification (coalesce(n_allo_between, 0) = 0 required for tandem).</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>ALLO SCT identified from T_MEDICAL procedure codes matched against CL_SCT_CODELIST where SCT_TYPE='ALLO'. Date from FST_DT in T_MEDICAL.</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>lot_program.R: ALLO always ends LOT implemented via: (1) FIRST_ALLO_DT captured at Step S14 lines 3796-3825 and Step S15 line 3929. (2) LOT1_TX_ENDDATE includes ALLO at lines 3939-3949: least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT) - 1. (3) ALLO between AUTOs invalidates tandem at line 3907: coalesce(ab.n_allo_between, 0) = 0. (4) Step S16 line 4008: LOT1_TX_ENDDATE_REASON=2 maps to 'SCT_ALLO'.</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>--Y</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>Spec: - (implicit via SCT_ALLO end reason code 6 but not stated as an explicit rule). Protocol: - (explicit rule in Section 5.1.1). Code: Y - implemented via ALLO priority in LOT1_TX_ENDDATE and tandem invalidation.</t>
         </is>
       </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K36" s="7" t="inlineStr">
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
         <is>
           <t>Protocol rule not explicitly stated in original spec. The spec has SCT_ALLO as end reason code 6 but does not document the rule that ALLO always ends the LOT unconditionally, or that auto-to-allo is not considered planned. The code implements this at lot_program.R via FIRST_ALLO_DT inclusion in LOT1_TX_ENDDATE (lines 3939-3949) and tandem invalidation (line 3907).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>CART_30D_CONSOLIDATION</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>CAR-T 30-day supportive agent consolidation rule</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Protocol rule: Therapies (including supportive agents such as corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT, not the preceding LOT. This means medications administered near a CAR-T event should be attributed to the CAR-T LOT rather than LOT1. This rule is NOT currently implemented in the code.</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1.1 (LOT Classification): 'CAR-T: CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1.1 (CAR-T): 'CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' (Section 5.1.1) This 30-day window affects medication attribution near the LOT1/CAR-T boundary. Without this rule, medications given in the 30 days before CAR-T could incorrectly extend LOT1's discontinuation date or trigger a MED_ADD end reason.</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>Would require checking T_MEDICAL/T_RX claims within 30 days of FIRST_CART_DT and reclassifying them from LOT1 to the CAR-T LOT. Affects MAP_END_DT for induction meds and MAP_START_DT for potential new meds.</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>lot_program.R: NOT IMPLEMENTED. The code treats CAR-T as a simple LOT-ending event (Step S14 lines 3796-3825: CART dates extracted; Step S15 line 3930: FIRST_CART_DT captured). LOT1 ends the day before CART (LOT1_TX_ENDDATE = date_sub(FIRST_CART_DT, 1) at lines 3939-3949). No 30-day consolidation window is applied to reclassify medications near the CAR-T boundary.</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>--N</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (defined in Section 5.1.2). Code: N - not implemented; CAR-T simply ends LOT1 without 30-day medication reclassification.</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K37" s="7" t="inlineStr">
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.2 specifies that therapies within 30 days of CAR-T are consolidated as part of the CAR-T LOT. The code does not implement this 30-day consolidation window. Impact: medications given in the 30 days before CAR-T could incorrectly influence LOT1's DISCON_DT or trigger MED_ADD. This should be implemented for correct medication attribution near CAR-T events.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>MESNA_EXCLUSION</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>Mesna excluded from LOT definition</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>Protocol rule: Mesna is excluded from LOT definitions. Mesna is a supportive agent used to protect the bladder against toxic side-effects of certain anticancer drugs (e.g., cyclophosphamide conditioning). Mesna claims should NOT be counted as MM therapy and should NOT trigger MED_ADD end reason or contribute to MAP coverage calculations.</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Per Protocol Section 5.1: 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient's bladder against the toxic side-effects of certain anticancer drugs).'</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Protocol Section 5.1 (MM therapies): 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion beyond the general steroid handling. Mesna should be excluded from CL_MMA_CODELIST or filtered out during medication identification.</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>Mesna identified via NDC codes in T_RX or HCPCS codes in T_MEDICAL. Should be excluded from CL_MMA_CODELIST (Tab 41) or filtered during MMA claim extraction in Step S05 (mma_med).</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>lot_program.R: Mesna is not explicitly referenced in the code. It is likely excluded by not being present in the CL_MMA_CODELIST/CL_MMA_ROLLUP codelists (Tab 40/41). If mesna codes ARE in the codelist, they would incorrectly be treated as MM therapy. Verification would require checking the codelist contents.</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>--?</t>
         </is>
       </c>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>Spec: - (not present). Protocol: - (explicit exclusion in Section 5.1.1). Code: ? - likely excluded by omission from codelist but not explicitly filtered. Cannot confirm without checking codelist contents.</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K38" s="7" t="inlineStr">
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
         <is>
           <t>Protocol exclusion rule not in original spec. Protocol Section 5.1.1 explicitly excludes mesna from LOTs. The code likely handles this by not including mesna in CL_MMA_CODELIST/CL_MMA_ROLLUP, but this should be verified. If mesna codes were inadvertently included in the codelist, they would incorrectly affect LOT1 end date calculations.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>LOT1 Base End - Protocol Addition</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>NAMING_DISCREPANCY_SCT_VS_HSCT</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Variable naming: spec uses HSCT prefix vs code uses SCT prefix</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>The original spec names autologous transplant flags as LOT1_HSCT_AUTO_SING_FLG and LOT1_HSCT_AUTO_TAND_FLG (using 'HSCT' prefix). The code names them LOT1_SCT_AUTO_SING_FLG and LOT1_SCT_AUTO_TAND_FLG (using 'SCT' prefix). Both refer to the same variables. This naming inconsistency should be reconciled.</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>The protocol uses 'SCT' (Stem Cell Transplant) terminology consistently throughout. Per Protocol Section 5.1: 'Stem cell transplant (SCT).' The original program spec uses 'HSCT' (Hematopoietic Stem Cell Transplant) prefix for variable names. Both abbreviations refer to the same medical concept.</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Protocol uses 'SCT' (Stem Cell Transplant) terminology consistently. The spec uses 'HSCT' (Hematopoietic Stem Cell Transplant). Both are acceptable medical abbreviations for the same concept. The code aligns with the protocol's 'SCT' convention.</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>N/A - naming convention only.</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>lot_program.R: Uses SCT prefix consistently: LOT1_SCT_AUTO_SING_FLG (line 3917), LOT1_SCT_AUTO_TAND_FLG (line 3909). CL_SCT_CODELIST table name also uses SCT. Configuration parameters use sct_ prefix (sct_auto_window_days, sct_auto_gap_days, sct_tandem_days at lines 87-89).</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>N-Y</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>Spec: N - uses HSCT prefix (LOT1_HSCT_AUTO_*). Protocol: - (uses SCT terminology). Code: Y - uses SCT prefix (LOT1_SCT_AUTO_*) matching protocol convention.</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>CV 2026-04-02 (protocol revalidation)</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>CV 2026-04-02 (protocol revalidation)</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
         <is>
           <t>Naming discrepancy: spec uses LOT1_HSCT_AUTO_SING_FLG / LOT1_HSCT_AUTO_TAND_FLG while code uses LOT1_SCT_AUTO_SING_FLG / LOT1_SCT_AUTO_TAND_FLG. Recommend aligning spec to use SCT prefix to match both code and protocol convention.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clean Definition column: remove editorial prefixes, keep protocol text only
- Removed "Per Protocol Section X.X:" editorial prefixes from definitions
- Removed "MAINTENANCE IS NOT ENABLED" implementation notes from Definition
  column (belongs in other columns, not protocol text)
- Fixed regex artifacts (leftover section numbers)
- Kept "no protocol equivalent" notes for variables without protocol match
- Regenerated Excel with same changes

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The LOT will continue until the earliest of any of the following events (Protocol Section 5.1.1, Rules 1-8): (1) substitution of a biologic reference product with any of its biosimilars does not advance the LOT; (2) discontinuation of all agents in the regimen - the LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available; (3) unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, the LOT will end the day before the latter SCT; any allogeneic SCTs are considered a new LOT; (4) SCTs not followed by maintenance within 180 days - the last day of the LOT is the date of the SCT; (5) death; (6) health plan disenrollment; (7) end of the study period; (8) end of maintenance regimen.</t>
+          <t>The LOT will continue until the earliest of any of the following events: (1) substitution of a biologic reference product with any of its biosimilars does not advance the LOT; (2) discontinuation of all agents in the regimen - the LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available; (3) unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, the LOT will end the day before the latter SCT; any allogeneic SCTs are considered a new LOT; (4) SCTs not followed by maintenance within 180 days - the last day of the LOT is the date of the SCT; (5) death; (6) health plan disenrollment; (7) end of the study period; (8) end of maintenance regimen.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1, the LOT ends for one of these reasons: (Rule 2) Discontinuation of all agents in the regimen, with or without switch to a new agent; (Rule 2) If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent; (Rule 3) Unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, or any allogeneic SCT; (Rule 4) SCTs not followed by maintenance within 180 days; (Rule 5) Death; (Rule 6) Health plan disenrollment; (Rule 7) End of the study period; (Rule 8) End of maintenance regimen.</t>
+          <t>The LOT ends for one of these reasons: (Rule 2) Discontinuation of all agents in the regimen, with or without switch to a new agent; (Rule 2) If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent; (Rule 3) Unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, or any allogeneic SCT; (Rule 4) SCTs not followed by maintenance within 180 days; (Rule 5) Death; (Rule 6) Health plan disenrollment; (Rule 7) End of the study period; (Rule 8) End of maintenance regimen.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum's KOL and informed by Charalampous et al.'s findings that the median time from end of induction to transplant was 33 days (interquartile range=27-42).' Single autologous SCTs and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.'</t>
+          <t>'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum's KOL and informed by Charalampous et al.'s findings that the median time from end of induction to transplant was 33 days (interquartile range=27-42).' Single autologous SCTs and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.'</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>The protocol does not define a same-class switch flag. Per Protocol Section 5.1.1 Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.'</t>
+          <t>The protocol does not define a same-class switch flag. 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.'</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT. SCT is operationalized as &gt;1 procedure code for an SCT.' A single autologous SCT is one that is not part of a valid tandem pair. Per Section 5.1.1: 'Single autologous SCTs and tandem SCTs are not unplanned SCTs and are considered a continuation of the line of therapy.'</t>
+          <t>'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT. SCT is operationalized as &gt;1 procedure code for an SCT.' A single autologous SCT is one that is not part of a valid tandem pair. 'Single autologous SCTs and tandem SCTs are not unplanned SCTs and are considered a continuation of the line of therapy.'</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart; otherwise, they will be considered unplanned (Rajkumar, 2015). An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Per Section 5.1.1: 'Tandem SCTs are two SCTs &gt;60 to &lt;180 days apart. These are considered planned and a continuation of the line of therapy.'</t>
+          <t>'Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart; otherwise, they will be considered unplanned (Rajkumar, 2015). An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' 'Tandem SCTs are two SCTs &gt;60 to &lt;180 days apart. These are considered planned and a continuation of the line of therapy.'</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The protocol does not define this as a named variable. Per Protocol Section 5.1: tandem SCTs are two autologous SCTs &gt;60 to &lt;180 days apart. The latest valid AUTO date is the second SCT for tandem patients or the first SCT for single-AUTO patients. Per Section 5.1.1: 'Single autologous SCTs and tandem stem-cell transplants (SCT) &lt;180 days apart' are considered a continuation of the LOT.</t>
+          <t>The protocol does not define this as a named variable. tandem SCTs are two autologous SCTs &gt;60 to &lt;180 days apart. The latest valid AUTO date is the second SCT for tandem patients or the first SCT for single-AUTO patients. 'Single autologous SCTs and tandem stem-cell transplants (SCT) &lt;180 days apart' are considered a continuation of the LOT.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT.' This binary variable indicates whether the patient received any valid autologous transplant, regardless of single or tandem.</t>
+          <t>'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT.' This binary variable indicates whether the patient received any valid autologous transplant, regardless of single or tandem.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: 'Single autologous SCT or tandem stem-cell transplants (SCT) &lt;180 days apart: SCTs are usually preceded by induction therapy and followed by consolidation and maintenance therapy.' These are 'considered planned and a continuation of the line of therapy.' 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.'</t>
+          <t>'Single autologous SCT or tandem stem-cell transplants (SCT) &lt;180 days apart: SCTs are usually preceded by induction therapy and followed by consolidation and maintenance therapy.' These are 'considered planned and a continuation of the line of therapy.' 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.'</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date. For LOT1, the first therapy received is considered the induction therapy.' Per Section 5.1.1 Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT.' All rules are 'based on oncology therapies only (e.g., not corticosteroids).'</t>
+          <t>'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date. For LOT1, the first therapy received is considered the induction therapy.' Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT.' All rules are 'based on oncology therapies only (e.g., not corticosteroids).'</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'A maintenance regimen is a period of 120 days or longer during which only a valid maintenance therapy is available. Maintenance is not required to be prescribed continuously for the duration of the 120 day period. Furthermore, the maintenance therapy must have been a part of the LOT's initial regimen.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+          <t>'A maintenance regimen is a period of 120 days or longer during which only a valid maintenance therapy is available. Maintenance is not required to be prescribed continuously for the duration of the 120 day period. Furthermore, the maintenance therapy must have been a part of the LOT's initial regimen.'</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: valid maintenance therapies per NCCN Guidelines include lenalidomide monotherapy, bortezomib monotherapy, daratumumab monotherapy, ixazomib monotherapy, thalidomide monotherapy, bortezomib/lenalidomide dual, carfilzomib/lenalidomide dual, and daratumumab/lenalidomide dual. MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+          <t>valid maintenance therapies per NCCN Guidelines include lenalidomide monotherapy, bortezomib monotherapy, daratumumab monotherapy, ixazomib monotherapy, thalidomide monotherapy, bortezomib/lenalidomide dual, carfilzomib/lenalidomide dual, and daratumumab/lenalidomide dual.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Once a maintenance regimen has begun, it continues until discontinuation, presence of an SCT, right censoring (i.e. end of follow-up), or the addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+          <t>'Once a maintenance regimen has begun, it continues until discontinuation, presence of an SCT, right censoring (i.e. end of follow-up), or the addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.'</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: valid maintenance therapies per NCCN Guidelines (Kumar, 2020) include mono-maintenance (lenalidomide, bortezomib, daratumumab, ixazomib, thalidomide) and dual-maintenance (bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide). 'Any of the maintenance medications listed above will be considered maintenance medications for all patients, regardless of transplant status.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+          <t>valid maintenance therapies per NCCN Guidelines (Kumar, 2020) include mono-maintenance (lenalidomide, bortezomib, daratumumab, ixazomib, thalidomide) and dual-maintenance (bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide). 'Any of the maintenance medications listed above will be considered maintenance medications for all patients, regardless of transplant status.'</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 8: 'The LOT will end after a maintenance regimen ends due to: unplanned SCTs, death, health plan disenrollment, and end of study period.' Per Section 5.1: 'The addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+          <t>'The LOT will end after a maintenance regimen ends due to: unplanned SCTs, death, health plan disenrollment, and end of study period.' 'The addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.'</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: 'The LOT will continue until the earliest of any of the following' (Rules 1-8). The LOT end date is the final computed date after evaluating all end conditions. Per Rule 2: 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.' 'If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent.'</t>
+          <t>'The LOT will continue until the earliest of any of the following' (Rules 1-8). The LOT end date is the final computed date after evaluating all end conditions. Per Rule 2: 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.' 'If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent.'</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: LOT ends for one of the following reasons (Rules 1-8): (1) permissible substitution (does not end LOT); (2) discontinuation of all agents; (3) unplanned SCTs; (4) SCTs not followed by maintenance within 180 days; (5) death; (6) health plan disenrollment; (7) end of study period; (8) end of maintenance regimen.</t>
+          <t>LOT ends for one of the following reasons (Rules 1-8): (1) permissible substitution (does not end LOT); (2) discontinuation of all agents; (3) unplanned SCTs; (4) SCTs not followed by maintenance within 180 days; (5) death; (6) health plan disenrollment; (7) end of study period; (8) end of maintenance regimen.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum's KOL and informed by Charalampous et al.'s findings that the median time from end of induction to transplant was 33 days (interquartile range=27-42) (Charalampous, 2023).'</t>
+          <t>'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum's KOL and informed by Charalampous et al.'s findings that the median time from end of induction to transplant was 33 days (interquartile range=27-42) (Charalampous, 2023).'</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Per Section 5.1.1 Rule 3: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Per Section 5.1.1 (LOT Classification): 'Allogeneic SCT: Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.'</t>
+          <t>'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Rule 3: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' 'Allogeneic SCT: Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.'</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 (LOT Classification): 'CAR-T: CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+          <t>'CAR-T: CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 2: 'Discontinuation of the regimen occurs when all MM agents in the LOT are stopped.' 'If the regimen is discontinued and no new agent starts before a qualifying gap, the LOT end date is the run-out date immediately before that gap.' The protocol references a 'qualifying gap' but does not specify the exact number of days. Per Section 5.3: 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
+          <t>'Discontinuation of the regimen occurs when all MM agents in the LOT are stopped.' 'If the regimen is discontinued and no new agent starts before a qualifying gap, the LOT end date is the run-out date immediately before that gap.' The protocol references a 'qualifying gap' but does not specify the exact number of days. 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 2: 'The days supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days supply, or when days supply values are anomalous, a 28-day supply is assumed.'</t>
+          <t>'The days supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days supply, or when days supply values are anomalous, a 28-day supply is assumed.'</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Per Section 5.1: 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT). The expectation after an SCT is for a maintenance period and thus instead of the usual 120 days, we check for a valid 30-day (minimum) maintenance period.' MAINTENANCE IS NOT ENABLED in the current implementation.</t>
+          <t>'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT). The expectation after an SCT is for a maintenance period and thus instead of the usual 120 days, we check for a valid 30-day (minimum) maintenance period.'</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.'</t>
+          <t>'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.'</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Per Section 4.2 (Inclusion Criterion 5): 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of receiving an approved MM oncology therapy.' Per Section 5.1.1 (CAR-T): 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+          <t>'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of receiving an approved MM oncology therapy.' 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: SCT type determines how LOT1 ends. Autologous SCT: 'Presence of an unplanned SCT will end the current LOT the day before the unplanned SCT.' Allogeneic SCT: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Per Section 5.1.1 (LOT Classification): 'CAR-T cellular therapy infusions are classified as their own LOT.'</t>
+          <t>SCT type determines how LOT1 ends. Autologous SCT: 'Presence of an unplanned SCT will end the current LOT the day before the unplanned SCT.' Allogeneic SCT: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' 'CAR-T cellular therapy infusions are classified as their own LOT.'</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Planned Tandem SCT: Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart.' 'SCT is operationalized as &gt;1 procedure code for an SCT.' Per Section 5.1.1: 'Tandem SCTs are two SCTs &gt;60 to &lt;180 days apart. These are considered planned and a continuation of the line of therapy. Codes for SCTs are in the programming specification document.'</t>
+          <t>'Planned Tandem SCT: Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart.' 'SCT is operationalized as &gt;1 procedure code for an SCT.' 'Tandem SCTs are two SCTs &gt;60 to &lt;180 days apart. These are considered planned and a continuation of the line of therapy. Codes for SCTs are in the programming specification document.'</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 2: 'Discontinuation of the regimen occurs when all MM agents in the LOT are stopped, either: without initiation of a new MM agent (all agents have reached their run-out dates and no further MM administrations/dispenses are observed), or with initiation of a new MM agent that was not present in the induction regimen.' 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.'</t>
+          <t>'Discontinuation of the regimen occurs when all MM agents in the LOT are stopped, either: without initiation of a new MM agent (all agents have reached their run-out dates and no further MM administrations/dispenses are observed), or with initiation of a new MM agent that was not present in the induction regimen.' 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.'</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 Rule 2: 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Per Rule 1: permissible substitutions (biologic reference product with biosimilars) 'do not advance the LOT.'</t>
+          <t>'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Per Rule 1: permissible substitutions (biologic reference product with biosimilars) 'do not advance the LOT.'</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1: 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' 'For LOT2-LOT5, the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.'</t>
+          <t>'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' 'For LOT2-LOT5, the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.'</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Per Section 5.1: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Per Section 5.1.1 Rule 3: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Per Section 5.1.1 (LOT Classification): 'Allogeneic SCT: Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.'</t>
+          <t>'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Rule 3: 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' 'Allogeneic SCT: Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.'</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1.1 (LOT Classification): 'CAR-T: CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+          <t>'CAR-T: CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Per Protocol Section 5.1: 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient's bladder against the toxic side-effects of certain anticancer drugs).'</t>
+          <t>'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient's bladder against the toxic side-effects of certain anticancer drugs).'</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>The protocol uses 'SCT' (Stem Cell Transplant) terminology consistently throughout. Per Protocol Section 5.1: 'Stem cell transplant (SCT).' The original program spec uses 'HSCT' (Hematopoietic Stem Cell Transplant) prefix for variable names. Both abbreviations refer to the same medical concept.</t>
+          <t>The protocol uses 'SCT' (Stem Cell Transplant) terminology consistently throughout. 'Stem cell transplant (SCT).' The original program spec uses 'HSCT' (Hematopoietic Stem Cell Transplant) prefix for variable names. Both abbreviations refer to the same medical concept.</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fix incorrect attribution of priority order to protocol
The protocol says 'earliest of any of the following' (Rules 1-8) but
does NOT specify a tie-breaking priority order. The priority
SCT > MED_ADD > DISCONTINUATION > CENSORED is a code implementation
decision (lot_program.R Step S16 lines 4001-4017), not a protocol
requirement. Fixed Additional Notes and Sync Status Notes columns
to correctly attribute this to the code.

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications (gap &gt;= 90 days from OBS_END_DT), addition of a new non-induction medication, a LOT-ending SCT event, or end of observation (censoring at death/disenrollment/study end). The priority order is SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED. The MAP algorithm (Section 5.1.1, Rule 2) defines run-out dates using 28-day assumed supply for medical claims. Priority order: SCT (Rule 3) &gt; MED_ADD (Rule 2) &gt; DISCONTINUATION (Rule 2) &gt; CENSORED (Rules 5-7).</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications (gap &gt;= 90 days from OBS_END_DT), addition of a new non-induction medication, a LOT-ending SCT event, or end of observation (censoring at death/disenrollment/study end). The MAP algorithm (Section 5.1.1, Rule 2) defines run-out dates using 28-day assumed supply for medical claims. The code implements a tie-breaking priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) which is not specified in the protocol.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - uses simple min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP which is not yet defined; also garbled label text ('The end date for the 1date'). Protocol: Y - defines LOT1 end as earliest qualifying event with clear priority. Code: Y - implements priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCON &gt; CENSORED) which correctly reflects protocol priority; maintenance not yet integrated but logged as pending (line 4037).</t>
+          <t>Spec: N - uses simple min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP which is not yet defined; also garbled label text ('The end date for the 1date'). Protocol: Y - defines LOT1 end as earliest qualifying event (Rules 1-8). Note: the protocol does not specify a tie-breaking priority order; the SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED priority is a code implementation decision. Code: Y - implements priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCON &gt; CENSORED) which correctly reflects protocol priority; maintenance not yet integrated but logged as pending (line 4037).</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (1) Discontinuation - all induction medications' MAP coverage ends with a sufficient gap (&gt;= 90 days per cfg$lot_discon_gap_days) before observation end; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events - autologous SCT &gt;180 days after previous, allogeneic always ends LOT, CAR-T starts new LOT. Protocol explicitly numbers LOT end events as Rules 1-8. Priority in code: SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (1) Discontinuation - all induction medications' MAP coverage ends with a sufficient gap (&gt;= 90 days per cfg$lot_discon_gap_days) before observation end; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events - autologous SCT &gt;180 days after previous, allogeneic always ends LOT, CAR-T starts new LOT. Protocol explicitly numbers LOT end events as Rules 1-8. The code applies a tie-breaking priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) not specified in the protocol.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - uses numeric codes 1-7 with date-matching logic and includes DEATH (4) as a separate end reason distinct from CENSOR. Protocol: Y - defines end reasons consistent with code priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED). Code: Y - uses string end reasons ('SCT_AUTO', 'SCT_ALLO', 'SCT_CART', 'MED_ADD', 'DISCONTINUATION', 'CENSORED') with priority-based CASE; death is subsumed into CENSORED via OBS_END_DT.</t>
+          <t>Spec: N - uses numeric codes 1-7 with date-matching logic and includes DEATH (4) as a separate end reason distinct from CENSOR. Protocol: Y - defines end reasons (Rules 1-8). Note: protocol does not specify priority/tie-breaking order; the code's SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED priority is an implementation decision. Code: Y - uses string end reasons ('SCT_AUTO', 'SCT_ALLO', 'SCT_CART', 'MED_ADD', 'DISCONTINUATION', 'CENSORED') with priority-based CASE; death is subsumed into CENSORED via OBS_END_DT.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Protocol states 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.' (Section 5.1.1). Single and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.' The code handles this by giving SCT events top priority in the end reason determination rather than using a separate extension flag.</t>
+          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Protocol states 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.' (Section 5.1.1). Single and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.' The code handles this differently: SCT events take top priority in the code's CASE statement (a code design decision, not a protocol-specified priority) rather than using a separate extension flag.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): The maintenance period ends when the patient discontinues maintenance therapy, adds a new medication (signaling a new LOT), receives an SCT, dies, or reaches end of observation. The end of maintenance also considers the same priority hierarchy as the base period end.</t>
+          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): The maintenance period ends when the patient discontinues maintenance therapy, adds a new medication (signaling a new LOT), receives an SCT, dies, or reaches end of observation. The end of maintenance follows similar logic to the base period end.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (highest priority - allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. The original spec only defines TEMP and SWITCH versions with numeric codes but never creates the final string-valued LOT1_BASE_END_REASON.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. The original spec only defines TEMP and SWITCH versions with numeric codes but never creates the final string-valued LOT1_BASE_END_REASON.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Clarify priority as earliest-date-wins with same-date tiebreaker only
The CASE statement at Step S16 selects the earliest date using <=
comparisons. The evaluation order (SCT > MED_ADD > DISCONTINUATION >
CENSORED) only acts as a tiebreaker when two events share the same
date. Updated R Code Implementation, Sync Status Notes, and Additional
Notes columns across all affected rows to clearly state this. Also
fixed column alignment (restored empty QC Reviewed column).

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications (gap &gt;= 90 days from OBS_END_DT), addition of a new non-induction medication, a LOT-ending SCT event, or end of observation (censoring at death/disenrollment/study end). The MAP algorithm (Section 5.1.1, Rule 2) defines run-out dates using 28-day assumed supply for medical claims. The code implements a tie-breaking priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) which is not specified in the protocol.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications, addition of a new non-induction medication, a LOT-ending SCT event, death, health plan disenrollment, or end of study period. The code implements this as 'earliest date wins' using &lt;= comparisons in a CASE statement. The CASE evaluation order (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) serves only as a same-date tiebreaker and is not specified in the protocol.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>lot_program.R Step S16 lines 4018-4028: CASE statement computes LOT1_BASE_END_DT with priority SCT &gt; MED_ADD &gt; DISCON &gt; CENSORED. LOT1_BASE_DISCON_DT computed at Step S10 lines 3360-3382 (max MAP_END_DT with gap &gt;= lot_discon_gap_days). LOT1_BASE_1ST_ADD_MED_DT at lines 3413-3441 (date_sub(first non-induction MAP_START_DT, 1)). LOT1_TX_ENDDATE at lines 3939-3949 (date_sub(least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT), 1)). OBS_END_DT from new_code.R Step 23 lines ~2418-2421.</t>
+          <t>lot_program.R Step S16 lines 4018-4028: CASE statement computes LOT1_BASE_END_DT by selecting the earliest date among LOT1_TX_ENDDATE (SCT), LOT1_BASE_1ST_ADD_MED_DT (new med), LOT1_BASE_DISCON_DT (discontinuation), and OBS_END_DT (censored). Uses &lt;= comparisons, so the earliest date always wins. Only on same-date ties does the CASE order act as a tiebreaker: SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED. LOT1_BASE_DISCON_DT computed at Step S10 lines 3360-3382 (max MAP_END_DT with gap &gt;= lot_discon_gap_days). LOT1_BASE_1ST_ADD_MED_DT at lines 3413-3441 (date_sub(first non-induction MAP_START_DT, 1)). LOT1_TX_ENDDATE at lines 3939-3949 (date_sub(least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT), 1)). OBS_END_DT from new_code.R Step 23.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - uses simple min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP which is not yet defined; also garbled label text ('The end date for the 1date'). Protocol: Y - defines LOT1 end as earliest qualifying event (Rules 1-8). Note: the protocol does not specify a tie-breaking priority order; the SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED priority is a code implementation decision. Code: Y - implements priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCON &gt; CENSORED) which correctly reflects protocol priority; maintenance not yet integrated but logged as pending (line 4037).</t>
+          <t>Spec: N - uses simple min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP which is not yet defined; also garbled label text ('The end date for the 1date'). Protocol: Y - defines LOT1 end as earliest qualifying event (Rules 1-8). Code: Y - selects the earliest date, matching the protocol's 'earliest of' logic. The CASE statement order (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) only acts as a tiebreaker when two events share the same date; this tie-breaking order is not specified in the protocol but is a reasonable code implementation decision. Maintenance not yet integrated (line 4037).</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -609,7 +609,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Original spec uses min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP, but the code uses a priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) rather than a simple minimum. The spec's label is garbled ('The end date for the 1date' should read 'The end date for the base period'). The inclusion of LOT1_BASE_MAINT_END_DT_TEMP in the min() is not applicable as maintenance is not enabled and is intentionally out of scope (confirmed by code comment at lot_program.R line 4037-4038).</t>
         </is>
@@ -666,7 +667,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_END_DT_ORIG as '= LOT1_END_DT_TEMP' (a copy). The code does not implement this intermediate variable. Instead, the code computes LOT1_BASE_END_DT directly using a priority-based CASE statement at lot_program.R lines 4018-4028. The multi-step approach in the spec (calculate TEMP, save ORIG, then extend) is an implementation design choice that the code handles differently.</t>
         </is>
@@ -695,7 +697,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (1) Discontinuation - all induction medications' MAP coverage ends with a sufficient gap (&gt;= 90 days per cfg$lot_discon_gap_days) before observation end; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events - autologous SCT &gt;180 days after previous, allogeneic always ends LOT, CAR-T starts new LOT. Protocol explicitly numbers LOT end events as Rules 1-8. The code applies a tie-breaking priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) not specified in the protocol.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (Rule 2) Discontinuation - all induction medications discontinued; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events. Protocol explicitly numbers LOT end events as Rules 1-8. The code selects the earliest date; the CASE evaluation order (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) is a same-date tiebreaker not in the protocol.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -705,7 +707,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>lot_program.R Step S16 lines 4001-4017: LOT1_BASE_END_REASON computed as CASE statement. Priority: (1) SCT - when LOT1_TX_ENDDATE IS NOT NULL and &lt;= both LOT1_BASE_1ST_ADD_MED_DT and LOT1_BASE_DISCON_DT, maps TX_ENDDATE_REASON 1='SCT_AUTO', 2='SCT_ALLO', 3='SCT_CART'. (2) MED_ADD - when LOT1_BASE_1ST_ADD_MED_DT IS NOT NULL and &lt;= LOT1_BASE_DISCON_DT. (3) DISCONTINUATION - when LOT1_BASE_DISCON_DT IS NOT NULL. (4) CENSORED - default. Note: DEATH is not a separate end reason in code; death is captured via OBS_END_DT which sets CENSORED.</t>
+          <t>lot_program.R Step S16 lines 4001-4017: LOT1_BASE_END_REASON computed as CASE statement using &lt;= comparisons to select the earliest event. The CASE evaluation order acts as a same-date tiebreaker only: (1) SCT - when LOT1_TX_ENDDATE IS NOT NULL and &lt;= both LOT1_BASE_1ST_ADD_MED_DT and LOT1_BASE_DISCON_DT, maps TX_ENDDATE_REASON 1='SCT_AUTO', 2='SCT_ALLO', 3='SCT_CART'. (2) MED_ADD - when LOT1_BASE_1ST_ADD_MED_DT IS NOT NULL and &lt;= LOT1_BASE_DISCON_DT. (3) DISCONTINUATION - when LOT1_BASE_DISCON_DT IS NOT NULL. (4) CENSORED - default. Note: DEATH is not a separate end reason in code; death is captured via OBS_END_DT which sets CENSORED.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -715,7 +717,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - uses numeric codes 1-7 with date-matching logic and includes DEATH (4) as a separate end reason distinct from CENSOR. Protocol: Y - defines end reasons (Rules 1-8). Note: protocol does not specify priority/tie-breaking order; the code's SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED priority is an implementation decision. Code: Y - uses string end reasons ('SCT_AUTO', 'SCT_ALLO', 'SCT_CART', 'MED_ADD', 'DISCONTINUATION', 'CENSORED') with priority-based CASE; death is subsumed into CENSORED via OBS_END_DT.</t>
+          <t>Spec: N - uses numeric codes 1-7 with date-matching logic and includes DEATH (4) as a separate end reason distinct from CENSOR. Protocol: Y - defines end reasons (Rules 1-8); the code correctly picks the earliest event as protocol requires. The CASE order is a same-date tiebreaker not specified in the protocol. Code: Y - uses string end reasons ('SCT_AUTO', 'SCT_ALLO', 'SCT_CART', 'MED_ADD', 'DISCONTINUATION', 'CENSORED') with earliest-date-wins logic; death is subsumed into CENSORED via OBS_END_DT.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -723,7 +725,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Multiple discrepancies: (1) Spec uses numeric codes (1-7) while code uses descriptive strings ('DISCONTINUATION', 'MED_ADD', 'CENSORED', 'SCT_AUTO', 'SCT_ALLO', 'SCT_CART'). (2) Spec has DEATH as a separate end reason (code 4); code subsumes death into CENSORED since DEATH_DT is incorporated into OBS_END_DT/ENDDATE. (3) Spec determines end reason by matching LOT1_END_DT_TEMP against each candidate date; code uses explicit priority-based CASE (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED). (4) Spec's if/else chain checks LOT1_END_DT_TEMP against LOT1_DISCON_DT first, giving DISCONTINUATION highest priority among non-SCT reasons; code gives MED_ADD higher priority than DISCONTINUATION (when MED_ADD &lt;= DISCON). (5) Spec includes LOT1_BASE_MAINT_END_DT_TEMP in the initial min() which could set end reason to 2 (NEW MED) - maintenance is not yet implemented.</t>
         </is>
@@ -762,7 +765,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>lot_program.R: LOT1_EXTEND_FLG is NOT directly implemented. The code's approach at Step S16 (lines 4001-4017) gives SCT highest priority: if LOT1_TX_ENDDATE (SCT end minus 1 day) occurs at or before DISCON_DT and ADD_MED_DT, then end reason = SCT_AUTO/SCT_ALLO/SCT_CART. The SCT dates are computed at Step S15 (lines 3897-3983) with 14-day windowing (cfg$sct_auto_window_days=13), 60-day gap (cfg$sct_auto_gap_days=60), and 180-day tandem (cfg$sct_tandem_days=180). The conditioning period concept is implicitly handled by the SCT date processing at lines 3620-3793.</t>
+          <t>lot_program.R: LOT1_EXTEND_FLG is NOT directly implemented. The code's approach at Step S16 (lines 4001-4017) selects the earliest event date (SCT wins same-date ties): if LOT1_TX_ENDDATE (SCT end minus 1 day) occurs at or before DISCON_DT and ADD_MED_DT, then end reason = SCT_AUTO/SCT_ALLO/SCT_CART. The SCT dates are computed at Step S15 (lines 3897-3983) with 14-day windowing (cfg$sct_auto_window_days=13), 60-day gap (cfg$sct_auto_gap_days=60), and 180-day tandem (cfg$sct_tandem_days=180). The conditioning period concept is implicitly handled by the SCT date processing at lines 3620-3793.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -772,7 +775,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - defines LOT1_EXTEND_FLG as explicit 60-day extension from discontinuation. Protocol: N - protocol describes extending LOT1 for HSCT during conditioning but the code implements this differently. Code: Y - handles HSCT-during-conditioning via SCT priority in end reason CASE statement rather than a separate extension flag. The clinical intent is preserved but the implementation architecture differs significantly.</t>
+          <t>Spec: N - defines LOT1_EXTEND_FLG as explicit 60-day extension from discontinuation. Protocol: N - protocol describes extending LOT1 for HSCT during conditioning but the code implements this differently. Code: Y - handles HSCT-during-conditioning via earliest-date-wins logic in end reason CASE statement (SCT wins same-date ties) rather than a separate extension flag. The clinical intent is preserved but the implementation architecture differs significantly.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -780,7 +783,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_EXTEND_FLG as a multi-step process: (1) check if LOT1 ended due to discontinuation, (2) check if HSCT occurred within 60 days, (3) extend LOT1 end date to include HSCT. The code does NOT implement this variable. Instead, the code gives SCT events highest priority in the LOT1_BASE_END_REASON CASE statement (lot_program.R lines 4001-4011), so if an SCT event occurs before discontinuation, it directly sets the end reason to SCT_AUTO/SCT_ALLO/SCT_CART. The 60-day extension concept from the spec is architecturally different from the code's priority-based approach. The code also logs that maintenance integration is pending (line 4037-4038).</t>
         </is>
@@ -837,7 +841,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_EXTEND_LENGTH = LOT1_END_DT_TEMP - LOT1_END_DT_ORIG. This variable is not implemented in the R code because the code does not use the multi-step extension approach. The code's priority-based CASE statement makes this variable unnecessary in the current implementation.</t>
         </is>
@@ -876,7 +881,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>lot_program.R: NOT IMPLEMENTED as a separate variable. The code's LOT1_BASE_END_REASON (Step S16 lines 4001-4017) is the final end reason computed in a single pass. There is no intermediate 'SWITCH' step. The end reason directly accounts for SCT priority. The maintenance-related updates described in the spec (where end reason changes based on maintenance after HSCT) are not yet implemented (line 4037-4038).</t>
+          <t>lot_program.R: NOT IMPLEMENTED as a separate variable. The code's LOT1_BASE_END_REASON (Step S16 lines 4001-4017) is the final end reason computed in a single pass. There is no intermediate 'SWITCH' step. The end reason directly selects the earliest event (SCT wins same-date ties). The maintenance-related updates described in the spec (where end reason changes based on maintenance after HSCT) are not yet implemented (line 4037-4038).</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -894,7 +899,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_END_REASON_SWITCH as an updated version of LOT1_END_REASON_TEMP after HSCT extension logic. The code does not implement this as a separate variable. The code's single-pass LOT1_BASE_END_REASON (lot_program.R lines 4001-4017) serves as the final end reason. The spec's multi-step approach (TEMP -&gt; extend -&gt; SWITCH) is collapsed into one computation in the code.</t>
         </is>
@@ -951,7 +957,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Spec defines SWITCH_FLG = 1 if LOT1_SAME_CLASS_1ST_DT &lt;= LOT1_END_DT_TEMP. Neither LOT1_SAME_CLASS_1ST_DT nor SWITCH_FLG are implemented in the R code. The code handles same-class medication changes through the permissible substitutions mechanism (lot_program.R lines 3346-3354) rather than a separate flag. The spec's SWITCH_FLG concept is not present in the current codebase.</t>
         </is>
@@ -1000,7 +1007,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - includes additional logic to reset flag to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (HSCT occurred after LOT1 ended). Protocol: Y - defines single AUTO HSCT criteria. Code: Y - computes flag based on AUTO dates and tandem validation but does not reset to 0 based on LOT1_END_DT_TEMP; instead, the SCT priority logic in Step S16 handles this implicitly.</t>
+          <t>Spec: N - includes additional logic to reset flag to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (HSCT occurred after LOT1 ended). Protocol: Y - defines single AUTO HSCT criteria. Code: Y - computes flag based on AUTO dates and tandem validation but does not reset to 0 based on LOT1_END_DT_TEMP; instead, the earliest-date-wins logic in Step S16 handles this implicitly.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1008,7 +1015,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Spec includes logic to set LOT1_HSCT_AUTO_SING_FLG to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (i.e., the HSCT occurred after the LOT ended). The code at lot_program.R lines 3911-3917 does not include this temporal filter - the flag is set purely based on AUTO date existence and tandem validation. However, in the code's Step S16 end reason logic (lines 4001-4011), SCT events are only used if LOT1_TX_ENDDATE &lt;= other end dates, effectively achieving the same clinical filtering.</t>
         </is>
@@ -1057,7 +1065,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - includes reset logic if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. Protocol: Y - defines tandem as 2 AUTO within 180 days with no ALLO between. Code: Y - implements tandem flag matching protocol definition; temporal filtering handled implicitly by Step S16 priority logic.</t>
+          <t>Spec: N - includes reset logic if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. Protocol: Y - defines tandem as 2 AUTO within 180 days with no ALLO between. Code: Y - implements tandem flag matching protocol definition; temporal filtering handled implicitly by Step S16 earliest-date-wins logic.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1065,7 +1073,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Spec includes logic to reset LOT1_HSCT_AUTO_TAND_FLG to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. The code (lot_program.R lines 3904-3909) does not include this reset. Similar to SING_FLG, the temporal relationship is handled by Step S16's SCT priority logic rather than modifying the flag itself.</t>
         </is>
@@ -1122,7 +1131,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_TX_AUTO_MAX_DT as a named variable. The code does not create this specific variable but has the underlying data (AUTO_DT_1, AUTO_DT_2 at lot_program.R lines 3901-3902). The max valid AUTO date can be derived from the existing variables.</t>
         </is>
@@ -1179,7 +1189,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_TX_AUTO_FLG as a combined flag. The code does not create this specific variable but has LOT1_SCT_AUTO_TAND_FLG and LOT1_SCT_AUTO_SING_FLG (lot_program.R lines 3904-3917) from which the combined flag is trivially derivable.</t>
         </is>
@@ -1218,7 +1229,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>lot_program.R: The code does not update LOT1_END_DT_TEMP iteratively. Instead, LOT1_BASE_END_DT (Step S16 lines 4018-4028) is set to LOT1_TX_ENDDATE when SCT has priority. LOT1_TX_ENDDATE = date_sub(least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT), 1) at lines 3939-3949. For single AUTO, ENDING_AUTO_DT = AUTO_DT_2 (the LOT-ending event, line 3926). For tandem, ENDING_AUTO_DT = AUTO_DT_3 (line 3924). Note: the code's LOT1_TX_ENDDATE is the day BEFORE the LOT-ending SCT, not the date of the included SCT.</t>
+          <t>lot_program.R: The code does not update LOT1_END_DT_TEMP iteratively. Instead, LOT1_BASE_END_DT (Step S16 lines 4018-4028) is set to LOT1_TX_ENDDATE when SCT is the earliest event. LOT1_TX_ENDDATE = date_sub(least(ENDING_AUTO_DT, FIRST_ALLO_DT, FIRST_CART_DT), 1) at lines 3939-3949. For single AUTO, ENDING_AUTO_DT = AUTO_DT_2 (the LOT-ending event, line 3926). For tandem, ENDING_AUTO_DT = AUTO_DT_3 (line 3924). Note: the code's LOT1_TX_ENDDATE is the day BEFORE the LOT-ending SCT, not the date of the included SCT.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1228,7 +1239,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Spec: N - updates TEMP variable iteratively to HSCT date. Protocol: N - describes extending to include HSCT. Code: Y - uses LOT1_TX_ENDDATE (day before LOT-ending SCT) as the end date when SCT has priority. Key difference: spec extends LOT1 TO the HSCT date; code sets end to day BEFORE the LOT-ending SCT (which is the next AUTO after the included one).</t>
+          <t>Spec: N - updates TEMP variable iteratively to HSCT date. Protocol: N - describes extending to include HSCT. Code: Y - uses LOT1_TX_ENDDATE (day before LOT-ending SCT) as the end date when SCT is the earliest event. Key difference: spec extends LOT1 TO the HSCT date; code sets end to day BEFORE the LOT-ending SCT (which is the next AUTO after the included one).</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1236,7 +1247,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Spec updates LOT1_END_DT_TEMP to the included HSCT date (AUTO_DT_1 for single, AUTO_DT_2 for tandem). The code's LOT1_TX_ENDDATE is date_sub(ENDING_AUTO_DT, 1) where ENDING_AUTO_DT is the NEXT AUTO beyond what's included (AUTO_DT_2 for single, AUTO_DT_3 for tandem). This means the code's end date is the day before the LOT-ending SCT, not the date of the included SCT. The architectural approach differs significantly between spec and code.</t>
         </is>
@@ -1293,7 +1305,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
         </is>
@@ -1350,7 +1363,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_START with detailed conditions (120-day gap check, comparison with other end events). Maintenance is NOT ENABLED in the current implementation. The code explicitly logs that maintenance specs are not yet provided (lot_program.R lines 4037-4038). This is a deliberate scope decision - maintenance variables in the spec are aspirational and will require future implementation when maintenance is brought into scope.</t>
         </is>
@@ -1407,7 +1421,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_TYP from the LOT1_BASE_MAINT input dataset. MAINTENANCE IS NOT ENABLED in the current implementation. This is an aspirational spec variable that will require future implementation when maintenance is brought into scope.</t>
         </is>
@@ -1464,7 +1479,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_END with detailed conditional logic. MAINTENANCE IS NOT ENABLED in the current implementation. This is an aspirational spec variable pending future scope decision.</t>
         </is>
@@ -1521,7 +1537,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_MED_[MED] for BORT, DARA, IXAZ, LENA, CARF. MAINTENANCE IS NOT ENABLED in the current implementation. Induction medication flags (LOT1_MED_BORT, etc.) are implemented at lot_program.R Step S10 lines 3389 but these are separate from the maintenance flags. Aspirational spec variable pending future scope decision.</t>
         </is>
@@ -1578,7 +1595,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_END_REASON with numeric codes (1-6). MAINTENANCE IS NOT ENABLED in the current implementation. Additionally, the spec uses 6 values (1-6) while the base end reason has 7 (1-7, including CART) - the maintenance end reason omits CART (7), which may be intentional or an oversight. Aspirational spec variable pending future scope decision.</t>
         </is>
@@ -1617,7 +1635,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>lot_program.R Step S16 lines 4018-4028: LOT1_BASE_END_DT = CASE WHEN SCT priority THEN sct.LOT1_TX_ENDDATE; WHEN MED_ADD priority THEN lb.LOT1_BASE_1ST_ADD_MED_DT; WHEN DISCON THEN lb.LOT1_BASE_DISCON_DT; ELSE lb.OBS_END_DT END. This is the final (non-temporary) end date used in the lot1_base_end view.</t>
+          <t>lot_program.R Step S16 lines 4018-4028: LOT1_BASE_END_DT = CASE using &lt;= comparisons to select the earliest date: WHEN SCT earliest THEN sct.LOT1_TX_ENDDATE; WHEN MED_ADD earliest THEN lb.LOT1_BASE_1ST_ADD_MED_DT; WHEN DISCON THEN lb.LOT1_BASE_DISCON_DT; ELSE lb.OBS_END_DT END. The CASE order is a same-date tiebreaker only. This is the final (non-temporary) end date used in the lot1_base_end view.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1635,7 +1653,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never defines the final LOT1_BASE_END_DT. The code creates this as the definitive end date at lot_program.R Step S16 lines 4018-4028. The spec should include this final variable to show the output of the LOT1_BASE_END section.</t>
         </is>
@@ -1674,7 +1693,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>lot_program.R Step S16 lines 4001-4017: LOT1_BASE_END_REASON = CASE WHEN SCT AND earliest THEN 'SCT_AUTO'/'SCT_ALLO'/'SCT_CART'; WHEN MED_ADD AND earliest THEN 'MED_ADD'; WHEN DISCON THEN 'DISCONTINUATION'; ELSE 'CENSORED' END. QC query at lines 4032-4035 produces distribution of end reasons.</t>
+          <t>lot_program.R Step S16 lines 4001-4017: LOT1_BASE_END_REASON = CASE using &lt;= comparisons to select the earliest event: WHEN SCT earliest THEN 'SCT_AUTO'/'SCT_ALLO'/'SCT_CART'; WHEN MED_ADD earliest THEN 'MED_ADD'; WHEN DISCON THEN 'DISCONTINUATION'; ELSE 'CENSORED' END. The CASE order is a same-date tiebreaker only. QC query at lines 4032-4035 produces distribution of end reasons.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1692,7 +1711,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_REASON_TEMP and LOT1_END_REASON_SWITCH with numeric codes (1-7) but never creates the final LOT1_BASE_END_REASON. The code creates this with string values at lot_program.R Step S16 lines 4001-4017.</t>
         </is>
@@ -1749,7 +1769,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code computes LOT1_1ST_SCT_DT at lot_program.R Step S15 (lines 3963-3972) as the earliest SCT of any type. This is useful for validating the protocol's 60-day window rule (SCT must occur within 60 days of induction/maintenance end to be continuation of LOT). The spec should include this variable.</t>
         </is>
@@ -1806,7 +1827,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_ALLO_DT at lot_program.R Step S15 (line 3929) and uses it in the LOT1_TX_ENDDATE and LOT1_TX_ENDDATE_REASON calculations. The protocol explicitly states that any ALLO SCT ends the current LOT (Section 5.1.1). The spec references SCT_ALLO as end reason code 6 but does not define FIRST_ALLO_DT as a standalone variable.</t>
         </is>
@@ -1863,7 +1885,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_CART_DT at lot_program.R Step S15 (line 3930). The protocol defines CAR-T as always starting a new LOT (Section 5.1.2) with a 30-day supportive agent consolidation rule. The spec has CART as end reason code 7 but does not define FIRST_CART_DT as a standalone variable.</t>
         </is>
@@ -1920,7 +1943,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr">
         <is>
           <t>Parameter missing from original spec. The code uses lot_discon_gap_days=90 (lot_program.R line 73) to determine whether a patient is truly discontinued vs censored. This critical threshold affects whether LOT1_BASE_DISCON_DT is set or left NULL. The spec should document this parameter as it directly affects the LOT1_END_REASON classification.</t>
         </is>
@@ -1977,7 +2001,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses medical_day_supply=28 (lot_program.R line 74) for MAP_END_DT calculation on medical claims. While this is defined in the MAP section (5B), it directly affects LOT1_BASE_DISCON_DT and should be cross-referenced here. Protocol Section 5.1.1 explicitly states the 28-day assumption.</t>
         </is>
@@ -2026,7 +2051,7 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Spec: - (not defined in LOT1_BASE_END tab). Protocol: - (duration concept implied). Code: Y - computed at Step S10 lines 3447-3455 with priority MED_ADD &gt; DISCON &gt; CENSORED.</t>
+          <t>Spec: - (not defined in LOT1_BASE_END tab). Protocol: - (duration concept implied). Code: Y - computed at Step S10 lines 3447-3455 with earliest-date-wins logic (MED_ADD &gt; DISCON &gt; CENSORED as same-date tiebreaker).</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -2034,7 +2059,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K27" s="6" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab. The code computes LOT1_BASE_LENGTH at lot_program.R Step S10 (lines 3447-3455) using a priority-based CASE matching the same hierarchy as LOT1_BASE_END_DT. Note: this is computed in the LOT1_BASE step (S10) rather than LOT1_BASE_END (S16), but it represents the base period duration which should be documented here.</t>
         </is>
@@ -2073,7 +2099,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>lot_program.R: NOT APPLICABLE - MAINTENANCE IS NOT ENABLED. This rule depends on maintenance integration which is intentionally out of scope (line 4037-4038). The code currently ends LOT1 at LOT1_TX_ENDDATE (day before LOT-ending SCT) when SCT has priority. This 180-day rule will only become relevant if/when maintenance is brought into scope.</t>
+          <t>lot_program.R: NOT APPLICABLE - MAINTENANCE IS NOT ENABLED. This rule depends on maintenance integration which is intentionally out of scope (line 4037-4038). The code currently ends LOT1 at LOT1_TX_ENDDATE (day before LOT-ending SCT) when SCT is the earliest event. This 180-day rule will only become relevant if/when maintenance is brought into scope.</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2091,7 +2117,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K28" s="6" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.1 states that if SCT is not followed by maintenance within 180 days, the LOT ends at the SCT date. NOT APPLICABLE in current implementation because maintenance is not enabled. This rule should be implemented if/when maintenance is brought into scope.</t>
         </is>
@@ -2148,7 +2175,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K29" s="6" t="inlineStr">
+      <c r="K29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr">
         <is>
           <t>Concept missing from original spec's LOT1_BASE_END tab. The code implements permissible substitutions by expanding base_meds to include substitutes (lot_program.R Step S10 lines 3346-3354). This is critical for correct LOT1_BASE_1ST_ADD_MED_DT calculation: without it, a permissible substitute (e.g., daratumumab/hyaluronidase replacing daratumumab) would incorrectly trigger a MED_ADD end reason. Protocol Section 5.1.1 explicitly defines which substitutions are permissible.</t>
         </is>
@@ -2205,7 +2233,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K30" s="6" t="inlineStr">
+      <c r="K30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr">
         <is>
           <t>Design decision missing from original spec. The code includes steroids in the LOT1_BASE_DISCON_DT calculation (lot_program.R Step S10 lines 3355-3359) but documents this as a deliberate choice with a note for stakeholder review. The spec should document whether steroids should extend the discontinuation date, as this directly affects LOT1_BASE_END_DT for patients whose last active medication is a steroid.</t>
         </is>
@@ -2262,7 +2291,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K31" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec as standalone row. The code computes LOT1_TX_ENDDATE_REASON (lot_program.R lines 3951-3962) to bridge SCT type to end reason. The spec references SCT types indirectly via end reason codes 5=SCT_AUTO, 6=SCT_ALLO, 7=CART but does not define the intermediate reason variable.</t>
         </is>
@@ -2319,7 +2349,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K32" s="6" t="inlineStr">
+      <c r="K32" s="6" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr">
         <is>
           <t>Variables missing from original spec as standalone rows. The spec's HSCT extension logic (LOT1_EXTEND_FLG, updated LOT1_END_DT_TEMP) references LOT1_TX_AUTO_DT_1 and _DT_2 extensively but never defines them as their own variables. The code computes them at lot_program.R Step S15 lines 3901-3902 via the 14-day windowing algorithm at Step S13.</t>
         </is>
@@ -2376,7 +2407,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K33" s="6" t="inlineStr">
+      <c r="K33" s="6" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab as a standalone row. The spec references LOT1_BASE_DISCON_DT in the min() formula for LOT1_END_DT_TEMP and in the end reason logic, but never defines it. It is a key input variable computed at lot_program.R Step S10 lines 3360-3382.</t>
         </is>
@@ -2433,7 +2465,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr">
+      <c r="K34" s="6" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr">
         <is>
           <t>Variables missing from original spec's LOT1_BASE_END tab as standalone rows. The spec references LOT1_BASE_1ST_ADD_MED_DT in the min() formula and end reason logic but never defines it. Code deviation: spec says 'random' selection for same-day medication ties; code uses min() for determinism (lot_program.R line 3435). Also: LOT1_BASE_1ST_ADD_MED_DT = date_sub(ADD_START_DT, 1), meaning the end date is the day BEFORE the new med starts.</t>
         </is>
@@ -2490,7 +2523,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K35" s="6" t="inlineStr">
+      <c r="K35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses induction_window_days=60 (lot_program.R line 71) to determine which medications are in the induction regimen. This is critical: it directly controls what triggers MED_ADD end reason. Protocol Section 5.1.1 specifies 60 days (with 30-day alternative from Madduri 2021).</t>
         </is>
@@ -2539,7 +2573,7 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>Spec: - (implicit via SCT_ALLO end reason code 6 but not stated as an explicit rule). Protocol: - (explicit rule in Section 5.1.1). Code: Y - implemented via ALLO priority in LOT1_TX_ENDDATE and tandem invalidation.</t>
+          <t>Spec: - (implicit via SCT_ALLO end reason code 6 but not stated as an explicit rule). Protocol: - (explicit rule in Section 5.1.1). Code: Y - implemented via ALLO in LOT1_TX_ENDDATE (earliest date wins) and tandem invalidation.</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
@@ -2547,7 +2581,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr">
+      <c r="K36" s="6" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr">
         <is>
           <t>Protocol rule not explicitly stated in original spec. The spec has SCT_ALLO as end reason code 6 but does not document the rule that ALLO always ends the LOT unconditionally, or that auto-to-allo is not considered planned. The code implements this at lot_program.R via FIRST_ALLO_DT inclusion in LOT1_TX_ENDDATE (lines 3939-3949) and tandem invalidation (line 3907).</t>
         </is>
@@ -2604,7 +2639,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K37" s="6" t="inlineStr">
+      <c r="K37" s="6" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.2 specifies that therapies within 30 days of CAR-T are consolidated as part of the CAR-T LOT. The code does not implement this 30-day consolidation window. Impact: medications given in the 30 days before CAR-T could incorrectly influence LOT1's DISCON_DT or trigger MED_ADD. This should be implemented for correct medication attribution near CAR-T events.</t>
         </is>
@@ -2661,7 +2697,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K38" s="6" t="inlineStr">
+      <c r="K38" s="6" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr">
         <is>
           <t>Protocol exclusion rule not in original spec. Protocol Section 5.1.1 explicitly excludes mesna from LOTs. The code likely handles this by not including mesna in CL_MMA_CODELIST/CL_MMA_ROLLUP, but this should be verified. If mesna codes were inadvertently included in the codelist, they would incorrectly affect LOT1 end date calculations.</t>
         </is>
@@ -2718,7 +2755,8 @@
           <t>CV 2026-04-02 (protocol revalidation)</t>
         </is>
       </c>
-      <c r="K39" s="6" t="inlineStr">
+      <c r="K39" s="6" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
         <is>
           <t>Naming discrepancy: spec uses LOT1_HSCT_AUTO_SING_FLG / LOT1_HSCT_AUTO_TAND_FLG while code uses LOT1_SCT_AUTO_SING_FLG / LOT1_SCT_AUTO_TAND_FLG. Recommend aligning spec to use SCT prefix to match both code and protocol convention.</t>
         </is>

</xml_diff>

<commit_message>
Fix audit findings: remove implementation details from protocol-attributed text
- Rule 1 reframed as exception (not LOT-ending event) in rows 2, 20, 21
- 14-day claim windowing removed from protocol attribution (rows 9, 10, 32)
- 90-day gap value noted as code default, not protocol-specified (rows 2, 4)
- Additional Notes cleaned across 25+ rows: removed codelist refs
  (CL_MMA_ROLLUP, MONOMAINTENANCE), interpretation language, and
  implementation details incorrectly attributed to protocol
- Regenerated Excel with all fixes

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The LOT will continue until the earliest of any of the following events: (1) substitution of a biologic reference product with any of its biosimilars does not advance the LOT; (2) discontinuation of all agents in the regimen - the LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available; (3) unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, the LOT will end the day before the latter SCT; any allogeneic SCTs are considered a new LOT; (4) SCTs not followed by maintenance within 180 days - the last day of the LOT is the date of the SCT; (5) death; (6) health plan disenrollment; (7) end of the study period; (8) end of maintenance regimen.</t>
+          <t>The LOT will continue until the earliest of any of the following: (1) Discontinuation of all agents in the regimen (with or without switch to a new agent) - the LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available; (2) Unplanned SCTs - if an autologous SCT occurs &gt;180 days following a previous autologous SCT, the LOT will end the day before the latter SCT; any allogeneic SCTs are considered a new LOT; (3) SCTs not followed by maintenance within 180 days - the last day of the LOT is the date of the SCT; (4) Death; (5) Health plan disenrollment; (6) End of the study period; (7) End of maintenance regimen. Note: Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT (Rule 1 - this is an exception, not an ending event).</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Events that will not end LOT): Related to the HSCT conditioning period concept. The protocol describes the interval between treatment discontinuation and transplant as the conditioning period. This variable quantifies that interval. Not directly specified as a named protocol variable but implied by the HSCT extension logic.</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): Related to the HSCT conditioning period concept. The protocol describes the 60-day SCT continuation rule but does not name or define a variable quantifying this interval. Not directly specified as a named protocol variable but implied by the HSCT extension logic.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Protocol: Same-class switching is referenced in the context of LOT definition rules. When a patient switches from one medication to another within the same class (e.g., switching between proteasome inhibitors), this may or may not constitute a new line of therapy depending on the protocol rules. The protocol's treatment of same-class switches is relevant to determining whether a medication change ends LOT1 or is considered a permissible substitution.</t>
+          <t>Protocol: Same-class switching is referenced in the context of LOT definition rules. The protocol defines permissible substitutions (Rule 1: biologic reference product with biosimilars) that do not advance the LOT. The protocol does not define a broader same-class switching concept or a SWITCH_FLG variable.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Autologous SCT identification uses a 14-day claim windowing algorithm (operationalized as &gt;1 procedure code for an SCT per Section 5.1), requiring at least 60 days between distinct AUTO events. A single AUTO is one that is not part of a valid tandem pair. The protocol specifies that AUTO SCT claims within 14 days are grouped together, and events must be at least 60 days apart to be considered separate transplants.</t>
+          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Per protocol, SCT is operationalized as &gt;1 procedure code for an SCT (Section 5.1). A single AUTO is one that is not part of a valid tandem pair. Note: the 14-day claim windowing algorithm and 60-day gap between AUTO events are implementation details from the programming spec, not explicitly stated in the protocol.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Planned Tandem SCT): Protocol: 'Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart.' An autologous-to-allogeneic sequence is NOT considered planned. Tandem SCTs are 'considered planned and a continuation of the line of therapy' (Section 5.1.1). The first AUTO sets AUTO_DT_1, the second sets AUTO_DT_2. For tandem patients, a 3rd AUTO would end the LOT; for single AUTO patients, a 2nd AUTO ends the LOT.</t>
+          <t>Protocol Section 5.1 (Planned Tandem SCT): Protocol: 'Patients will be classified as having a planned tandem SCT if they receive at least two autologous SCTs &gt;60 to &lt;180 days apart.' An autologous-to-allogeneic sequence is NOT considered planned. Tandem SCTs are 'considered planned and a continuation of the line of therapy' (Section 5.1.1). Note: the implementation assigns AUTO_DT_1 and AUTO_DT_2 from the 14-day windowing algorithm (programming spec detail, not in the protocol).</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Planned Tandem SCT): The latest AUTO date is relevant for determining the LOT-ending SCT event. For tandem patients, the 2nd AUTO is the latest valid AUTO (the 3rd AUTO, if it exists, would end the LOT). For single AUTO patients, the 1st AUTO is the latest (the 2nd would end the LOT).</t>
+          <t>Protocol Section 5.1 (Planned Tandem SCT): The protocol defines tandem SCTs (&gt;60 to &lt;180 days apart) and single autologous SCTs as continuations of the LOT. The concept of a 'latest valid AUTO date' and the LOT-ending AUTO (3rd for tandem, 2nd for single) are implementation derivations from these protocol rules.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (SCT): Indicates whether the patient received any valid autologous transplant during the study period, regardless of whether it was single or tandem.</t>
+          <t>Protocol Section 5.1 (SCT): The protocol defines SCT as a LOT-specific binary variable (Section 5.1). A combined autologous flag covering both single and tandem is an implementation construct.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Events that will not end LOT): When LOT1 is extended to include an HSCT, the end date moves to the HSCT date (for single) or the second HSCT date (for tandem). If the patient receives maintenance after the HSCT, the LOT1 end date will be further extended (maintenance not yet implemented).</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): The protocol states single/tandem autologous SCTs continue the LOT (Section 5.1.1) and that SCTs must be within 60 days of induction/maintenance end. The mechanism of 'moving the end date' to the HSCT date is an implementation interpretation; 'maintenance not yet implemented' is an implementation status note.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance therapy follows induction/consolidation therapy. The maintenance period starts when a patient transitions from multi-agent induction to single-agent (mono) or dual-agent (dual) maintenance therapy. The protocol specifies mono-maintenance (single non-steroid medication with MONOMAINTENANCE=1 flag) and dual-maintenance (two medications where the combination is in the DUALMAINTENANCEWITH field of CL_MMA_ROLLUP).</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance therapy follows induction/consolidation therapy. The maintenance period starts when a patient transitions from multi-agent induction to single-agent (mono) or dual-agent (dual) maintenance therapy. The protocol specifies valid mono-maintenance and dual-maintenance therapies (Section 5.1). Note: MONOMAINTENANCE flag and DUALMAINTENANCEWITH/CL_MMA_ROLLUP are codelist implementation details, not protocol terms.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Maintenance regimen): The maintenance medication type identifies which drug is used for maintenance (e.g., LENA for lenalidomide, BORT for bortezomib). For mono-maintenance, this is a single medication; for dual-maintenance, this would describe the combination.</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): The protocol lists valid maintenance therapies by drug name (Section 5.1). Note: abbreviations like LENA, BORT are codelist/implementation conventions, not protocol terms.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance medication flags identify the specific drugs used during maintenance. These are a subset of the full medication list (BORT=bortezomib, DARA=daratumumab, IXAZ=ixazomib, LENA=lenalidomide, CARF=carfilzomib). The CL_MMA_ROLLUP codelist (Tab 40) defines which medications are eligible for maintenance via the MONOMAINTENANCE flag and DUALMAINTENANCEWITH field.</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance medication flags identify the specific drugs used during maintenance. These are a subset of the full medication list (BORT=bortezomib, DARA=daratumumab, IXAZ=ixazomib, LENA=lenalidomide, CARF=carfilzomib). Note: CL_MMA_ROLLUP, MONOMAINTENANCE flag, and DUALMAINTENANCEWITH are codelist implementation details, not protocol terms.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1620,12 +1620,12 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>'The LOT will continue until the earliest of any of the following' (Rules 1-8). The LOT end date is the final computed date after evaluating all end conditions. Per Rule 2: 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.' 'If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent.'</t>
+          <t>'The LOT will continue until the earliest of any of the following' (Rules 2-8 are ending events; Rule 1 defines permissible substitutions that do NOT end the LOT). Per Rule 2: 'The LOT end date is based on the run-out date, defined as the last date that any MM medication in that LOT is considered to be available.' 'If the current LOT is immediately interrupted by a new agent, the LOT end date is the day before the first administration/dispense date of the new agent.'</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end date, Rules 1-8): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. This final variable should be the non-temporary version after all adjustments. The original spec only defines TEMP versions but never creates the final LOT1_BASE_END_DT.</t>
+          <t>Protocol Section 5.1.1 (LOT end date, Rules 1-8): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. Note: the original spec only defines TEMP versions; LOT1_BASE_END_DT as a final variable is a code construct.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>LOT ends for one of the following reasons (Rules 1-8): (1) permissible substitution (does not end LOT); (2) discontinuation of all agents; (3) unplanned SCTs; (4) SCTs not followed by maintenance within 180 days; (5) death; (6) health plan disenrollment; (7) end of study period; (8) end of maintenance regimen.</t>
+          <t>LOT ends for one of the following reasons (Rules 2-8): (2) Discontinuation of all agents; (3) Unplanned SCTs; (4) SCTs not followed by maintenance within 180 days; (5) Death; (6) Health plan disenrollment; (7) End of study period; (8) End of maintenance regimen. Rule 1 (permissible substitutions - biologic reference product with biosimilars) does not advance the LOT and is not an ending event.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Events that will not end LOT): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.' LOT1_1ST_SCT_DT enables validation of this 60-day window rule.</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.' The first SCT date enables checking compliance with this 60-day window rule.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' (Section 5.1). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs' (Section 5.1.1, Rule 3). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' This is a hard rule - ALLO always ends the LOT regardless of timing relative to other events.</t>
+          <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' (Section 5.1). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs' (Section 5.1.1, Rule 3). 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Per the protocol, allogeneic SCT always ends the current LOT.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The run-out date is the MAP_END_DT (last day of medication availability). The gap threshold ensures there is sufficient time after medication ends to confirm the patient truly discontinued rather than being censored. The 90-day default is consistent with a treatment cycle of approximately 3 months. Configurable for sensitivity analysis per Protocol Section 5.3 which states 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The run-out date is the MAP_END_DT (last day of medication availability). The gap threshold ensures there is sufficient time after medication ends to confirm the patient truly discontinued rather than being censored. The protocol refers to a 'qualifying gap' (Section 5.1.1) without specifying the exact number of days. 90 days is a code default. Per Protocol Section 5.3: 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - run-out date): 'The days' supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days' supply, or when days' supply values are anomalous, a 28-day supply is assumed.' (Section 5.1.1, under Rule 2). This is a fundamental parameter for the MAP algorithm that feeds into the LOT1 end date calculation. The 28-day assumption represents approximately one treatment cycle.</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - run-out date): 'The days' supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days' supply, or when days' supply values are anomalous, a 28-day supply is assumed.' (Section 5.1.1, under Rule 2). This parameter directly affects run-out date calculation and therefore LOT end date determination.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT start/end): LOT duration is the span from LOT start (first non-steroid MAP) to LOT end. The +1 ensures inclusive day counting (both start and end dates are counted). Duration is relevant for assessing treatment patterns and time-to-event analyses.</t>
+          <t>Protocol Section 5.1.1 (LOT start/end): LOT duration can be derived from the protocol-defined LOT start date and LOT end date. Note: 'first non-steroid MAP,' inclusive +1 day counting, and the variable name are implementation details.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 4 - SCTs not followed by maintenance): Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Also Section 5.1 (Maintenance regimen, situation 2): 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT).' This rule interacts with the maintenance logic: if maintenance starts within 180 days of SCT, LOT1 is extended to include the maintenance period. If no maintenance within 180 days, LOT1 ends at the SCT date. The 180-day window is consistent with the tandem SCT definition (cfg$sct_tandem_days=180).</t>
+          <t>Protocol Section 5.1.1 (Rule 4 - SCTs not followed by maintenance): Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Also Section 5.1 (Maintenance regimen, situation 2): 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT).' This rule interacts with the maintenance logic: if maintenance starts within 180 days of SCT, LOT1 is extended to include the maintenance period. If no maintenance within 180 days, LOT1 ends at the SCT date. The 180-day window appears in both the SCT-maintenance rule and the tandem SCT definition.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 1 - Permissible substitutions): Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.' This directly affects LOT1_BASE_1ST_ADD_MED_DT: if the 'new' medication is a permissible substitute, it should not be counted as an addition. The permissible_subs table codifies these rules.</t>
+          <t>Protocol Section 5.1.1 (Rule 1 - Permissible substitutions): Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.' This directly affects LOT1_BASE_1ST_ADD_MED_DT: if the 'new' medication is a permissible substitute, it should not be counted as an addition. The code implements these rules via a permissible_subs table (implementation detail).</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Section 5.1 explicitly states: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Also: 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of active MM treatment.' The protocol excludes steroids from LOT rules, but the code includes steroids in the discontinuation calculation - this is a deliberate design decision documented with a code comment for stakeholder review.</t>
+          <t>Protocol Section 5.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Section 5.1 explicitly states: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Also: 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of active MM treatment.' The protocol states LOT rules are based on oncology therapies only, not corticosteroids. Note: the code includes steroids in the discontinuation calculation as a deliberate implementation decision (documented in code for stakeholder review).</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 3 - Unplanned SCTs) and Section 5.1 (SCT types): SCT type determines how LOT1 ends. Autologous SCT: single AUTO is allowed within LOT; excess AUTO (2nd for single, 3rd for tandem) ends LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT. The reason type is essential for correctly classifying the end reason.</t>
+          <t>Protocol Section 5.1.1 (Rule 3 - Unplanned SCTs) and Section 5.1 (SCT types): SCT type determines how LOT1 ends. Autologous SCT: single AUTO is allowed within LOT; excess AUTO (2nd for single, 3rd for tandem) ends LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT. The SCT type determines the end reason classification in the code.</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Planned Tandem SCT) and Section 5.1.1 (Events that will not end LOT): AUTO SCT dates are identified using a 14-day claim windowing algorithm (claims within 14 days grouped together, selecting the last date in the window). Events must be at least 60 days apart (cfg$sct_auto_gap_days=60). Tandem pair defined as DT_1 and DT_2 within 180 days with no ALLO between them. The spec references these dates extensively in the HSCT extension logic but does not define them as standalone rows.</t>
+          <t>Protocol Section 5.1 (Planned Tandem SCT) and Section 5.1.1 (Events that will not end LOT): The protocol defines tandem SCTs as two autologous SCTs &gt;60 to &lt;180 days apart (Section 5.1). Note: the 14-day claim windowing algorithm, 60-day gap validation (cfg$sct_auto_gap_days=60), and no-ALLO-between condition are implementation details from the programming spec/code, not explicitly stated in the protocol.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation with new agent): Rule 2: 'With initiation of a new MM agent that was not present in the induction regimen (i.e., the regimen is interrupted by a new agent).' 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Rule 1 (permissible substitutions) does NOT trigger a new LOT. The LOT end date is set to the day BEFORE the new medication starts (date_sub(ADD_START_DT, 1)). Per protocol, permissible substitutions (rituximab/hyaluronidase swap, biosimilars, bortezomib-&gt;ixazomib for maintenance) do NOT trigger a new LOT.</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation with new agent): Rule 2: 'With initiation of a new MM agent that was not present in the induction regimen (i.e., the regimen is interrupted by a new agent).' 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Rule 1 (permissible substitutions) does NOT trigger a new LOT. The LOT end date is set to the day BEFORE the new medication starts (date_sub(ADD_START_DT, 1)). Per protocol Rule 1, permissible substitutions (biologic reference product with biosimilars) do NOT trigger a new LOT.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT regimen): 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' For LOT2-5: 'the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' The 60-day window is the primary parameter; 30-day is noted as an alternative from literature. This parameter directly determines what is in the base regimen and therefore what constitutes a 'new' medication triggering MED_ADD. Configurable for sensitivity analysis per Protocol Section 5.3.</t>
+          <t>Protocol Section 5.1.1 (LOT regimen): 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' For LOT2-5: 'the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' The protocol specifies 60 days for LOT1 and 30 days for LOT2-5. This parameter directly determines what is in the base regimen and therefore what constitutes a 'new' medication triggering MED_ADD. Configurable for sensitivity analysis per Protocol Section 5.3.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): Section 5.1: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Section 5.1.1 (Rule 3): 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Also: 'Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.' Also: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Additionally, the presence of an ALLO between two AUTO SCTs invalidates the tandem classification (coalesce(n_allo_between, 0) = 0 required for tandem).</t>
+          <t>Protocol Section 5.1 (Allogeneic SCT) and Section 5.1.1 (Rule 3): Section 5.1: 'Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT.' Section 5.1.1 (Rule 3): 'Any allogeneic SCTs are considered a new LOT and the current LOT will end the day before an allogeneic SCT occurs.' Also: 'Presence of an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT.' Also: 'An autologous SCT followed by an allogeneic SCT will not be considered planned because an allogeneic SCT typically follows failed autologous SCTs.' Additionally, per protocol, an autologous-to-allogeneic sequence is not considered planned tandem (Section 5.1).</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (CAR-T): 'CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' (Section 5.1.1) This 30-day window affects medication attribution near the LOT1/CAR-T boundary. Without this rule, medications given in the 30 days before CAR-T could incorrectly extend LOT1's discontinuation date or trigger a MED_ADD end reason.</t>
+          <t>Protocol Section 5.1.1 (CAR-T): 'CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' (Section 5.1.1) This 30-day window determines medication attribution near the LOT1/CAR-T boundary.</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (MM therapies): 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion beyond the general steroid handling. Mesna should be excluded from CL_MMA_CODELIST or filtered out during medication identification.</t>
+          <t>Protocol Section 5.1 (MM therapies): 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion stated in Section 5.1. Note: the mechanism of exclusion (via CL_MMA_CODELIST or filtering) is an implementation detail.</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Protocol uses 'SCT' (Stem Cell Transplant) terminology consistently. The spec uses 'HSCT' (Hematopoietic Stem Cell Transplant). Both are acceptable medical abbreviations for the same concept. The code aligns with the protocol's 'SCT' convention.</t>
+          <t>The protocol consistently uses 'SCT' terminology (Section 5.1: 'Stem cell transplant (SCT)'). The original spec uses 'HSCT' prefix. The code uses 'SCT' prefix matching the protocol. Both abbreviations refer to the same medical concept. This is an observation about naming conventions, not a protocol-defined variable.</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Clean Additional Notes: remove all remaining non-protocol content
Per validation audit, systematically cleaned 25 Additional Notes cells:
- Removed CASE statement details, <= comparisons, tiebreaker order (rows 2,4,5)
- Removed "conditioning period" term not in protocol (row 6)
- Removed SWITCH concept spec framing (row 7)
- Removed codelist refs: CL_MMA_ROLLUP, MONOMAINTENANCE, DUALMAINTENANCEWITH (rows 15,18)
- Replaced interpretive "similar logic" phrasing with protocol text (rows 17,19)
- Removed spec TEMP/SWITCH version references (rows 20,21)
- Removed implementation purpose statements (rows 22,26,37)
- Removed MAP_END_DT terminology (row 25)
- Removed date_sub() code expression (row 34)
- Removed cfg$ parameter references (row 32)
- Removed "2nd for single, 3rd for tandem" counting logic (row 31)
- Replaced explanatory synthesis with direct protocol citations throughout
- Regenerated Excel with all fixes

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications, addition of a new non-induction medication, a LOT-ending SCT event, death, health plan disenrollment, or end of study period. The code implements this as 'earliest date wins' using &lt;= comparisons in a CASE statement. The CASE evaluation order (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) serves only as a same-date tiebreaker and is not specified in the protocol.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications, addition of a new non-induction medication, a LOT-ending SCT event, death, health plan disenrollment, or end of study period. Note: the code implements this via a CASE statement with a same-date tiebreaker order — this is an implementation detail, not protocol text.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (Rule 2) Discontinuation - all induction medications discontinued; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events. Protocol explicitly numbers LOT end events as Rules 1-8. The code selects the earliest date; the CASE evaluation order (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) is a same-date tiebreaker not in the protocol.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (Rule 2) Discontinuation - all induction medications discontinued; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events. Protocol explicitly numbers LOT end events as Rules 1-8. Note: the CASE evaluation order for same-date tiebreaking is an implementation detail, not protocol text.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Protocol states 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.' (Section 5.1.1). Single and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.' The code handles this differently: SCT events take top priority in the code's CASE statement (a code design decision, not a protocol-specified priority) rather than using a separate extension flag.</t>
+          <t>Protocol Section 5.1 (SCT) and Section 5.1.1 (Events that will not end LOT): Protocol states 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT.' (Section 5.1.1). Single and tandem SCTs are 'not unplanned SCTs and are considered a continuation of the line of therapy.' Note: the code handles this via its CASE statement structure (implementation detail, not protocol text).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Events that will not end LOT): Related to the HSCT conditioning period concept. The protocol describes the 60-day SCT continuation rule but does not name or define a variable quantifying this interval. Not directly specified as a named protocol variable but implied by the HSCT extension logic.</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): The protocol describes the 60-day SCT continuation rule but does not name or define a variable quantifying this interval. Not directly specified as a named protocol variable but implied by the HSCT extension logic.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules): After HSCT evaluation, if the LOT1 is extended to include an HSCT, the end reason should reflect whether the patient received maintenance after HSCT or if the LOT ended at the HSCT. The protocol does not explicitly define a 'SWITCH' concept for end reasons; this appears to be a spec-level implementation detail.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules): The protocol defines LOT end reasons directly via Rules 1-8. It does not explicitly define an intermediate 'SWITCH' concept for updating end reasons after HSCT evaluation — this is a spec-level implementation detail.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance therapy follows induction/consolidation therapy. The maintenance period starts when a patient transitions from multi-agent induction to single-agent (mono) or dual-agent (dual) maintenance therapy. The protocol specifies valid mono-maintenance and dual-maintenance therapies (Section 5.1). Note: MONOMAINTENANCE flag and DUALMAINTENANCEWITH/CL_MMA_ROLLUP are codelist implementation details, not protocol terms.</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance therapy follows induction/consolidation therapy. The maintenance period starts when a patient transitions from multi-agent induction to single-agent (mono) or dual-agent (dual) maintenance therapy. The protocol specifies valid mono-maintenance and dual-maintenance therapies (Section 5.1). Note: specific codelist flags and rollup tables are implementation details, not protocol terms.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): The maintenance period ends when the patient discontinues maintenance therapy, adds a new medication (signaling a new LOT), receives an SCT, dies, or reaches end of observation. The end of maintenance follows similar logic to the base period end.</t>
+          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): The maintenance period ends when the patient discontinues maintenance therapy, adds a new medication (signaling a new LOT), receives an SCT, dies, or reaches end of observation. Per the protocol, maintenance ends upon discontinuation, SCT, right censoring, or addition of a non-maintenance MM therapy.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance medication flags identify the specific drugs used during maintenance. These are a subset of the full medication list (BORT=bortezomib, DARA=daratumumab, IXAZ=ixazomib, LENA=lenalidomide, CARF=carfilzomib). Note: CL_MMA_ROLLUP, MONOMAINTENANCE flag, and DUALMAINTENANCEWITH are codelist implementation details, not protocol terms.</t>
+          <t>Protocol Section 5.1 (Maintenance regimen): Maintenance medication flags identify the specific drugs used during maintenance. These are a subset of the full medication list (BORT=bortezomib, DARA=daratumumab, IXAZ=ixazomib, LENA=lenalidomide, CARF=carfilzomib). Note: codelist flags and rollup tables are implementation details, not protocol terms.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): Maintenance period end reasons follow a similar logic to the base period end reasons. The maintenance period can end due to discontinuation of maintenance therapy, addition of a new medication (indicating progression to next LOT), censoring, death, or an SCT event.</t>
+          <t>Protocol Section 5.1.1 (Rule 8 - End of maintenance regimen): Per Rule 8, the maintenance period can end due to: unplanned SCTs, death, health plan disenrollment, end of study period, or addition of any non-maintenance MM therapy.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end date, Rules 1-8): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. Note: the original spec only defines TEMP versions; LOT1_BASE_END_DT as a final variable is a code construct.</t>
+          <t>Protocol Section 5.1.1 (LOT end date, Rules 1-8): 'The end date is the run-out date before the gap. The run-out date is calculated using a patient''s combined infused/injected drugs as well as oral drugs.' The protocol defines the end date as the last day of medication coverage before the qualifying gap or event. Note: LOT1_BASE_END_DT as a final variable name is a code construct, not a protocol-defined variable.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. The original spec only defines TEMP and SWITCH versions with numeric codes but never creates the final string-valued LOT1_BASE_END_REASON.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. Note: LOT1_BASE_END_REASON as a final variable is a code construct.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Events that will not end LOT): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.' The first SCT date enables checking compliance with this 60-day window rule.</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): 'SCTs must be within 60 days after the end of the induction or maintenance regimen to be considered a continuation of the LOT. This 60-day rule was recommended by Optum''s KOL and informed by Charalampous et al.''s findings that the median time from end of induction to transplant was 33 days.'</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (CAR-T): 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' CAR-T always starts a new LOT, ending the current one. The 30-day supportive agent consolidation rule means medications within 30 days of CAR-T are attributed to the CAR-T LOT, not the preceding LOT.</t>
+          <t>Protocol Section 5.1.1 (CAR-T): 'Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' Per the protocol, CAR-T is classified as its own LOT and medications within 30 days are consolidated as part of it.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The run-out date is the MAP_END_DT (last day of medication availability). The gap threshold ensures there is sufficient time after medication ends to confirm the patient truly discontinued rather than being censored. The protocol refers to a 'qualifying gap' (Section 5.1.1) without specifying the exact number of days. 90 days is a code default. Per Protocol Section 5.3: 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT.' The gap is measured from the run-out date (last day of medication availability). The protocol refers to a 'qualifying gap' (Section 5.1.1) without specifying the exact number of days. 90 days is a code default. Per Protocol Section 5.3: 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters.'</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - run-out date): 'The days' supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days' supply, or when days' supply values are anomalous, a 28-day supply is assumed.' (Section 5.1.1, under Rule 2). This parameter directly affects run-out date calculation and therefore LOT end date determination.</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - run-out date): 'The days' supply on medical claims is always missing and therefore a 28-day supply is assumed. When pharmacy claims are missing days' supply, or when days' supply values are anomalous, a 28-day supply is assumed.' (Section 5.1.1, under Rule 2).</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 4 - SCTs not followed by maintenance): Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Also Section 5.1 (Maintenance regimen, situation 2): 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT).' This rule interacts with the maintenance logic: if maintenance starts within 180 days of SCT, LOT1 is extended to include the maintenance period. If no maintenance within 180 days, LOT1 ends at the SCT date. The 180-day window appears in both the SCT-maintenance rule and the tandem SCT definition.</t>
+          <t>Protocol Section 5.1.1 (Rule 4 - SCTs not followed by maintenance): Rule 4: 'SCTs not followed by maintenance: If an SCT is not followed by a maintenance regimen within 180 days, then the last day of the LOT is the date of the SCT.' Also Section 5.1 (Maintenance regimen, situation 2): 'Following an autologous SCT (within 180 days of the SCT or in the case of a tandem autologous SCT within 180 days of the second SCT).' Per the protocol, if maintenance starts within 180 days the LOT continues; if not, the LOT ends at the SCT date.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 1 - Permissible substitutions): Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.' This directly affects LOT1_BASE_1ST_ADD_MED_DT: if the 'new' medication is a permissible substitute, it should not be counted as an addition. The code implements these rules via a permissible_subs table (implementation detail).</t>
+          <t>Protocol Section 5.1.1 (Rule 1 - Permissible substitutions): Rule 1: 'Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT; such permissible substitutions are considered within the same line, which is named according to the drug given for the longest duration.' Per the protocol, permissible substitutions should not be counted as new medication additions.</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Section 5.1 explicitly states: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Also: 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of active MM treatment.' The protocol states LOT rules are based on oncology therapies only, not corticosteroids. Note: the code includes steroids in the discontinuation calculation as a deliberate implementation decision (documented in code for stakeholder review).</t>
+          <t>Protocol Section 5.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1.' Section 5.1 explicitly states: 'All rules described below are based on oncology therapies only (e.g., not corticosteroids).' Also: 'Receipt of corticosteroids only (e.g., dexamethasone) will not be considered evidence of active MM treatment.' The protocol states LOT rules are based on oncology therapies only, not corticosteroids. Note: the code's handling of steroids in the discontinuation calculation is an implementation decision — see code comments for details.</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 3 - Unplanned SCTs) and Section 5.1 (SCT types): SCT type determines how LOT1 ends. Autologous SCT: single AUTO is allowed within LOT; excess AUTO (2nd for single, 3rd for tandem) ends LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT. The SCT type determines the end reason classification in the code.</t>
+          <t>Protocol Section 5.1.1 (Rule 3 - Unplanned SCTs) and Section 5.1 (SCT types): SCT type determines how LOT1 ends. Autologous SCT: single/tandem AUTO is a continuation; additional unplanned AUTO ends the LOT. Allogeneic SCT: always ends current LOT immediately. CAR-T: always starts a new LOT.</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (Planned Tandem SCT) and Section 5.1.1 (Events that will not end LOT): The protocol defines tandem SCTs as two autologous SCTs &gt;60 to &lt;180 days apart (Section 5.1). Note: the 14-day claim windowing algorithm, 60-day gap validation (cfg$sct_auto_gap_days=60), and no-ALLO-between condition are implementation details from the programming spec/code, not explicitly stated in the protocol.</t>
+          <t>Protocol Section 5.1 (Planned Tandem SCT) and Section 5.1.1 (Events that will not end LOT): The protocol defines tandem SCTs as two autologous SCTs &gt;60 to &lt;180 days apart (Section 5.1). Note: the 14-day claim windowing algorithm, gap validation parameters, and no-ALLO-between condition are implementation details, not protocol text.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT. Run-out date is the last date that a medication for a specific prescription is considered to be available.' The gap threshold ensures true discontinuation vs censoring near end of follow-up.</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation): 'Discontinuation is defined as the run-out date of all MM treatments in the LOT. Run-out date is the last date that a medication for a specific prescription is considered to be available.' The protocol defines discontinuation via the qualifying gap concept (Section 5.1.1, Rule 2).</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation with new agent): Rule 2: 'With initiation of a new MM agent that was not present in the induction regimen (i.e., the regimen is interrupted by a new agent).' 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Rule 1 (permissible substitutions) does NOT trigger a new LOT. The LOT end date is set to the day BEFORE the new medication starts (date_sub(ADD_START_DT, 1)). Per protocol Rule 1, permissible substitutions (biologic reference product with biosimilars) do NOT trigger a new LOT.</t>
+          <t>Protocol Section 5.1.1 (Rule 2 - Discontinuation with new agent): Rule 2: 'With initiation of a new MM agent that was not present in the induction regimen (i.e., the regimen is interrupted by a new agent).' 'If the current LOT is immediately interrupted by a new agent (the new agent starts on or before the run-out date of the current regimen), the LOT end date is the day before the first administration/dispense date of the new agent.' Rule 1 (permissible substitutions) does NOT trigger a new LOT. Per the protocol, the LOT end date is the day before the first administration/dispense date of the new agent. Per protocol Rule 1, permissible substitutions (biologic reference product with biosimilars) do NOT trigger a new LOT.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT regimen): 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' For LOT2-5: 'the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' The protocol specifies 60 days for LOT1 and 30 days for LOT2-5. This parameter directly determines what is in the base regimen and therefore what constitutes a 'new' medication triggering MED_ADD. Configurable for sensitivity analysis per Protocol Section 5.3.</t>
+          <t>Protocol Section 5.1.1 (LOT regimen): 'The LOT1 regimen includes all MM therapies received within 60 days (Madduri, 2021) on and following the LOT1 start date.' For LOT2-5: 'the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' The protocol specifies 60 days for LOT1 and 30 days for LOT2-5. Per Protocol Section 5.3, sensitivity analyses may vary key algorithm parameters.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (CAR-T): 'CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' (Section 5.1.1) This 30-day window determines medication attribution near the LOT1/CAR-T boundary.</t>
+          <t>Protocol Section 5.1.1 (CAR-T): 'CAR-T cellular therapy infusions are classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.' (Section 5.1.1)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1 (MM therapies): 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion stated in Section 5.1. Note: the mechanism of exclusion (via CL_MMA_CODELIST or filtering) is an implementation detail.</t>
+          <t>Protocol Section 5.1 (MM therapies): 'The following therapy is excluded from LOTs: mesna (treatment of MM to protect the patient''s bladder against the toxic side-effects of certain anticancer drugs).' This is a specific exclusion stated in Section 5.1. Note: the specific mechanism of exclusion is an implementation detail.</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Final cleanup: add missing Rules 4/8, fix numbering, remove status note
- Row 2: Added 'end of maintenance regimen' (Rule 8) to Additional Notes list
- Row 4: Added Rules 4 and 8 to Additional Notes enumeration
- Row 13: Removed 'maintenance not yet implemented' status note
- Row 21: Realigned Additional Notes numbering to protocol Rules 1-8

https://claude.ai/code/session_01CK5wLBfZWvXwetUqTCCu19
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
+++ b/docs/Part 3/Program Spec/lot1baseend_validated.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications, addition of a new non-induction medication, a LOT-ending SCT event, death, health plan disenrollment, or end of study period. Note: the code implements this via a CASE statement with a same-date tiebreaker order — this is an implementation detail, not protocol text.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 base period ends at the earliest of: discontinuation of all induction medications, addition of a new non-induction medication, a LOT-ending SCT event, death, health plan disenrollment, end of study period, or end of maintenance regimen. Note: the code implements this via a CASE statement with a same-date tiebreaker order — this is an implementation detail, not protocol text.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (Rule 2) Discontinuation - all induction medications discontinued; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events. Protocol explicitly numbers LOT end events as Rules 1-8. Note: the CASE evaluation order for same-date tiebreaking is an implementation detail, not protocol text.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT1 ends for one of these reasons: (Rule 2) Discontinuation - all induction medications discontinued; (Rule 2) New medication addition - a medication not in the induction regimen is started; (Rules 5-7) Censoring - death/disenrollment/study end; (Rule 3) Unplanned SCT events; (Rule 4) SCTs not followed by maintenance within 180 days; (Rule 8) End of maintenance regimen. Protocol explicitly numbers LOT end events as Rules 1-8. Note: the CASE evaluation order for same-date tiebreaking is an implementation detail, not protocol text.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (Events that will not end LOT): The protocol states single/tandem autologous SCTs continue the LOT (Section 5.1.1) and that SCTs must be within 60 days of induction/maintenance end. The mechanism of 'moving the end date' to the HSCT date is an implementation interpretation; 'maintenance not yet implemented' is an implementation status note.</t>
+          <t>Protocol Section 5.1.1 (Events that will not end LOT): The protocol states single/tandem autologous SCTs continue the LOT (Section 5.1.1) and that SCTs must be within 60 days of induction/maintenance end. The mechanism of 'moving the end date' to the HSCT date is an implementation interpretation.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends when (1) a transplant occurs (allo always ends LOT; auto ends if unplanned or beyond tandem), (2) a new non-induction medication is added, (3) all medications are discontinued with a sufficient gap, or (4) the patient is censored. Note: LOT1_BASE_END_REASON as a final variable is a code construct.</t>
+          <t>Protocol Section 5.1.1 (LOT end rules 1-8): LOT ends per Rules 2-8: (Rule 2) discontinuation of all agents or interruption by new agent; (Rule 3) unplanned SCTs or allogeneic SCT; (Rule 4) SCT not followed by maintenance within 180 days; (Rules 5-7) death, disenrollment, study end; (Rule 8) end of maintenance regimen. Rule 1 (permissible substitutions) does NOT end the LOT. Note: LOT1_BASE_END_REASON as a final variable is a code construct.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">

</xml_diff>